<commit_message>
Daily Thornton Place tracker update - 2026-08-23
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BW41"/>
+  <dimension ref="A1:BX41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -948,14 +948,17 @@
         <v>46255.57755599537</v>
       </c>
       <c r="BU1" s="56" t="n">
-        <v>46256.56776790856</v>
-      </c>
-      <c r="BV1" s="44" t="inlineStr">
+        <v>46256.56776790509</v>
+      </c>
+      <c r="BV1" s="56" t="n">
+        <v>46257.56858499269</v>
+      </c>
+      <c r="BW1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BW1" s="44" t="inlineStr">
+      <c r="BX1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1009,12 +1012,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BV2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW2" s="58" t="inlineStr">
+      <c r="BW2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1068,12 +1071,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BV3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW3" s="58" t="inlineStr">
+      <c r="BW3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1128,12 +1131,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BV4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1198,12 +1201,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BV5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1263,12 +1266,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BV6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1323,12 +1326,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BV7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1368,7 +1371,11 @@
           <t>Available Now</t>
         </is>
       </c>
-      <c r="H8" s="42" t="n"/>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="V8" s="42" t="n">
         <v>3439.06</v>
       </c>
@@ -1405,12 +1412,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BV8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1458,12 +1465,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BV9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1511,12 +1518,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BV10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1559,12 +1566,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BV11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1617,8 +1624,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BV13" s="42" t="n"/>
       <c r="BW13" s="42" t="n"/>
+      <c r="BX13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1674,12 +1681,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BV14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW14" s="58" t="inlineStr">
+      <c r="BW14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1733,12 +1740,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BV15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BW15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1825,12 +1832,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BV16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW16" s="58" t="inlineStr">
+      <c r="BW16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1909,12 +1916,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BV17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW17" s="58" t="inlineStr">
+      <c r="BW17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1977,12 +1984,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BV18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW18" s="58" t="inlineStr">
+      <c r="BW18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2049,12 +2056,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BV19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW19" s="71" t="inlineStr">
+      <c r="BW19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2118,12 +2125,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BV20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW20" s="58" t="inlineStr">
+      <c r="BW20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2183,12 +2190,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BV21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW21" s="71" t="inlineStr">
+      <c r="BW21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2250,12 +2257,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BV22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW22" s="71" t="inlineStr">
+      <c r="BW22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2310,12 +2317,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BV23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BW23" s="58" t="inlineStr">
+      <c r="BW23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BX23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-24
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BX41"/>
+  <dimension ref="A1:BY41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -951,14 +951,17 @@
         <v>46256.56776790509</v>
       </c>
       <c r="BV1" s="56" t="n">
-        <v>46257.56858499269</v>
-      </c>
-      <c r="BW1" s="44" t="inlineStr">
+        <v>46257.56858498842</v>
+      </c>
+      <c r="BW1" s="56" t="n">
+        <v>46258.58133451459</v>
+      </c>
+      <c r="BX1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BX1" s="44" t="inlineStr">
+      <c r="BY1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1012,12 +1015,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BW2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX2" s="58" t="inlineStr">
+      <c r="BX2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1071,12 +1074,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BW3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX3" s="58" t="inlineStr">
+      <c r="BX3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1131,12 +1134,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BW4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1201,12 +1204,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BW5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1266,12 +1269,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BW6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1326,12 +1329,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BW7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1412,12 +1415,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BW8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1465,12 +1468,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BW9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1518,12 +1521,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BW10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1566,12 +1569,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BW11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1624,8 +1627,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BW13" s="42" t="n"/>
       <c r="BX13" s="42" t="n"/>
+      <c r="BY13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1681,12 +1684,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BW14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX14" s="58" t="inlineStr">
+      <c r="BX14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1740,12 +1743,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BW15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BX15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1832,12 +1835,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BW16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX16" s="58" t="inlineStr">
+      <c r="BX16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1916,12 +1919,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BW17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX17" s="58" t="inlineStr">
+      <c r="BX17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1984,12 +1987,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BW18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX18" s="58" t="inlineStr">
+      <c r="BX18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2056,12 +2059,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BW19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX19" s="71" t="inlineStr">
+      <c r="BX19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2125,12 +2128,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BW20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX20" s="58" t="inlineStr">
+      <c r="BX20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2190,12 +2193,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BW21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX21" s="71" t="inlineStr">
+      <c r="BX21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2257,12 +2260,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BW22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX22" s="71" t="inlineStr">
+      <c r="BX22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2317,12 +2320,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BW23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BX23" s="58" t="inlineStr">
+      <c r="BX23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BY23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-25
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BY41"/>
+  <dimension ref="A1:BZ41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -954,14 +954,17 @@
         <v>46257.56858498842</v>
       </c>
       <c r="BW1" s="56" t="n">
-        <v>46258.58133451459</v>
-      </c>
-      <c r="BX1" s="44" t="inlineStr">
+        <v>46258.58133451389</v>
+      </c>
+      <c r="BX1" s="56" t="n">
+        <v>46259.58072687677</v>
+      </c>
+      <c r="BY1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BY1" s="44" t="inlineStr">
+      <c r="BZ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1015,12 +1018,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BX2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY2" s="58" t="inlineStr">
+      <c r="BY2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1074,12 +1077,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BX3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY3" s="58" t="inlineStr">
+      <c r="BY3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1134,12 +1137,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BX4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1204,12 +1207,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BX5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1269,12 +1272,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BX6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1329,12 +1332,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BX7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1415,12 +1418,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BX8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1468,12 +1471,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BX9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1521,12 +1524,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BX10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1569,12 +1572,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BX11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1627,8 +1630,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BX13" s="42" t="n"/>
       <c r="BY13" s="42" t="n"/>
+      <c r="BZ13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1684,12 +1687,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BX14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY14" s="58" t="inlineStr">
+      <c r="BY14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1743,12 +1746,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BX15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BY15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1835,12 +1838,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BX16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY16" s="58" t="inlineStr">
+      <c r="BY16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1919,12 +1922,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BX17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY17" s="58" t="inlineStr">
+      <c r="BY17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1987,12 +1990,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BX18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY18" s="58" t="inlineStr">
+      <c r="BY18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2059,12 +2062,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BX19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY19" s="71" t="inlineStr">
+      <c r="BY19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2128,12 +2131,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BX20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY20" s="58" t="inlineStr">
+      <c r="BY20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2193,12 +2196,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BX21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY21" s="71" t="inlineStr">
+      <c r="BY21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2260,12 +2263,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BX22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY22" s="71" t="inlineStr">
+      <c r="BY22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2320,12 +2323,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BX23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BY23" s="58" t="inlineStr">
+      <c r="BY23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="BZ23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-26
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BZ41"/>
+  <dimension ref="A1:CA41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -957,14 +957,17 @@
         <v>46258.58133451389</v>
       </c>
       <c r="BX1" s="56" t="n">
-        <v>46259.58072687677</v>
-      </c>
-      <c r="BY1" s="44" t="inlineStr">
+        <v>46259.580726875</v>
+      </c>
+      <c r="BY1" s="56" t="n">
+        <v>46260.5830187789</v>
+      </c>
+      <c r="BZ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="BZ1" s="44" t="inlineStr">
+      <c r="CA1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1018,12 +1021,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BY2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ2" s="58" t="inlineStr">
+      <c r="BZ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1077,12 +1080,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BY3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ3" s="58" t="inlineStr">
+      <c r="BZ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1137,12 +1140,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BY4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1207,12 +1210,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BY5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1272,12 +1275,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BY6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1332,12 +1335,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BY7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1418,12 +1421,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BY8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1471,12 +1474,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BY9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1524,12 +1527,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BY10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1572,12 +1575,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BY11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1630,8 +1633,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BY13" s="42" t="n"/>
       <c r="BZ13" s="42" t="n"/>
+      <c r="CA13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1687,12 +1690,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BY14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ14" s="58" t="inlineStr">
+      <c r="BZ14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1746,12 +1749,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BY15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="BZ15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1838,12 +1841,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BY16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ16" s="58" t="inlineStr">
+      <c r="BZ16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1922,12 +1925,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BY17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ17" s="58" t="inlineStr">
+      <c r="BZ17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1990,12 +1993,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BY18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ18" s="58" t="inlineStr">
+      <c r="BZ18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2062,12 +2065,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BY19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ19" s="71" t="inlineStr">
+      <c r="BZ19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2131,12 +2134,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BY20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ20" s="58" t="inlineStr">
+      <c r="BZ20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2196,12 +2199,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BY21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ21" s="71" t="inlineStr">
+      <c r="BZ21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2263,12 +2266,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BY22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ22" s="71" t="inlineStr">
+      <c r="BZ22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2323,12 +2326,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BY23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="BZ23" s="58" t="inlineStr">
+      <c r="BZ23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CA23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-27
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CA41"/>
+  <dimension ref="A1:CB41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -960,14 +960,17 @@
         <v>46259.580726875</v>
       </c>
       <c r="BY1" s="56" t="n">
-        <v>46260.5830187789</v>
-      </c>
-      <c r="BZ1" s="44" t="inlineStr">
+        <v>46260.58301877315</v>
+      </c>
+      <c r="BZ1" s="56" t="n">
+        <v>46261.9551563497</v>
+      </c>
+      <c r="CA1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CA1" s="44" t="inlineStr">
+      <c r="CB1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1021,12 +1024,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BZ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA2" s="58" t="inlineStr">
+      <c r="CA2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1080,12 +1083,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="BZ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA3" s="58" t="inlineStr">
+      <c r="CA3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1140,12 +1143,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="BZ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1210,12 +1213,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="BZ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1275,12 +1278,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BZ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1335,12 +1338,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="BZ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1421,12 +1424,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="BZ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1474,12 +1477,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="BZ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1527,12 +1530,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="BZ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1575,12 +1578,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="BZ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1633,8 +1636,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="BZ13" s="42" t="n"/>
       <c r="CA13" s="42" t="n"/>
+      <c r="CB13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1690,12 +1693,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="BZ14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA14" s="58" t="inlineStr">
+      <c r="CA14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1749,12 +1752,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="BZ15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CA15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1841,12 +1844,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="BZ16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA16" s="58" t="inlineStr">
+      <c r="CA16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1925,12 +1928,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="BZ17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA17" s="58" t="inlineStr">
+      <c r="CA17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1993,12 +1996,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="BZ18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA18" s="58" t="inlineStr">
+      <c r="CA18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2065,12 +2068,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="BZ19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA19" s="71" t="inlineStr">
+      <c r="CA19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2134,12 +2137,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="BZ20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA20" s="58" t="inlineStr">
+      <c r="CA20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2199,12 +2202,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="BZ21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA21" s="71" t="inlineStr">
+      <c r="CA21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2266,12 +2269,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="BZ22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA22" s="71" t="inlineStr">
+      <c r="CA22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2326,12 +2329,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="BZ23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CA23" s="58" t="inlineStr">
+      <c r="CA23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-28
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CB41"/>
+  <dimension ref="A1:CC41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -963,14 +963,17 @@
         <v>46260.58301877315</v>
       </c>
       <c r="BZ1" s="56" t="n">
-        <v>46261.9551563497</v>
-      </c>
-      <c r="CA1" s="44" t="inlineStr">
+        <v>46261.95515635417</v>
+      </c>
+      <c r="CA1" s="56" t="n">
+        <v>46262.95832460877</v>
+      </c>
+      <c r="CB1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CB1" s="44" t="inlineStr">
+      <c r="CC1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1024,12 +1027,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CA2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB2" s="58" t="inlineStr">
+      <c r="CB2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1083,12 +1086,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CA3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB3" s="58" t="inlineStr">
+      <c r="CB3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1143,12 +1146,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CA4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1213,12 +1216,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CA5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1278,12 +1281,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CA6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1338,12 +1341,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CA7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1424,12 +1427,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CA8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1477,12 +1480,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CA9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1530,12 +1533,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CA10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1578,12 +1581,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CA11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1636,8 +1639,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CA13" s="42" t="n"/>
       <c r="CB13" s="42" t="n"/>
+      <c r="CC13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1693,12 +1696,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CA14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB14" s="58" t="inlineStr">
+      <c r="CB14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1752,12 +1755,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CA15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CB15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1844,12 +1847,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CA16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB16" s="58" t="inlineStr">
+      <c r="CB16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1928,12 +1931,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CA17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB17" s="58" t="inlineStr">
+      <c r="CB17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1996,12 +1999,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CA18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB18" s="58" t="inlineStr">
+      <c r="CB18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2068,12 +2071,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CA19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB19" s="71" t="inlineStr">
+      <c r="CB19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2137,12 +2140,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CA20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB20" s="58" t="inlineStr">
+      <c r="CB20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2202,12 +2205,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CA21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB21" s="71" t="inlineStr">
+      <c r="CB21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2269,12 +2272,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CA22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB22" s="71" t="inlineStr">
+      <c r="CB22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2329,12 +2332,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CA23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CB23" s="58" t="inlineStr">
+      <c r="CB23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CC23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-29
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CC41"/>
+  <dimension ref="A1:CD41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -966,14 +966,17 @@
         <v>46261.95515635417</v>
       </c>
       <c r="CA1" s="56" t="n">
-        <v>46262.95832460877</v>
-      </c>
-      <c r="CB1" s="44" t="inlineStr">
+        <v>46262.95832460648</v>
+      </c>
+      <c r="CB1" s="56" t="n">
+        <v>46263.71121492308</v>
+      </c>
+      <c r="CC1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CC1" s="44" t="inlineStr">
+      <c r="CD1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1027,12 +1030,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CB2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC2" s="58" t="inlineStr">
+      <c r="CC2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1086,12 +1089,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CB3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC3" s="58" t="inlineStr">
+      <c r="CC3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1146,12 +1149,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CB4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1216,12 +1219,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CB5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1281,12 +1284,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CB6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1341,12 +1344,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CB7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1427,12 +1430,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CB8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1480,12 +1483,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CB9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1533,12 +1536,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CB10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1581,12 +1584,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CB11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1639,8 +1642,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CB13" s="42" t="n"/>
       <c r="CC13" s="42" t="n"/>
+      <c r="CD13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1696,12 +1699,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CB14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC14" s="58" t="inlineStr">
+      <c r="CC14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1755,12 +1758,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CB15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CC15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1847,12 +1850,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CB16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC16" s="58" t="inlineStr">
+      <c r="CC16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1931,12 +1934,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CB17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC17" s="58" t="inlineStr">
+      <c r="CC17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1999,12 +2002,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CB18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC18" s="58" t="inlineStr">
+      <c r="CC18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2071,12 +2074,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CB19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC19" s="71" t="inlineStr">
+      <c r="CC19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2140,12 +2143,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CB20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC20" s="58" t="inlineStr">
+      <c r="CC20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2205,12 +2208,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CB21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC21" s="71" t="inlineStr">
+      <c r="CC21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2272,12 +2275,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CB22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC22" s="71" t="inlineStr">
+      <c r="CC22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2332,12 +2335,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CB23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CC23" s="58" t="inlineStr">
+      <c r="CC23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CD23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-30
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CD41"/>
+  <dimension ref="A1:CE41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -969,14 +969,17 @@
         <v>46262.95832460648</v>
       </c>
       <c r="CB1" s="56" t="n">
-        <v>46263.71121492308</v>
-      </c>
-      <c r="CC1" s="44" t="inlineStr">
+        <v>46263.71121491898</v>
+      </c>
+      <c r="CC1" s="56" t="n">
+        <v>46264.72132995239</v>
+      </c>
+      <c r="CD1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CD1" s="44" t="inlineStr">
+      <c r="CE1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1030,12 +1033,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CC2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD2" s="58" t="inlineStr">
+      <c r="CD2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1089,12 +1092,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CC3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD3" s="58" t="inlineStr">
+      <c r="CD3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1149,12 +1152,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CC4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1219,12 +1222,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CC5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1284,12 +1287,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CC6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1344,12 +1347,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CC7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1430,12 +1433,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CC8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1483,12 +1486,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CC9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1536,12 +1539,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CC10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1584,12 +1587,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CC11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1642,8 +1645,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CC13" s="42" t="n"/>
       <c r="CD13" s="42" t="n"/>
+      <c r="CE13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1699,12 +1702,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CC14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD14" s="58" t="inlineStr">
+      <c r="CD14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1758,12 +1761,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CC15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CD15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1850,12 +1853,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CC16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD16" s="58" t="inlineStr">
+      <c r="CD16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1934,12 +1937,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CC17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD17" s="58" t="inlineStr">
+      <c r="CD17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2002,12 +2005,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CC18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD18" s="58" t="inlineStr">
+      <c r="CD18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2074,12 +2077,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CC19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD19" s="71" t="inlineStr">
+      <c r="CD19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2143,12 +2146,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CC20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD20" s="58" t="inlineStr">
+      <c r="CD20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2208,12 +2211,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CC21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD21" s="71" t="inlineStr">
+      <c r="CD21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2275,12 +2278,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CC22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD22" s="71" t="inlineStr">
+      <c r="CD22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2335,12 +2338,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CC23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CD23" s="58" t="inlineStr">
+      <c r="CD23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CE23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-08-31
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CE41"/>
+  <dimension ref="A1:CF41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -972,14 +972,17 @@
         <v>46263.71121491898</v>
       </c>
       <c r="CC1" s="56" t="n">
-        <v>46264.72132995239</v>
-      </c>
-      <c r="CD1" s="44" t="inlineStr">
+        <v>46264.7213299537</v>
+      </c>
+      <c r="CD1" s="56" t="n">
+        <v>46265.81185383846</v>
+      </c>
+      <c r="CE1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CE1" s="44" t="inlineStr">
+      <c r="CF1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1033,12 +1036,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CD2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE2" s="58" t="inlineStr">
+      <c r="CE2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1092,12 +1095,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CD3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE3" s="58" t="inlineStr">
+      <c r="CE3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1152,12 +1155,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CD4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1222,12 +1225,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CD5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1287,12 +1290,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CD6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1347,12 +1350,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CD7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1433,12 +1436,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CD8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1486,12 +1489,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CD9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1539,12 +1542,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CD10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1587,12 +1590,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CD11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1645,8 +1648,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CD13" s="42" t="n"/>
       <c r="CE13" s="42" t="n"/>
+      <c r="CF13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1702,12 +1705,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CD14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE14" s="58" t="inlineStr">
+      <c r="CE14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1761,12 +1764,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CD15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CE15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1853,12 +1856,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CD16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE16" s="58" t="inlineStr">
+      <c r="CE16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1937,12 +1940,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CD17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE17" s="58" t="inlineStr">
+      <c r="CE17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2005,12 +2008,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CD18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE18" s="58" t="inlineStr">
+      <c r="CE18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2077,12 +2080,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CD19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE19" s="71" t="inlineStr">
+      <c r="CE19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2146,12 +2149,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CD20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE20" s="58" t="inlineStr">
+      <c r="CE20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2211,12 +2214,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CD21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE21" s="71" t="inlineStr">
+      <c r="CE21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2278,12 +2281,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CD22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE22" s="71" t="inlineStr">
+      <c r="CE22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2338,12 +2341,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CD23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CE23" s="58" t="inlineStr">
+      <c r="CE23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CF23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-01
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CF41"/>
+  <dimension ref="A1:CG41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -975,14 +975,17 @@
         <v>46264.7213299537</v>
       </c>
       <c r="CD1" s="56" t="n">
-        <v>46265.81185383846</v>
-      </c>
-      <c r="CE1" s="44" t="inlineStr">
+        <v>46265.81185384259</v>
+      </c>
+      <c r="CE1" s="56" t="n">
+        <v>46266.72073216853</v>
+      </c>
+      <c r="CF1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CF1" s="44" t="inlineStr">
+      <c r="CG1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1036,12 +1039,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CE2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF2" s="58" t="inlineStr">
+      <c r="CF2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1095,12 +1098,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CE3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF3" s="58" t="inlineStr">
+      <c r="CF3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1155,12 +1158,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CE4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1225,12 +1228,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CE5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1290,12 +1293,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CE6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1350,12 +1353,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CE7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1436,12 +1439,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CE8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1489,12 +1492,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CE9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1542,12 +1545,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CE10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1590,12 +1593,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CE11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1648,8 +1651,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CE13" s="42" t="n"/>
       <c r="CF13" s="42" t="n"/>
+      <c r="CG13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1705,12 +1708,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CE14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF14" s="58" t="inlineStr">
+      <c r="CF14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1764,12 +1767,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CE15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CF15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1856,12 +1859,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CE16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF16" s="58" t="inlineStr">
+      <c r="CF16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1940,12 +1943,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CE17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF17" s="58" t="inlineStr">
+      <c r="CF17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2008,12 +2011,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CE18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF18" s="58" t="inlineStr">
+      <c r="CF18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2080,12 +2083,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CE19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF19" s="71" t="inlineStr">
+      <c r="CF19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2149,12 +2152,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CE20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF20" s="58" t="inlineStr">
+      <c r="CF20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2214,12 +2217,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CE21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF21" s="71" t="inlineStr">
+      <c r="CF21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2281,12 +2284,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CE22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF22" s="71" t="inlineStr">
+      <c r="CF22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2341,12 +2344,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CE23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CF23" s="58" t="inlineStr">
+      <c r="CF23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CG23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-02
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CG41"/>
+  <dimension ref="A1:CH41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -978,14 +978,17 @@
         <v>46265.81185384259</v>
       </c>
       <c r="CE1" s="56" t="n">
-        <v>46266.72073216853</v>
-      </c>
-      <c r="CF1" s="44" t="inlineStr">
+        <v>46266.72073216435</v>
+      </c>
+      <c r="CF1" s="56" t="n">
+        <v>46267.7132605185</v>
+      </c>
+      <c r="CG1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CG1" s="44" t="inlineStr">
+      <c r="CH1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1039,12 +1042,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CF2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG2" s="58" t="inlineStr">
+      <c r="CG2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1098,12 +1101,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CF3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG3" s="58" t="inlineStr">
+      <c r="CG3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1158,12 +1161,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CF4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1228,12 +1231,12 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CF5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1293,12 +1296,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CF6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1353,12 +1356,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CF7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1439,12 +1442,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CF8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1492,12 +1495,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CF9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1545,12 +1548,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CF10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1593,12 +1596,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CF11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1651,8 +1654,8 @@
       <c r="AJ13" s="42" t="n"/>
       <c r="AN13" s="42" t="n"/>
       <c r="AP13" s="42" t="n"/>
-      <c r="CF13" s="42" t="n"/>
       <c r="CG13" s="42" t="n"/>
+      <c r="CH13" s="42" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1708,12 +1711,12 @@
       <c r="AJ14" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CF14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG14" s="58" t="inlineStr">
+      <c r="CG14" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH14" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1767,12 +1770,12 @@
       <c r="AI15" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CF15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CG15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH15" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1859,12 +1862,12 @@
       <c r="AC16" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CF16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG16" s="58" t="inlineStr">
+      <c r="CG16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1943,12 +1946,12 @@
       <c r="W17" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CF17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG17" s="58" t="inlineStr">
+      <c r="CG17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2011,12 +2014,12 @@
       <c r="W18" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CF18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG18" s="58" t="inlineStr">
+      <c r="CG18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2083,12 +2086,12 @@
       <c r="Q19" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CF19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG19" s="71" t="inlineStr">
+      <c r="CG19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH19" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2152,12 +2155,12 @@
       <c r="O20" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CF20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG20" s="58" t="inlineStr">
+      <c r="CG20" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2217,12 +2220,12 @@
         <v>1964.85</v>
       </c>
       <c r="O21" s="69" t="n"/>
-      <c r="CF21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG21" s="71" t="inlineStr">
+      <c r="CG21" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2284,12 +2287,12 @@
       <c r="M22" s="83" t="n"/>
       <c r="N22" s="84" t="n"/>
       <c r="O22" s="69" t="n"/>
-      <c r="CF22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG22" s="71" t="inlineStr">
+      <c r="CG22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2344,12 +2347,12 @@
       <c r="L23" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CF23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CG23" s="58" t="inlineStr">
+      <c r="CG23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CH23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-03
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CH41"/>
+  <dimension ref="A1:CI42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -981,14 +981,17 @@
         <v>46266.72073216435</v>
       </c>
       <c r="CF1" s="56" t="n">
-        <v>46267.7132605185</v>
-      </c>
-      <c r="CG1" s="44" t="inlineStr">
+        <v>46267.71326052083</v>
+      </c>
+      <c r="CG1" s="56" t="n">
+        <v>46268.70873561063</v>
+      </c>
+      <c r="CH1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CH1" s="44" t="inlineStr">
+      <c r="CI1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1042,12 +1045,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CG2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH2" s="58" t="inlineStr">
+      <c r="CH2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1101,12 +1104,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CG3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH3" s="58" t="inlineStr">
+      <c r="CH3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1161,12 +1164,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CG4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1231,12 +1234,15 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CG5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CG5" t="n">
+        <v>2469.06</v>
       </c>
       <c r="CH5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1296,12 +1302,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CG6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1356,12 +1362,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CG7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1442,12 +1448,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CG8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1495,12 +1501,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CG9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1548,12 +1554,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CG10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1596,12 +1602,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CG11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CH11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1638,94 +1644,64 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="n"/>
-      <c r="C13" s="42" t="n"/>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="42" t="n"/>
-      <c r="F13" s="42" t="n"/>
-      <c r="G13" s="42" t="n"/>
-      <c r="H13" s="42" t="n"/>
-      <c r="AH13" s="42" t="n"/>
-      <c r="AJ13" s="42" t="n"/>
-      <c r="AN13" s="42" t="n"/>
-      <c r="AP13" s="42" t="n"/>
-      <c r="CG13" s="42" t="n"/>
-      <c r="CH13" s="42" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>#9-482B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>814</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Oct 07</t>
+        </is>
+      </c>
+      <c r="CG13" t="n">
+        <v>2504.06</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C14" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D14" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E14" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F14" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G14" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H14" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z14" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB14" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE14" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG14" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ14" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CG14" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH14" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="42" t="n"/>
+      <c r="E14" s="42" t="n"/>
+      <c r="F14" s="42" t="n"/>
+      <c r="G14" s="42" t="n"/>
+      <c r="H14" s="42" t="n"/>
+      <c r="AH14" s="42" t="n"/>
+      <c r="AJ14" s="42" t="n"/>
+      <c r="AN14" s="42" t="n"/>
+      <c r="AP14" s="42" t="n"/>
+      <c r="CH14" s="42" t="n"/>
+      <c r="CI14" s="42" t="n"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B15" s="42" t="inlineStr">
@@ -1735,25 +1711,25 @@
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D15" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E15" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F15" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G15" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H15" s="42" t="inlineStr">
@@ -1761,21 +1737,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF15" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z15" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB15" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE15" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG15" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI15" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CG15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ15" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CH15" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI15" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1784,581 +1766,639 @@
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E16" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F16" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H16" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF16" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG16" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI16" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CH16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1" s="43">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B17" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C17" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D16" s="42" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E16" s="42" t="n">
+      <c r="E17" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F16" s="42" t="inlineStr">
+      <c r="F17" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G16" s="42" t="inlineStr">
+      <c r="G17" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H16" s="42" t="inlineStr">
+      <c r="H17" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I16" s="42" t="n">
+      <c r="I17" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J16" s="42" t="n">
+      <c r="J17" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K16" s="42" t="n">
+      <c r="K17" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L16" s="42" t="n">
+      <c r="L17" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N16" s="42" t="n">
+      <c r="N17" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O16" s="42" t="n">
+      <c r="O17" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q16" s="42" t="n">
+      <c r="Q17" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T16" s="42" t="n">
+      <c r="T17" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U16" s="42" t="n">
+      <c r="U17" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V16" s="42" t="n">
+      <c r="V17" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W16" s="42" t="n">
+      <c r="W17" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA16" s="42" t="n">
+      <c r="AA17" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB16" s="42" t="n">
+      <c r="AB17" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC16" s="42" t="n">
+      <c r="AC17" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CG16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH16" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1" s="43">
-      <c r="A17" s="61" t="inlineStr">
+      <c r="CH17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI17" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="43">
+      <c r="A18" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B17" s="62" t="inlineStr">
+      <c r="B18" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C18" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D17" s="61" t="inlineStr">
+      <c r="D18" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E17" s="63" t="n">
+      <c r="E18" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F17" s="64" t="inlineStr">
+      <c r="F18" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G17" s="64" t="inlineStr">
+      <c r="G18" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H17" s="65" t="inlineStr">
+      <c r="H18" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I17" s="66" t="n">
+      <c r="I18" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J17" s="67" t="n">
+      <c r="J18" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K17" s="66" t="n">
+      <c r="K18" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L17" s="68" t="n">
+      <c r="L18" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M17" s="68" t="n"/>
-      <c r="N17" s="69" t="n">
+      <c r="M18" s="68" t="n"/>
+      <c r="N18" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O17" s="69" t="n">
+      <c r="O18" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q17" s="42" t="n">
+      <c r="Q18" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T17" s="42" t="n">
+      <c r="T18" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U17" s="42" t="n">
+      <c r="U18" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V17" s="42" t="n">
+      <c r="V18" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W17" s="42" t="n">
+      <c r="W18" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CG17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH17" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="43">
-      <c r="A18" s="42" t="inlineStr">
+      <c r="CH18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI18" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="43">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D18" s="42" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E18" s="42" t="n">
+      <c r="E19" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F18" s="42" t="inlineStr">
+      <c r="F19" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G18" s="42" t="inlineStr">
+      <c r="G19" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H18" s="42" t="inlineStr">
+      <c r="H19" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I18" s="42" t="n">
+      <c r="I19" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M18" s="42" t="n">
+      <c r="M19" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N18" s="42" t="n">
+      <c r="N19" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q18" s="42" t="n">
+      <c r="Q19" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V18" s="42" t="n">
+      <c r="V19" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W18" s="42" t="n">
+      <c r="W19" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CG18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH18" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" s="61" t="inlineStr">
+      <c r="CH19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI19" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="43">
+      <c r="A20" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="B20" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D19" s="61" t="inlineStr">
+      <c r="D20" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E19" s="63" t="n">
+      <c r="E20" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F19" s="64" t="inlineStr">
+      <c r="F20" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G19" s="64" t="inlineStr">
+      <c r="G20" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H19" s="65" t="inlineStr">
+      <c r="H20" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I19" s="66" t="n">
+      <c r="I20" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J19" s="67" t="n">
+      <c r="J20" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K19" s="66" t="n">
+      <c r="K20" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L19" s="68" t="n">
+      <c r="L20" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M19" s="68" t="n"/>
-      <c r="N19" s="69" t="n">
+      <c r="M20" s="68" t="n"/>
+      <c r="N20" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O19" s="69" t="n">
+      <c r="O20" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q19" s="42" t="n">
+      <c r="Q20" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CG19" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH19" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="CH20" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI20" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D20" s="42" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E21" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F20" s="42" t="inlineStr">
+      <c r="F21" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G20" s="42" t="inlineStr">
+      <c r="G21" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H20" s="42" t="inlineStr">
+      <c r="H21" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="72" t="n">
+      <c r="I21" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J20" s="72" t="n">
+      <c r="J21" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K20" s="72" t="n">
+      <c r="K21" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L20" s="72" t="n">
+      <c r="L21" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M20" s="72" t="n"/>
-      <c r="N20" s="42" t="n">
+      <c r="M21" s="72" t="n"/>
+      <c r="N21" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O20" s="42" t="n">
+      <c r="O21" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CG20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH20" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="61" t="inlineStr">
+      <c r="CH21" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI21" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="B22" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="61" t="inlineStr">
+      <c r="C22" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D21" s="61" t="inlineStr">
+      <c r="D22" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E21" s="64" t="n">
+      <c r="E22" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F21" s="64" t="inlineStr">
+      <c r="F22" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G21" s="73" t="n">
+      <c r="G22" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H21" s="65" t="inlineStr">
+      <c r="H22" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="66" t="n">
+      <c r="I22" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J21" s="66" t="n">
+      <c r="J22" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K21" s="67" t="n">
+      <c r="K22" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L21" s="68" t="n">
+      <c r="L22" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M21" s="68" t="n"/>
-      <c r="N21" s="69" t="n">
+      <c r="M22" s="68" t="n"/>
+      <c r="N22" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O21" s="69" t="n"/>
-      <c r="CG21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH21" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="75" t="inlineStr">
+      <c r="O22" s="69" t="n"/>
+      <c r="CH22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI22" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B22" s="76" t="inlineStr">
+      <c r="B23" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="75" t="inlineStr">
+      <c r="C23" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D22" s="75" t="inlineStr">
+      <c r="D23" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E22" s="77" t="n">
+      <c r="E23" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F22" s="78" t="inlineStr">
+      <c r="F23" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G22" s="79" t="n">
+      <c r="G23" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H22" s="80" t="inlineStr">
+      <c r="H23" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I22" s="81" t="n">
+      <c r="I23" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J22" s="81" t="n">
+      <c r="J23" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K22" s="82" t="inlineStr">
+      <c r="K23" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L22" s="83" t="inlineStr">
+      <c r="L23" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M22" s="83" t="n"/>
-      <c r="N22" s="84" t="n"/>
-      <c r="O22" s="69" t="n"/>
-      <c r="CG22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH22" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="42" t="inlineStr">
+      <c r="M23" s="83" t="n"/>
+      <c r="N23" s="84" t="n"/>
+      <c r="O23" s="69" t="n"/>
+      <c r="CH23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI23" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B24" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E24" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F23" s="42" t="inlineStr">
+      <c r="F24" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G23" s="47" t="n">
+      <c r="G24" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H23" s="42" t="inlineStr">
+      <c r="H24" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="72" t="n">
+      <c r="I24" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J23" s="72" t="n">
+      <c r="J24" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K23" s="72" t="n">
+      <c r="K24" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L23" s="72" t="n">
+      <c r="L24" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CG23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CH23" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43"/>
+      <c r="CH24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CI24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="15.75" customHeight="1" s="43"/>
     <row r="26" ht="15.75" customHeight="1" s="43"/>
     <row r="27" ht="15.75" customHeight="1" s="43"/>
@@ -2366,29 +2406,30 @@
     <row r="29"/>
     <row r="30"/>
     <row r="31" ht="15.75" customHeight="1" s="43"/>
-    <row r="32">
-      <c r="A32" s="42" t="n"/>
-    </row>
-    <row r="33"/>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="42" t="n"/>
+    </row>
     <row r="34" ht="15.75" customHeight="1" s="43"/>
-    <row r="35" ht="15.75" customHeight="1" s="43">
-      <c r="A35" s="42" t="n"/>
-    </row>
+    <row r="35" ht="15.75" customHeight="1" s="43"/>
     <row r="36" ht="15.75" customHeight="1" s="43">
       <c r="A36" s="42" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="42" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="43"/>
-    <row r="39" ht="15.75" customHeight="1" s="43">
-      <c r="A39" s="42" t="n"/>
-    </row>
+    <row r="38" ht="15.75" customHeight="1" s="43">
+      <c r="A38" s="42" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="43"/>
     <row r="40" ht="15.75" customHeight="1" s="43">
       <c r="A40" s="42" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="42" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-04
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CI42"/>
+  <dimension ref="A1:CJ43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -984,14 +984,17 @@
         <v>46267.71326052083</v>
       </c>
       <c r="CG1" s="56" t="n">
-        <v>46268.70873561063</v>
-      </c>
-      <c r="CH1" s="44" t="inlineStr">
+        <v>46268.70873561343</v>
+      </c>
+      <c r="CH1" s="56" t="n">
+        <v>46269.70105107836</v>
+      </c>
+      <c r="CI1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CI1" s="44" t="inlineStr">
+      <c r="CJ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1045,12 +1048,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CH2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI2" s="58" t="inlineStr">
+      <c r="CI2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1104,12 +1107,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CH3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI3" s="58" t="inlineStr">
+      <c r="CI3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1164,12 +1167,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CH4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1234,15 +1237,15 @@
       <c r="BJ5" s="59" t="n">
         <v>2441.06</v>
       </c>
-      <c r="CG5" t="n">
+      <c r="CG5" s="42" t="n">
         <v>2469.06</v>
       </c>
-      <c r="CH5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1302,12 +1305,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CH6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1362,12 +1365,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CH7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1448,12 +1451,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CH8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1501,12 +1504,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CH9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1554,12 +1557,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CH10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1602,12 +1605,12 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CH11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CI11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1644,129 +1647,99 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>#9-482B</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="42" t="inlineStr">
         <is>
           <t>814</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="42" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="42" t="inlineStr">
         <is>
           <t>Oct 07</t>
         </is>
       </c>
-      <c r="CG13" t="n">
+      <c r="CG13" s="42" t="n">
         <v>2504.06</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B14" s="42" t="n"/>
-      <c r="C14" s="42" t="n"/>
-      <c r="D14" s="42" t="n"/>
-      <c r="E14" s="42" t="n"/>
-      <c r="F14" s="42" t="n"/>
-      <c r="G14" s="42" t="n"/>
-      <c r="H14" s="42" t="n"/>
-      <c r="AH14" s="42" t="n"/>
-      <c r="AJ14" s="42" t="n"/>
-      <c r="AN14" s="42" t="n"/>
-      <c r="AP14" s="42" t="n"/>
-      <c r="CH14" s="42" t="n"/>
-      <c r="CI14" s="42" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>#5-428</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2 bed, 2.5 bath</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1313</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>B31</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Sep 28</t>
+        </is>
+      </c>
+      <c r="CH14" t="n">
+        <v>3718.06</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C15" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E15" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F15" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G15" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z15" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB15" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE15" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG15" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ15" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CH15" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI15" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="42" t="n"/>
+      <c r="F15" s="42" t="n"/>
+      <c r="G15" s="42" t="n"/>
+      <c r="H15" s="42" t="n"/>
+      <c r="AH15" s="42" t="n"/>
+      <c r="AJ15" s="42" t="n"/>
+      <c r="AN15" s="42" t="n"/>
+      <c r="AP15" s="42" t="n"/>
+      <c r="CI15" s="42" t="n"/>
+      <c r="CJ15" s="42" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B16" s="42" t="inlineStr">
@@ -1776,25 +1749,25 @@
       </c>
       <c r="C16" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D16" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E16" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F16" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G16" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H16" s="42" t="inlineStr">
@@ -1802,21 +1775,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF16" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z16" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB16" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE16" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG16" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI16" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CH16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ16" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CI16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1825,581 +1804,639 @@
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C17" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E17" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F17" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H17" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF17" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG17" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI17" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CI17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="43">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n">
+      <c r="E18" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F17" s="42" t="inlineStr">
+      <c r="F18" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G17" s="42" t="inlineStr">
+      <c r="G18" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H17" s="42" t="inlineStr">
+      <c r="H18" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I17" s="42" t="n">
+      <c r="I18" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J17" s="42" t="n">
+      <c r="J18" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K17" s="42" t="n">
+      <c r="K18" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L17" s="42" t="n">
+      <c r="L18" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N17" s="42" t="n">
+      <c r="N18" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O17" s="42" t="n">
+      <c r="O18" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q17" s="42" t="n">
+      <c r="Q18" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T17" s="42" t="n">
+      <c r="T18" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U17" s="42" t="n">
+      <c r="U18" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V17" s="42" t="n">
+      <c r="V18" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W17" s="42" t="n">
+      <c r="W18" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA17" s="42" t="n">
+      <c r="AA18" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB17" s="42" t="n">
+      <c r="AB18" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC17" s="42" t="n">
+      <c r="AC18" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CH17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI17" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="43">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="CI18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ18" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="43">
+      <c r="A19" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B18" s="62" t="inlineStr">
+      <c r="B19" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C19" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D18" s="61" t="inlineStr">
+      <c r="D19" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E18" s="63" t="n">
+      <c r="E19" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F18" s="64" t="inlineStr">
+      <c r="F19" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G18" s="64" t="inlineStr">
+      <c r="G19" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H18" s="65" t="inlineStr">
+      <c r="H19" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I18" s="66" t="n">
+      <c r="I19" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J18" s="67" t="n">
+      <c r="J19" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K18" s="66" t="n">
+      <c r="K19" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L18" s="68" t="n">
+      <c r="L19" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M18" s="68" t="n"/>
-      <c r="N18" s="69" t="n">
+      <c r="M19" s="68" t="n"/>
+      <c r="N19" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O18" s="69" t="n">
+      <c r="O19" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q18" s="42" t="n">
+      <c r="Q19" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T18" s="42" t="n">
+      <c r="T19" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U18" s="42" t="n">
+      <c r="U19" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V18" s="42" t="n">
+      <c r="V19" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W18" s="42" t="n">
+      <c r="W19" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CH18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI18" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="CI19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ19" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="43">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E19" s="42" t="n">
+      <c r="E20" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F19" s="42" t="inlineStr">
+      <c r="F20" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G19" s="42" t="inlineStr">
+      <c r="G20" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H19" s="42" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I19" s="42" t="n">
+      <c r="I20" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M19" s="42" t="n">
+      <c r="M20" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N19" s="42" t="n">
+      <c r="N20" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q19" s="42" t="n">
+      <c r="Q20" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V19" s="42" t="n">
+      <c r="V20" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W19" s="42" t="n">
+      <c r="W20" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CH19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI19" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="61" t="inlineStr">
+      <c r="CI20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ20" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="B21" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C21" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D20" s="61" t="inlineStr">
+      <c r="D21" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E20" s="63" t="n">
+      <c r="E21" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F20" s="64" t="inlineStr">
+      <c r="F21" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G20" s="64" t="inlineStr">
+      <c r="G21" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H20" s="65" t="inlineStr">
+      <c r="H21" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="66" t="n">
+      <c r="I21" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J20" s="67" t="n">
+      <c r="J21" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K20" s="66" t="n">
+      <c r="K21" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L20" s="68" t="n">
+      <c r="L21" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M20" s="68" t="n"/>
-      <c r="N20" s="69" t="n">
+      <c r="M21" s="68" t="n"/>
+      <c r="N21" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O20" s="69" t="n">
+      <c r="O21" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q20" s="42" t="n">
+      <c r="Q21" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CH20" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI20" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="42" t="inlineStr">
+      <c r="CI21" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ21" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E21" s="42" t="n">
+      <c r="E22" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F21" s="42" t="inlineStr">
+      <c r="F22" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="G22" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H21" s="42" t="inlineStr">
+      <c r="H22" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="72" t="n">
+      <c r="I22" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J21" s="72" t="n">
+      <c r="J22" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K21" s="72" t="n">
+      <c r="K22" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L21" s="72" t="n">
+      <c r="L22" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M21" s="72" t="n"/>
-      <c r="N21" s="42" t="n">
+      <c r="M22" s="72" t="n"/>
+      <c r="N22" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O21" s="42" t="n">
+      <c r="O22" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CH21" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI21" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="61" t="inlineStr">
+      <c r="CI22" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ22" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B22" s="62" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="61" t="inlineStr">
+      <c r="C23" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D22" s="61" t="inlineStr">
+      <c r="D23" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="64" t="n">
+      <c r="E23" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F22" s="64" t="inlineStr">
+      <c r="F23" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G22" s="73" t="n">
+      <c r="G23" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H22" s="65" t="inlineStr">
+      <c r="H23" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="66" t="n">
+      <c r="I23" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J22" s="66" t="n">
+      <c r="J23" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K22" s="67" t="n">
+      <c r="K23" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L22" s="68" t="n">
+      <c r="L23" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M22" s="68" t="n"/>
-      <c r="N22" s="69" t="n">
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O22" s="69" t="n"/>
-      <c r="CH22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI22" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="75" t="inlineStr">
+      <c r="O23" s="69" t="n"/>
+      <c r="CI23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ23" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B23" s="76" t="inlineStr">
+      <c r="B24" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="75" t="inlineStr">
+      <c r="C24" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D23" s="75" t="inlineStr">
+      <c r="D24" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E23" s="77" t="n">
+      <c r="E24" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F23" s="78" t="inlineStr">
+      <c r="F24" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G23" s="79" t="n">
+      <c r="G24" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H23" s="80" t="inlineStr">
+      <c r="H24" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I23" s="81" t="n">
+      <c r="I24" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J23" s="81" t="n">
+      <c r="J24" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K23" s="82" t="inlineStr">
+      <c r="K24" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L23" s="83" t="inlineStr">
+      <c r="L24" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M23" s="83" t="n"/>
-      <c r="N23" s="84" t="n"/>
-      <c r="O23" s="69" t="n"/>
-      <c r="CH23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI23" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="M24" s="83" t="n"/>
+      <c r="N24" s="84" t="n"/>
+      <c r="O24" s="69" t="n"/>
+      <c r="CI24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ24" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B25" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="42" t="inlineStr">
+      <c r="C25" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D24" s="42" t="inlineStr">
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E25" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F24" s="42" t="inlineStr">
+      <c r="F25" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G24" s="47" t="n">
+      <c r="G25" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H24" s="42" t="inlineStr">
+      <c r="H25" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="72" t="n">
+      <c r="I25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J24" s="72" t="n">
+      <c r="J25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K24" s="72" t="n">
+      <c r="K25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L24" s="72" t="n">
+      <c r="L25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CH24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CI24" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43"/>
+      <c r="CI25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CJ25" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="15.75" customHeight="1" s="43"/>
     <row r="27" ht="15.75" customHeight="1" s="43"/>
     <row r="28" ht="15.75" customHeight="1" s="43"/>
@@ -2407,29 +2444,30 @@
     <row r="30"/>
     <row r="31" ht="15.75" customHeight="1" s="43"/>
     <row r="32"/>
-    <row r="33">
-      <c r="A33" s="42" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="43"/>
+    <row r="33"/>
+    <row r="34" ht="15.75" customHeight="1" s="43">
+      <c r="A34" s="42" t="n"/>
+    </row>
     <row r="35" ht="15.75" customHeight="1" s="43"/>
-    <row r="36" ht="15.75" customHeight="1" s="43">
-      <c r="A36" s="42" t="n"/>
-    </row>
+    <row r="36" ht="15.75" customHeight="1" s="43"/>
     <row r="37">
       <c r="A37" s="42" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="43">
       <c r="A38" s="42" t="n"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1" s="43"/>
-    <row r="40" ht="15.75" customHeight="1" s="43">
-      <c r="A40" s="42" t="n"/>
-    </row>
+    <row r="39" ht="15.75" customHeight="1" s="43">
+      <c r="A39" s="42" t="n"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="43"/>
     <row r="41">
       <c r="A41" s="42" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="42" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-06
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CJ43"/>
+  <dimension ref="A1:CK43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -987,14 +987,17 @@
         <v>46268.70873561343</v>
       </c>
       <c r="CH1" s="56" t="n">
-        <v>46269.70105107836</v>
-      </c>
-      <c r="CI1" s="44" t="inlineStr">
+        <v>46269.70105107639</v>
+      </c>
+      <c r="CI1" s="56" t="n">
+        <v>46271.67262636655</v>
+      </c>
+      <c r="CJ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CJ1" s="44" t="inlineStr">
+      <c r="CK1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1048,12 +1051,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CI2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ2" s="58" t="inlineStr">
+      <c r="CJ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1107,12 +1110,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CI3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ3" s="58" t="inlineStr">
+      <c r="CJ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1167,12 +1170,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CI4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1240,12 +1243,15 @@
       <c r="CG5" s="42" t="n">
         <v>2469.06</v>
       </c>
-      <c r="CI5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CI5" t="n">
+        <v>2418.06</v>
       </c>
       <c r="CJ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1305,12 +1311,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CI6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1365,12 +1371,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CI7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1451,12 +1457,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CI8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1504,12 +1510,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CI9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1557,12 +1563,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CI10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1605,12 +1611,15 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CI11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CI11" t="n">
+        <v>2581.06</v>
       </c>
       <c r="CJ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1645,6 +1654,9 @@
       <c r="BK12" s="42" t="n">
         <v>2064.06</v>
       </c>
+      <c r="CI12" t="n">
+        <v>2044.06</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -1680,40 +1692,46 @@
       <c r="CG13" s="42" t="n">
         <v>2504.06</v>
       </c>
+      <c r="CI13" t="n">
+        <v>2482.06</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>#5-428</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
         <is>
           <t>1313</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="42" t="inlineStr">
         <is>
           <t>B31</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="42" t="inlineStr">
         <is>
           <t>Sep 28</t>
         </is>
       </c>
-      <c r="CH14" t="n">
+      <c r="CH14" s="42" t="n">
         <v>3718.06</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>3684.06</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
@@ -1733,8 +1751,8 @@
       <c r="AJ15" s="42" t="n"/>
       <c r="AN15" s="42" t="n"/>
       <c r="AP15" s="42" t="n"/>
-      <c r="CI15" s="42" t="n"/>
       <c r="CJ15" s="42" t="n"/>
+      <c r="CK15" s="42" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
@@ -1790,12 +1808,12 @@
       <c r="AJ16" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CI16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ16" s="58" t="inlineStr">
+      <c r="CJ16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1849,12 +1867,12 @@
       <c r="AI17" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CI17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CJ17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK17" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1941,12 +1959,12 @@
       <c r="AC18" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CI18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ18" s="58" t="inlineStr">
+      <c r="CJ18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2025,12 +2043,12 @@
       <c r="W19" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CI19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ19" s="58" t="inlineStr">
+      <c r="CJ19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2093,12 +2111,12 @@
       <c r="W20" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CI20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ20" s="58" t="inlineStr">
+      <c r="CJ20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2165,12 +2183,12 @@
       <c r="Q21" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CI21" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ21" s="71" t="inlineStr">
+      <c r="CJ21" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2234,12 +2252,12 @@
       <c r="O22" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CI22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ22" s="58" t="inlineStr">
+      <c r="CJ22" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2299,12 +2317,12 @@
         <v>1964.85</v>
       </c>
       <c r="O23" s="69" t="n"/>
-      <c r="CI23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ23" s="71" t="inlineStr">
+      <c r="CJ23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2366,12 +2384,12 @@
       <c r="M24" s="83" t="n"/>
       <c r="N24" s="84" t="n"/>
       <c r="O24" s="69" t="n"/>
-      <c r="CI24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ24" s="71" t="inlineStr">
+      <c r="CJ24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2426,12 +2444,12 @@
       <c r="L25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CI25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CJ25" s="58" t="inlineStr">
+      <c r="CJ25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CK25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-07
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CK43"/>
+  <dimension ref="A1:CL43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -990,14 +990,17 @@
         <v>46269.70105107639</v>
       </c>
       <c r="CI1" s="56" t="n">
-        <v>46271.67262636655</v>
-      </c>
-      <c r="CJ1" s="44" t="inlineStr">
+        <v>46271.67262636574</v>
+      </c>
+      <c r="CJ1" s="56" t="n">
+        <v>46272.75873433046</v>
+      </c>
+      <c r="CK1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CK1" s="44" t="inlineStr">
+      <c r="CL1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1051,12 +1054,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CJ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK2" s="58" t="inlineStr">
+      <c r="CK2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1110,12 +1113,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CJ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK3" s="58" t="inlineStr">
+      <c r="CK3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1170,12 +1173,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CJ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1243,15 +1246,18 @@
       <c r="CG5" s="42" t="n">
         <v>2469.06</v>
       </c>
-      <c r="CI5" t="n">
+      <c r="CI5" s="42" t="n">
         <v>2418.06</v>
       </c>
-      <c r="CJ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CJ5" t="n">
+        <v>2390.06</v>
       </c>
       <c r="CK5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1311,12 +1317,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CJ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1371,12 +1377,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CJ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1457,12 +1463,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CJ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1510,12 +1516,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CJ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1563,12 +1569,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CJ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1611,15 +1617,15 @@
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
-      <c r="CI11" t="n">
+      <c r="CI11" s="42" t="n">
         <v>2581.06</v>
       </c>
-      <c r="CJ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1654,7 +1660,7 @@
       <c r="BK12" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CI12" t="n">
+      <c r="CI12" s="42" t="n">
         <v>2044.06</v>
       </c>
     </row>
@@ -1692,7 +1698,7 @@
       <c r="CG13" s="42" t="n">
         <v>2504.06</v>
       </c>
-      <c r="CI13" t="n">
+      <c r="CI13" s="42" t="n">
         <v>2482.06</v>
       </c>
     </row>
@@ -1730,7 +1736,7 @@
       <c r="CH14" s="42" t="n">
         <v>3718.06</v>
       </c>
-      <c r="CI14" t="n">
+      <c r="CI14" s="42" t="n">
         <v>3684.06</v>
       </c>
     </row>
@@ -1751,8 +1757,8 @@
       <c r="AJ15" s="42" t="n"/>
       <c r="AN15" s="42" t="n"/>
       <c r="AP15" s="42" t="n"/>
-      <c r="CJ15" s="42" t="n"/>
       <c r="CK15" s="42" t="n"/>
+      <c r="CL15" s="42" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
@@ -1808,12 +1814,12 @@
       <c r="AJ16" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CJ16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK16" s="58" t="inlineStr">
+      <c r="CK16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1867,12 +1873,12 @@
       <c r="AI17" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CJ17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CK17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL17" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1959,12 +1965,12 @@
       <c r="AC18" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CJ18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK18" s="58" t="inlineStr">
+      <c r="CK18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2043,12 +2049,12 @@
       <c r="W19" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CJ19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK19" s="58" t="inlineStr">
+      <c r="CK19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2111,12 +2117,12 @@
       <c r="W20" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CJ20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK20" s="58" t="inlineStr">
+      <c r="CK20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2183,12 +2189,12 @@
       <c r="Q21" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CJ21" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK21" s="71" t="inlineStr">
+      <c r="CK21" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2252,12 +2258,12 @@
       <c r="O22" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CJ22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK22" s="58" t="inlineStr">
+      <c r="CK22" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2317,12 +2323,12 @@
         <v>1964.85</v>
       </c>
       <c r="O23" s="69" t="n"/>
-      <c r="CJ23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK23" s="71" t="inlineStr">
+      <c r="CK23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2384,12 +2390,12 @@
       <c r="M24" s="83" t="n"/>
       <c r="N24" s="84" t="n"/>
       <c r="O24" s="69" t="n"/>
-      <c r="CJ24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK24" s="71" t="inlineStr">
+      <c r="CK24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2444,12 +2450,12 @@
       <c r="L25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CJ25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CK25" s="58" t="inlineStr">
+      <c r="CK25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CL25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-08
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CL43"/>
+  <dimension ref="A1:CM43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -993,14 +993,17 @@
         <v>46271.67262636574</v>
       </c>
       <c r="CJ1" s="56" t="n">
-        <v>46272.75873433046</v>
-      </c>
-      <c r="CK1" s="44" t="inlineStr">
+        <v>46272.7587343287</v>
+      </c>
+      <c r="CK1" s="56" t="n">
+        <v>46273.71742669532</v>
+      </c>
+      <c r="CL1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CL1" s="44" t="inlineStr">
+      <c r="CM1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1054,12 +1057,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CK2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL2" s="58" t="inlineStr">
+      <c r="CL2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1113,12 +1116,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CK3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL3" s="58" t="inlineStr">
+      <c r="CL3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1173,12 +1176,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CK4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1249,15 +1252,15 @@
       <c r="CI5" s="42" t="n">
         <v>2418.06</v>
       </c>
-      <c r="CJ5" t="n">
+      <c r="CJ5" s="42" t="n">
         <v>2390.06</v>
       </c>
-      <c r="CK5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1317,12 +1320,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CK6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1377,12 +1380,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CK7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1463,12 +1466,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CK8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1516,12 +1519,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CK9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1569,12 +1572,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CK10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1620,12 +1623,12 @@
       <c r="CI11" s="42" t="n">
         <v>2581.06</v>
       </c>
-      <c r="CK11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1757,8 +1760,8 @@
       <c r="AJ15" s="42" t="n"/>
       <c r="AN15" s="42" t="n"/>
       <c r="AP15" s="42" t="n"/>
-      <c r="CK15" s="42" t="n"/>
       <c r="CL15" s="42" t="n"/>
+      <c r="CM15" s="42" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
@@ -1814,12 +1817,12 @@
       <c r="AJ16" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CK16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL16" s="58" t="inlineStr">
+      <c r="CL16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1873,12 +1876,12 @@
       <c r="AI17" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CK17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CL17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM17" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1965,12 +1968,12 @@
       <c r="AC18" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CK18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL18" s="58" t="inlineStr">
+      <c r="CL18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2049,12 +2052,12 @@
       <c r="W19" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CK19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL19" s="58" t="inlineStr">
+      <c r="CL19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2117,12 +2120,12 @@
       <c r="W20" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CK20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL20" s="58" t="inlineStr">
+      <c r="CL20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2189,12 +2192,12 @@
       <c r="Q21" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CK21" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL21" s="71" t="inlineStr">
+      <c r="CL21" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2258,12 +2261,12 @@
       <c r="O22" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CK22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL22" s="58" t="inlineStr">
+      <c r="CL22" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2323,12 +2326,12 @@
         <v>1964.85</v>
       </c>
       <c r="O23" s="69" t="n"/>
-      <c r="CK23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL23" s="71" t="inlineStr">
+      <c r="CL23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2390,12 +2393,12 @@
       <c r="M24" s="83" t="n"/>
       <c r="N24" s="84" t="n"/>
       <c r="O24" s="69" t="n"/>
-      <c r="CK24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL24" s="71" t="inlineStr">
+      <c r="CL24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2450,12 +2453,12 @@
       <c r="L25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CK25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CL25" s="58" t="inlineStr">
+      <c r="CL25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CM25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-09
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CM43"/>
+  <dimension ref="A1:CN43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -996,14 +996,17 @@
         <v>46272.7587343287</v>
       </c>
       <c r="CK1" s="56" t="n">
-        <v>46273.71742669532</v>
-      </c>
-      <c r="CL1" s="44" t="inlineStr">
+        <v>46273.71742668981</v>
+      </c>
+      <c r="CL1" s="56" t="n">
+        <v>46274.71308054416</v>
+      </c>
+      <c r="CM1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CM1" s="44" t="inlineStr">
+      <c r="CN1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1057,12 +1060,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CL2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM2" s="58" t="inlineStr">
+      <c r="CM2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1116,12 +1119,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CL3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM3" s="58" t="inlineStr">
+      <c r="CM3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1176,12 +1179,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CL4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1255,12 +1258,12 @@
       <c r="CJ5" s="42" t="n">
         <v>2390.06</v>
       </c>
-      <c r="CL5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1320,12 +1323,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CL6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1380,12 +1383,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CL7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1466,12 +1469,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CL8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1519,12 +1522,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CL9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1572,12 +1575,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CL10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1623,12 +1626,12 @@
       <c r="CI11" s="42" t="n">
         <v>2581.06</v>
       </c>
-      <c r="CL11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1760,8 +1763,8 @@
       <c r="AJ15" s="42" t="n"/>
       <c r="AN15" s="42" t="n"/>
       <c r="AP15" s="42" t="n"/>
-      <c r="CL15" s="42" t="n"/>
       <c r="CM15" s="42" t="n"/>
+      <c r="CN15" s="42" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
@@ -1817,12 +1820,12 @@
       <c r="AJ16" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CL16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM16" s="58" t="inlineStr">
+      <c r="CM16" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN16" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1876,12 +1879,12 @@
       <c r="AI17" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CL17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CM17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN17" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1968,12 +1971,12 @@
       <c r="AC18" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CL18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM18" s="58" t="inlineStr">
+      <c r="CM18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2052,12 +2055,12 @@
       <c r="W19" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CL19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM19" s="58" t="inlineStr">
+      <c r="CM19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2120,12 +2123,12 @@
       <c r="W20" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CL20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM20" s="58" t="inlineStr">
+      <c r="CM20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2192,12 +2195,12 @@
       <c r="Q21" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CL21" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM21" s="71" t="inlineStr">
+      <c r="CM21" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN21" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2261,12 +2264,12 @@
       <c r="O22" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CL22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM22" s="58" t="inlineStr">
+      <c r="CM22" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2326,12 +2329,12 @@
         <v>1964.85</v>
       </c>
       <c r="O23" s="69" t="n"/>
-      <c r="CL23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM23" s="71" t="inlineStr">
+      <c r="CM23" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2393,12 +2396,12 @@
       <c r="M24" s="83" t="n"/>
       <c r="N24" s="84" t="n"/>
       <c r="O24" s="69" t="n"/>
-      <c r="CL24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM24" s="71" t="inlineStr">
+      <c r="CM24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2453,12 +2456,12 @@
       <c r="L25" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CL25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CM25" s="58" t="inlineStr">
+      <c r="CM25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CN25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-10
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CN43"/>
+  <dimension ref="A1:CO44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -999,14 +999,17 @@
         <v>46273.71742668981</v>
       </c>
       <c r="CL1" s="56" t="n">
-        <v>46274.71308054416</v>
-      </c>
-      <c r="CM1" s="44" t="inlineStr">
+        <v>46274.71308054398</v>
+      </c>
+      <c r="CM1" s="56" t="n">
+        <v>46275.7069701232</v>
+      </c>
+      <c r="CN1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CN1" s="44" t="inlineStr">
+      <c r="CO1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1060,12 +1063,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CM2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN2" s="58" t="inlineStr">
+      <c r="CN2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1119,12 +1122,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CM3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN3" s="58" t="inlineStr">
+      <c r="CN3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1179,12 +1182,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CM4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1258,12 +1261,15 @@
       <c r="CJ5" s="42" t="n">
         <v>2390.06</v>
       </c>
-      <c r="CM5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CM5" t="n">
+        <v>2371.06</v>
       </c>
       <c r="CN5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1323,12 +1329,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CM6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1383,12 +1389,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CM7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1469,12 +1475,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CM8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1522,12 +1528,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CM9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1575,12 +1581,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CM10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CN10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1626,12 +1632,15 @@
       <c r="CI11" s="42" t="n">
         <v>2581.06</v>
       </c>
-      <c r="CM11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CM11" t="n">
+        <v>2558.06</v>
       </c>
       <c r="CN11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1669,6 +1678,9 @@
       <c r="CI12" s="42" t="n">
         <v>2044.06</v>
       </c>
+      <c r="CM12" t="n">
+        <v>2024.06</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -1707,6 +1719,9 @@
       <c r="CI13" s="42" t="n">
         <v>2482.06</v>
       </c>
+      <c r="CM13" t="n">
+        <v>2459.06</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -1739,6 +1754,11 @@
           <t>Sep 28</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="CH14" s="42" t="n">
         <v>3718.06</v>
       </c>
@@ -1747,94 +1767,64 @@
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="n"/>
-      <c r="C15" s="42" t="n"/>
-      <c r="D15" s="42" t="n"/>
-      <c r="E15" s="42" t="n"/>
-      <c r="F15" s="42" t="n"/>
-      <c r="G15" s="42" t="n"/>
-      <c r="H15" s="42" t="n"/>
-      <c r="AH15" s="42" t="n"/>
-      <c r="AJ15" s="42" t="n"/>
-      <c r="AN15" s="42" t="n"/>
-      <c r="AP15" s="42" t="n"/>
-      <c r="CM15" s="42" t="n"/>
-      <c r="CN15" s="42" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>#8-466B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2 bed, 2 bath</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1065</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Oct 07</t>
+        </is>
+      </c>
+      <c r="CM15" t="n">
+        <v>3410.06</v>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
       <c r="A16" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C16" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D16" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E16" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F16" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G16" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H16" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z16" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB16" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE16" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG16" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ16" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CM16" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN16" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="n"/>
+      <c r="C16" s="42" t="n"/>
+      <c r="D16" s="42" t="n"/>
+      <c r="E16" s="42" t="n"/>
+      <c r="F16" s="42" t="n"/>
+      <c r="G16" s="42" t="n"/>
+      <c r="H16" s="42" t="n"/>
+      <c r="AH16" s="42" t="n"/>
+      <c r="AJ16" s="42" t="n"/>
+      <c r="AN16" s="42" t="n"/>
+      <c r="AP16" s="42" t="n"/>
+      <c r="CN16" s="42" t="n"/>
+      <c r="CO16" s="42" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B17" s="42" t="inlineStr">
@@ -1844,25 +1834,25 @@
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E17" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F17" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G17" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H17" s="42" t="inlineStr">
@@ -1870,21 +1860,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF17" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z17" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB17" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE17" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG17" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI17" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CM17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ17" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CN17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1893,581 +1889,639 @@
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C18" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E18" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F18" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H18" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF18" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG18" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI18" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CN18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="43">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D18" s="42" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E18" s="42" t="n">
+      <c r="E19" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F18" s="42" t="inlineStr">
+      <c r="F19" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G18" s="42" t="inlineStr">
+      <c r="G19" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H18" s="42" t="inlineStr">
+      <c r="H19" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I18" s="42" t="n">
+      <c r="I19" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J18" s="42" t="n">
+      <c r="J19" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K18" s="42" t="n">
+      <c r="K19" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L18" s="42" t="n">
+      <c r="L19" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N18" s="42" t="n">
+      <c r="N19" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O18" s="42" t="n">
+      <c r="O19" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q18" s="42" t="n">
+      <c r="Q19" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T18" s="42" t="n">
+      <c r="T19" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U18" s="42" t="n">
+      <c r="U19" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V18" s="42" t="n">
+      <c r="V19" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W18" s="42" t="n">
+      <c r="W19" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA18" s="42" t="n">
+      <c r="AA19" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB18" s="42" t="n">
+      <c r="AB19" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC18" s="42" t="n">
+      <c r="AC19" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CM18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN18" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" s="61" t="inlineStr">
+      <c r="CN19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO19" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="43">
+      <c r="A20" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="B20" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D19" s="61" t="inlineStr">
+      <c r="D20" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E19" s="63" t="n">
+      <c r="E20" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F19" s="64" t="inlineStr">
+      <c r="F20" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G19" s="64" t="inlineStr">
+      <c r="G20" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H19" s="65" t="inlineStr">
+      <c r="H20" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I19" s="66" t="n">
+      <c r="I20" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J19" s="67" t="n">
+      <c r="J20" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K19" s="66" t="n">
+      <c r="K20" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L19" s="68" t="n">
+      <c r="L20" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M19" s="68" t="n"/>
-      <c r="N19" s="69" t="n">
+      <c r="M20" s="68" t="n"/>
+      <c r="N20" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O19" s="69" t="n">
+      <c r="O20" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q19" s="42" t="n">
+      <c r="Q20" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T19" s="42" t="n">
+      <c r="T20" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U19" s="42" t="n">
+      <c r="U20" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V19" s="42" t="n">
+      <c r="V20" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W19" s="42" t="n">
+      <c r="W20" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CM19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN19" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="CN20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO20" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D20" s="42" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E21" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F20" s="42" t="inlineStr">
+      <c r="F21" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G20" s="42" t="inlineStr">
+      <c r="G21" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H20" s="42" t="inlineStr">
+      <c r="H21" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="42" t="n">
+      <c r="I21" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M20" s="42" t="n">
+      <c r="M21" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N20" s="42" t="n">
+      <c r="N21" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q20" s="42" t="n">
+      <c r="Q21" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V20" s="42" t="n">
+      <c r="V21" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W20" s="42" t="n">
+      <c r="W21" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CM20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN20" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="61" t="inlineStr">
+      <c r="CN21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO21" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="B22" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="61" t="inlineStr">
+      <c r="C22" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D21" s="61" t="inlineStr">
+      <c r="D22" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E21" s="63" t="n">
+      <c r="E22" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F21" s="64" t="inlineStr">
+      <c r="F22" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G21" s="64" t="inlineStr">
+      <c r="G22" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H21" s="65" t="inlineStr">
+      <c r="H22" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="66" t="n">
+      <c r="I22" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J21" s="67" t="n">
+      <c r="J22" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K21" s="66" t="n">
+      <c r="K22" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L21" s="68" t="n">
+      <c r="L22" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M21" s="68" t="n"/>
-      <c r="N21" s="69" t="n">
+      <c r="M22" s="68" t="n"/>
+      <c r="N22" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O21" s="69" t="n">
+      <c r="O22" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q21" s="42" t="n">
+      <c r="Q22" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CM21" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN21" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="42" t="inlineStr">
+      <c r="CN22" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO22" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E23" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F22" s="42" t="inlineStr">
+      <c r="F23" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G22" s="42" t="inlineStr">
+      <c r="G23" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H22" s="42" t="inlineStr">
+      <c r="H23" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="72" t="n">
+      <c r="I23" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J22" s="72" t="n">
+      <c r="J23" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K22" s="72" t="n">
+      <c r="K23" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L22" s="72" t="n">
+      <c r="L23" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M22" s="72" t="n"/>
-      <c r="N22" s="42" t="n">
+      <c r="M23" s="72" t="n"/>
+      <c r="N23" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O22" s="42" t="n">
+      <c r="O23" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CM22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN22" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="CN23" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B24" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="61" t="inlineStr">
+      <c r="C24" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D23" s="61" t="inlineStr">
+      <c r="D24" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="64" t="n">
+      <c r="E24" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F23" s="64" t="inlineStr">
+      <c r="F24" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G23" s="73" t="n">
+      <c r="G24" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H23" s="65" t="inlineStr">
+      <c r="H24" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="66" t="n">
+      <c r="I24" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J23" s="66" t="n">
+      <c r="J24" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K23" s="67" t="n">
+      <c r="K24" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L23" s="68" t="n">
+      <c r="L24" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M23" s="68" t="n"/>
-      <c r="N23" s="69" t="n">
+      <c r="M24" s="68" t="n"/>
+      <c r="N24" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O23" s="69" t="n"/>
-      <c r="CM23" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN23" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="75" t="inlineStr">
+      <c r="O24" s="69" t="n"/>
+      <c r="CN24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO24" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B24" s="76" t="inlineStr">
+      <c r="B25" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="75" t="inlineStr">
+      <c r="C25" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D24" s="75" t="inlineStr">
+      <c r="D25" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E24" s="77" t="n">
+      <c r="E25" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F24" s="78" t="inlineStr">
+      <c r="F25" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G24" s="79" t="n">
+      <c r="G25" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H24" s="80" t="inlineStr">
+      <c r="H25" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I24" s="81" t="n">
+      <c r="I25" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J24" s="81" t="n">
+      <c r="J25" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K24" s="82" t="inlineStr">
+      <c r="K25" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L24" s="83" t="inlineStr">
+      <c r="L25" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M24" s="83" t="n"/>
-      <c r="N24" s="84" t="n"/>
-      <c r="O24" s="69" t="n"/>
-      <c r="CM24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN24" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="42" t="inlineStr">
+      <c r="M25" s="83" t="n"/>
+      <c r="N25" s="84" t="n"/>
+      <c r="O25" s="69" t="n"/>
+      <c r="CN25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO25" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C26" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D25" s="42" t="inlineStr">
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E25" s="42" t="n">
+      <c r="E26" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F25" s="42" t="inlineStr">
+      <c r="F26" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G25" s="47" t="n">
+      <c r="G26" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H25" s="42" t="inlineStr">
+      <c r="H26" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I25" s="72" t="n">
+      <c r="I26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J25" s="72" t="n">
+      <c r="J26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K25" s="72" t="n">
+      <c r="K26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L25" s="72" t="n">
+      <c r="L26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CM25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CN25" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43"/>
+      <c r="CN26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CO26" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="27" ht="15.75" customHeight="1" s="43"/>
     <row r="28" ht="15.75" customHeight="1" s="43"/>
     <row r="29"/>
@@ -2475,29 +2529,30 @@
     <row r="31" ht="15.75" customHeight="1" s="43"/>
     <row r="32"/>
     <row r="33"/>
-    <row r="34" ht="15.75" customHeight="1" s="43">
-      <c r="A34" s="42" t="n"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" s="43"/>
+    <row r="34" ht="15.75" customHeight="1" s="43"/>
+    <row r="35" ht="15.75" customHeight="1" s="43">
+      <c r="A35" s="42" t="n"/>
+    </row>
     <row r="36" ht="15.75" customHeight="1" s="43"/>
-    <row r="37">
-      <c r="A37" s="42" t="n"/>
-    </row>
+    <row r="37"/>
     <row r="38" ht="15.75" customHeight="1" s="43">
       <c r="A38" s="42" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="43">
       <c r="A39" s="42" t="n"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1" s="43"/>
-    <row r="41">
-      <c r="A41" s="42" t="n"/>
-    </row>
+    <row r="40" ht="15.75" customHeight="1" s="43">
+      <c r="A40" s="42" t="n"/>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="42" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="42" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-11
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CO44"/>
+  <dimension ref="A1:CP44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1002,14 +1002,17 @@
         <v>46274.71308054398</v>
       </c>
       <c r="CM1" s="56" t="n">
-        <v>46275.7069701232</v>
-      </c>
-      <c r="CN1" s="44" t="inlineStr">
+        <v>46275.70697012731</v>
+      </c>
+      <c r="CN1" s="56" t="n">
+        <v>46276.70813928841</v>
+      </c>
+      <c r="CO1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CO1" s="44" t="inlineStr">
+      <c r="CP1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1063,12 +1066,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CN2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO2" s="58" t="inlineStr">
+      <c r="CO2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1122,12 +1125,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CN3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO3" s="58" t="inlineStr">
+      <c r="CO3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1182,12 +1185,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CN4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1261,15 +1264,15 @@
       <c r="CJ5" s="42" t="n">
         <v>2390.06</v>
       </c>
-      <c r="CM5" t="n">
+      <c r="CM5" s="42" t="n">
         <v>2371.06</v>
       </c>
-      <c r="CN5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1329,12 +1332,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CN6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1389,12 +1392,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CN7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1475,12 +1478,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CN8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1528,12 +1531,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CN9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1581,12 +1584,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CN10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1632,15 +1635,15 @@
       <c r="CI11" s="42" t="n">
         <v>2581.06</v>
       </c>
-      <c r="CM11" t="n">
+      <c r="CM11" s="42" t="n">
         <v>2558.06</v>
       </c>
-      <c r="CN11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1678,7 +1681,7 @@
       <c r="CI12" s="42" t="n">
         <v>2044.06</v>
       </c>
-      <c r="CM12" t="n">
+      <c r="CM12" s="42" t="n">
         <v>2024.06</v>
       </c>
     </row>
@@ -1719,7 +1722,7 @@
       <c r="CI13" s="42" t="n">
         <v>2482.06</v>
       </c>
-      <c r="CM13" t="n">
+      <c r="CM13" s="42" t="n">
         <v>2459.06</v>
       </c>
     </row>
@@ -1754,7 +1757,7 @@
           <t>Sep 28</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1767,37 +1770,37 @@
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>#8-466B</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>2 bed, 2 bath</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="42" t="inlineStr">
         <is>
           <t>1065</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="42" t="inlineStr">
         <is>
           <t>B17</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="42" t="inlineStr">
         <is>
           <t>Oct 07</t>
         </is>
       </c>
-      <c r="CM15" t="n">
+      <c r="CM15" s="42" t="n">
         <v>3410.06</v>
       </c>
     </row>
@@ -1818,8 +1821,8 @@
       <c r="AJ16" s="42" t="n"/>
       <c r="AN16" s="42" t="n"/>
       <c r="AP16" s="42" t="n"/>
-      <c r="CN16" s="42" t="n"/>
       <c r="CO16" s="42" t="n"/>
+      <c r="CP16" s="42" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -1875,12 +1878,12 @@
       <c r="AJ17" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CN17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO17" s="58" t="inlineStr">
+      <c r="CO17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1934,12 +1937,12 @@
       <c r="AI18" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CN18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CO18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP18" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2026,12 +2029,12 @@
       <c r="AC19" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CN19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO19" s="58" t="inlineStr">
+      <c r="CO19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2110,12 +2113,12 @@
       <c r="W20" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CN20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO20" s="58" t="inlineStr">
+      <c r="CO20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2178,12 +2181,12 @@
       <c r="W21" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CN21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO21" s="58" t="inlineStr">
+      <c r="CO21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2250,12 +2253,12 @@
       <c r="Q22" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CN22" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO22" s="71" t="inlineStr">
+      <c r="CO22" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2319,12 +2322,12 @@
       <c r="O23" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CN23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO23" s="58" t="inlineStr">
+      <c r="CO23" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2384,12 +2387,12 @@
         <v>1964.85</v>
       </c>
       <c r="O24" s="69" t="n"/>
-      <c r="CN24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO24" s="71" t="inlineStr">
+      <c r="CO24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2451,12 +2454,12 @@
       <c r="M25" s="83" t="n"/>
       <c r="N25" s="84" t="n"/>
       <c r="O25" s="69" t="n"/>
-      <c r="CN25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO25" s="71" t="inlineStr">
+      <c r="CO25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2511,12 +2514,12 @@
       <c r="L26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CN26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CO26" s="58" t="inlineStr">
+      <c r="CO26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CP26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-13
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CP44"/>
+  <dimension ref="A1:CQ44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1005,14 +1005,17 @@
         <v>46275.70697012731</v>
       </c>
       <c r="CN1" s="56" t="n">
-        <v>46276.70813928841</v>
-      </c>
-      <c r="CO1" s="44" t="inlineStr">
+        <v>46276.70813929398</v>
+      </c>
+      <c r="CO1" s="56" t="n">
+        <v>46278.70608798438</v>
+      </c>
+      <c r="CP1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CP1" s="44" t="inlineStr">
+      <c r="CQ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1066,12 +1069,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CO2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP2" s="58" t="inlineStr">
+      <c r="CP2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1125,12 +1128,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CO3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP3" s="58" t="inlineStr">
+      <c r="CP3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1185,12 +1188,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CO4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1267,12 +1270,15 @@
       <c r="CM5" s="42" t="n">
         <v>2371.06</v>
       </c>
-      <c r="CO5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CO5" t="n">
+        <v>2352.06</v>
       </c>
       <c r="CP5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1332,12 +1338,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CO6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1392,12 +1398,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CO7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1478,12 +1484,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CO8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1531,12 +1537,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CO9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1584,12 +1590,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CO10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1638,12 +1644,12 @@
       <c r="CM11" s="42" t="n">
         <v>2558.06</v>
       </c>
-      <c r="CO11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1684,6 +1690,9 @@
       <c r="CM12" s="42" t="n">
         <v>2024.06</v>
       </c>
+      <c r="CO12" t="n">
+        <v>2004.06</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -1802,6 +1811,9 @@
       </c>
       <c r="CM15" s="42" t="n">
         <v>3410.06</v>
+      </c>
+      <c r="CO15" t="n">
+        <v>3377.06</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
@@ -1821,8 +1833,8 @@
       <c r="AJ16" s="42" t="n"/>
       <c r="AN16" s="42" t="n"/>
       <c r="AP16" s="42" t="n"/>
-      <c r="CO16" s="42" t="n"/>
       <c r="CP16" s="42" t="n"/>
+      <c r="CQ16" s="42" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -1878,12 +1890,12 @@
       <c r="AJ17" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CO17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP17" s="58" t="inlineStr">
+      <c r="CP17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1937,12 +1949,12 @@
       <c r="AI18" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CO18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CP18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ18" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2029,12 +2041,12 @@
       <c r="AC19" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CO19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP19" s="58" t="inlineStr">
+      <c r="CP19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2113,12 +2125,12 @@
       <c r="W20" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CO20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP20" s="58" t="inlineStr">
+      <c r="CP20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2181,12 +2193,12 @@
       <c r="W21" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CO21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP21" s="58" t="inlineStr">
+      <c r="CP21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2253,12 +2265,12 @@
       <c r="Q22" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CO22" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP22" s="71" t="inlineStr">
+      <c r="CP22" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2322,12 +2334,12 @@
       <c r="O23" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CO23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP23" s="58" t="inlineStr">
+      <c r="CP23" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2387,12 +2399,12 @@
         <v>1964.85</v>
       </c>
       <c r="O24" s="69" t="n"/>
-      <c r="CO24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP24" s="71" t="inlineStr">
+      <c r="CP24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2454,12 +2466,12 @@
       <c r="M25" s="83" t="n"/>
       <c r="N25" s="84" t="n"/>
       <c r="O25" s="69" t="n"/>
-      <c r="CO25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP25" s="71" t="inlineStr">
+      <c r="CP25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2514,12 +2526,12 @@
       <c r="L26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CO26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CP26" s="58" t="inlineStr">
+      <c r="CP26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CQ26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-14
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CQ44"/>
+  <dimension ref="A1:CR44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1008,14 +1008,17 @@
         <v>46276.70813929398</v>
       </c>
       <c r="CO1" s="56" t="n">
-        <v>46278.70608798438</v>
-      </c>
-      <c r="CP1" s="44" t="inlineStr">
+        <v>46278.70608798611</v>
+      </c>
+      <c r="CP1" s="56" t="n">
+        <v>46279.77128908392</v>
+      </c>
+      <c r="CQ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CQ1" s="44" t="inlineStr">
+      <c r="CR1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1069,12 +1072,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CP2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ2" s="58" t="inlineStr">
+      <c r="CQ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1128,12 +1131,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CP3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ3" s="58" t="inlineStr">
+      <c r="CQ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1188,12 +1191,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CP4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1270,15 +1273,15 @@
       <c r="CM5" s="42" t="n">
         <v>2371.06</v>
       </c>
-      <c r="CO5" t="n">
+      <c r="CO5" s="42" t="n">
         <v>2352.06</v>
       </c>
-      <c r="CP5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1338,12 +1341,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CP6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1398,12 +1401,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CP7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1484,12 +1487,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CP8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1537,12 +1540,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CP9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1590,12 +1593,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CP10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1644,12 +1647,12 @@
       <c r="CM11" s="42" t="n">
         <v>2558.06</v>
       </c>
-      <c r="CP11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1690,7 +1693,7 @@
       <c r="CM12" s="42" t="n">
         <v>2024.06</v>
       </c>
-      <c r="CO12" t="n">
+      <c r="CO12" s="42" t="n">
         <v>2004.06</v>
       </c>
     </row>
@@ -1725,6 +1728,11 @@
           <t>Oct 07</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="CG13" s="42" t="n">
         <v>2504.06</v>
       </c>
@@ -1812,7 +1820,7 @@
       <c r="CM15" s="42" t="n">
         <v>3410.06</v>
       </c>
-      <c r="CO15" t="n">
+      <c r="CO15" s="42" t="n">
         <v>3377.06</v>
       </c>
     </row>
@@ -1833,8 +1841,8 @@
       <c r="AJ16" s="42" t="n"/>
       <c r="AN16" s="42" t="n"/>
       <c r="AP16" s="42" t="n"/>
-      <c r="CP16" s="42" t="n"/>
       <c r="CQ16" s="42" t="n"/>
+      <c r="CR16" s="42" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -1890,12 +1898,12 @@
       <c r="AJ17" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CP17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ17" s="58" t="inlineStr">
+      <c r="CQ17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1949,12 +1957,12 @@
       <c r="AI18" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CP18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CQ18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR18" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2041,12 +2049,12 @@
       <c r="AC19" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CP19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ19" s="58" t="inlineStr">
+      <c r="CQ19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2125,12 +2133,12 @@
       <c r="W20" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CP20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ20" s="58" t="inlineStr">
+      <c r="CQ20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2193,12 +2201,12 @@
       <c r="W21" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CP21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ21" s="58" t="inlineStr">
+      <c r="CQ21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2265,12 +2273,12 @@
       <c r="Q22" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CP22" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ22" s="71" t="inlineStr">
+      <c r="CQ22" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2334,12 +2342,12 @@
       <c r="O23" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CP23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ23" s="58" t="inlineStr">
+      <c r="CQ23" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2399,12 +2407,12 @@
         <v>1964.85</v>
       </c>
       <c r="O24" s="69" t="n"/>
-      <c r="CP24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ24" s="71" t="inlineStr">
+      <c r="CQ24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2466,12 +2474,12 @@
       <c r="M25" s="83" t="n"/>
       <c r="N25" s="84" t="n"/>
       <c r="O25" s="69" t="n"/>
-      <c r="CP25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ25" s="71" t="inlineStr">
+      <c r="CQ25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2526,12 +2534,12 @@
       <c r="L26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CP26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CQ26" s="58" t="inlineStr">
+      <c r="CQ26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CR26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-16
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CR44"/>
+  <dimension ref="A1:CS44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1011,14 +1011,17 @@
         <v>46278.70608798611</v>
       </c>
       <c r="CP1" s="56" t="n">
-        <v>46279.77128908392</v>
-      </c>
-      <c r="CQ1" s="44" t="inlineStr">
+        <v>46279.77128908565</v>
+      </c>
+      <c r="CQ1" s="56" t="n">
+        <v>46281.73324260033</v>
+      </c>
+      <c r="CR1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CR1" s="44" t="inlineStr">
+      <c r="CS1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1072,12 +1075,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CQ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR2" s="58" t="inlineStr">
+      <c r="CR2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1131,12 +1134,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CQ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR3" s="58" t="inlineStr">
+      <c r="CR3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1191,12 +1194,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CQ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1276,12 +1279,15 @@
       <c r="CO5" s="42" t="n">
         <v>2352.06</v>
       </c>
-      <c r="CQ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CQ5" t="n">
+        <v>2334.35</v>
       </c>
       <c r="CR5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1341,12 +1347,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CQ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1401,12 +1407,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CQ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1487,12 +1493,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CQ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1540,12 +1546,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CQ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1593,12 +1599,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CQ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1647,12 +1653,15 @@
       <c r="CM11" s="42" t="n">
         <v>2558.06</v>
       </c>
-      <c r="CQ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CQ11" t="n">
+        <v>2581.35</v>
       </c>
       <c r="CR11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1696,6 +1705,9 @@
       <c r="CO12" s="42" t="n">
         <v>2004.06</v>
       </c>
+      <c r="CQ12" t="n">
+        <v>1985.35</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -1728,7 +1740,7 @@
           <t>Oct 07</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1785,6 +1797,9 @@
       <c r="CI14" s="42" t="n">
         <v>3684.06</v>
       </c>
+      <c r="CQ14" t="n">
+        <v>3584.35</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
@@ -1815,6 +1830,11 @@
       <c r="G15" s="42" t="inlineStr">
         <is>
           <t>Oct 07</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Off Market</t>
         </is>
       </c>
       <c r="CM15" s="42" t="n">
@@ -1841,8 +1861,8 @@
       <c r="AJ16" s="42" t="n"/>
       <c r="AN16" s="42" t="n"/>
       <c r="AP16" s="42" t="n"/>
-      <c r="CQ16" s="42" t="n"/>
       <c r="CR16" s="42" t="n"/>
+      <c r="CS16" s="42" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -1898,12 +1918,12 @@
       <c r="AJ17" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CQ17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR17" s="58" t="inlineStr">
+      <c r="CR17" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS17" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1957,12 +1977,12 @@
       <c r="AI18" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CQ18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CR18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS18" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2049,12 +2069,12 @@
       <c r="AC19" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CQ19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR19" s="58" t="inlineStr">
+      <c r="CR19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2133,12 +2153,12 @@
       <c r="W20" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CQ20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR20" s="58" t="inlineStr">
+      <c r="CR20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2201,12 +2221,12 @@
       <c r="W21" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CQ21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR21" s="58" t="inlineStr">
+      <c r="CR21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2273,12 +2293,12 @@
       <c r="Q22" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CQ22" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR22" s="71" t="inlineStr">
+      <c r="CR22" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS22" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2342,12 +2362,12 @@
       <c r="O23" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CQ23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR23" s="58" t="inlineStr">
+      <c r="CR23" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2407,12 +2427,12 @@
         <v>1964.85</v>
       </c>
       <c r="O24" s="69" t="n"/>
-      <c r="CQ24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR24" s="71" t="inlineStr">
+      <c r="CR24" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2474,12 +2494,12 @@
       <c r="M25" s="83" t="n"/>
       <c r="N25" s="84" t="n"/>
       <c r="O25" s="69" t="n"/>
-      <c r="CQ25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR25" s="71" t="inlineStr">
+      <c r="CR25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2534,12 +2554,12 @@
       <c r="L26" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CQ26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CR26" s="58" t="inlineStr">
+      <c r="CR26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CS26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-20
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CS44"/>
+  <dimension ref="A1:CT45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1014,14 +1014,17 @@
         <v>46279.77128908565</v>
       </c>
       <c r="CQ1" s="56" t="n">
-        <v>46281.73324260033</v>
-      </c>
-      <c r="CR1" s="44" t="inlineStr">
+        <v>46281.73324260417</v>
+      </c>
+      <c r="CR1" s="56" t="n">
+        <v>46285.69801302979</v>
+      </c>
+      <c r="CS1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CS1" s="44" t="inlineStr">
+      <c r="CT1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1075,12 +1078,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CR2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS2" s="58" t="inlineStr">
+      <c r="CS2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1134,12 +1137,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CR3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS3" s="58" t="inlineStr">
+      <c r="CS3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1194,12 +1197,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CR4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1279,15 +1282,18 @@
       <c r="CO5" s="42" t="n">
         <v>2352.06</v>
       </c>
-      <c r="CQ5" t="n">
+      <c r="CQ5" s="42" t="n">
         <v>2334.35</v>
       </c>
-      <c r="CR5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CR5" t="n">
+        <v>2239.35</v>
       </c>
       <c r="CS5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1347,12 +1353,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CR6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1407,12 +1413,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CR7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1493,12 +1499,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CR8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1546,12 +1552,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CR9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1599,12 +1605,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CR10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1653,15 +1659,15 @@
       <c r="CM11" s="42" t="n">
         <v>2558.06</v>
       </c>
-      <c r="CQ11" t="n">
+      <c r="CQ11" s="42" t="n">
         <v>2581.35</v>
       </c>
-      <c r="CR11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CS11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1705,8 +1711,11 @@
       <c r="CO12" s="42" t="n">
         <v>2004.06</v>
       </c>
-      <c r="CQ12" t="n">
+      <c r="CQ12" s="42" t="n">
         <v>1985.35</v>
+      </c>
+      <c r="CR12" t="n">
+        <v>1986.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1797,8 +1806,11 @@
       <c r="CI14" s="42" t="n">
         <v>3684.06</v>
       </c>
-      <c r="CQ14" t="n">
+      <c r="CQ14" s="42" t="n">
         <v>3584.35</v>
+      </c>
+      <c r="CR14" t="n">
+        <v>3519.35</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
@@ -1832,7 +1844,7 @@
           <t>Oct 07</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1845,94 +1857,64 @@
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="n"/>
-      <c r="C16" s="42" t="n"/>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="42" t="n"/>
-      <c r="F16" s="42" t="n"/>
-      <c r="G16" s="42" t="n"/>
-      <c r="H16" s="42" t="n"/>
-      <c r="AH16" s="42" t="n"/>
-      <c r="AJ16" s="42" t="n"/>
-      <c r="AN16" s="42" t="n"/>
-      <c r="AP16" s="42" t="n"/>
-      <c r="CR16" s="42" t="n"/>
-      <c r="CS16" s="42" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>#8-460C</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1 bath</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>732</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Oct 13</t>
+        </is>
+      </c>
+      <c r="CR16" t="n">
+        <v>2158.35</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C17" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E17" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F17" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G17" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H17" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z17" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB17" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE17" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG17" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ17" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CR17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS17" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="n"/>
+      <c r="C17" s="42" t="n"/>
+      <c r="D17" s="42" t="n"/>
+      <c r="E17" s="42" t="n"/>
+      <c r="F17" s="42" t="n"/>
+      <c r="G17" s="42" t="n"/>
+      <c r="H17" s="42" t="n"/>
+      <c r="AH17" s="42" t="n"/>
+      <c r="AJ17" s="42" t="n"/>
+      <c r="AN17" s="42" t="n"/>
+      <c r="AP17" s="42" t="n"/>
+      <c r="CS17" s="42" t="n"/>
+      <c r="CT17" s="42" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B18" s="42" t="inlineStr">
@@ -1942,25 +1924,25 @@
       </c>
       <c r="C18" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D18" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E18" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F18" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G18" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H18" s="42" t="inlineStr">
@@ -1968,21 +1950,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF18" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z18" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB18" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE18" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG18" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI18" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CR18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ18" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CS18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1991,581 +1979,639 @@
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E19" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F19" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G19" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H19" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF19" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG19" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI19" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CS19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="43">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E19" s="42" t="n">
+      <c r="E20" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F19" s="42" t="inlineStr">
+      <c r="F20" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G19" s="42" t="inlineStr">
+      <c r="G20" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H19" s="42" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I19" s="42" t="n">
+      <c r="I20" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J19" s="42" t="n">
+      <c r="J20" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K19" s="42" t="n">
+      <c r="K20" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L19" s="42" t="n">
+      <c r="L20" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N19" s="42" t="n">
+      <c r="N20" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O19" s="42" t="n">
+      <c r="O20" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q19" s="42" t="n">
+      <c r="Q20" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T19" s="42" t="n">
+      <c r="T20" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U19" s="42" t="n">
+      <c r="U20" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V19" s="42" t="n">
+      <c r="V20" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W19" s="42" t="n">
+      <c r="W20" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA19" s="42" t="n">
+      <c r="AA20" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB19" s="42" t="n">
+      <c r="AB20" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC19" s="42" t="n">
+      <c r="AC20" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CR19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS19" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="61" t="inlineStr">
+      <c r="CS20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT20" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="B21" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C21" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D20" s="61" t="inlineStr">
+      <c r="D21" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" s="63" t="n">
+      <c r="E21" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F20" s="64" t="inlineStr">
+      <c r="F21" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G20" s="64" t="inlineStr">
+      <c r="G21" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H20" s="65" t="inlineStr">
+      <c r="H21" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="66" t="n">
+      <c r="I21" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J20" s="67" t="n">
+      <c r="J21" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K20" s="66" t="n">
+      <c r="K21" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L20" s="68" t="n">
+      <c r="L21" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M20" s="68" t="n"/>
-      <c r="N20" s="69" t="n">
+      <c r="M21" s="68" t="n"/>
+      <c r="N21" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O20" s="69" t="n">
+      <c r="O21" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q20" s="42" t="n">
+      <c r="Q21" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T20" s="42" t="n">
+      <c r="T21" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U20" s="42" t="n">
+      <c r="U21" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V20" s="42" t="n">
+      <c r="V21" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W20" s="42" t="n">
+      <c r="W21" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CR20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS20" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="42" t="inlineStr">
+      <c r="CS21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT21" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E21" s="42" t="n">
+      <c r="E22" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F21" s="42" t="inlineStr">
+      <c r="F22" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="G22" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H21" s="42" t="inlineStr">
+      <c r="H22" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="42" t="n">
+      <c r="I22" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M21" s="42" t="n">
+      <c r="M22" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N21" s="42" t="n">
+      <c r="N22" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q21" s="42" t="n">
+      <c r="Q22" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V21" s="42" t="n">
+      <c r="V22" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W21" s="42" t="n">
+      <c r="W22" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CR21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS21" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="61" t="inlineStr">
+      <c r="CS22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT22" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B22" s="62" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="61" t="inlineStr">
+      <c r="C23" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D22" s="61" t="inlineStr">
+      <c r="D23" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E22" s="63" t="n">
+      <c r="E23" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F22" s="64" t="inlineStr">
+      <c r="F23" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G22" s="64" t="inlineStr">
+      <c r="G23" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H22" s="65" t="inlineStr">
+      <c r="H23" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="66" t="n">
+      <c r="I23" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J22" s="67" t="n">
+      <c r="J23" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K22" s="66" t="n">
+      <c r="K23" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L22" s="68" t="n">
+      <c r="L23" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M22" s="68" t="n"/>
-      <c r="N22" s="69" t="n">
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O22" s="69" t="n">
+      <c r="O23" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q22" s="42" t="n">
+      <c r="Q23" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CR22" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS22" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="42" t="inlineStr">
+      <c r="CS23" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT23" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B24" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E24" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F23" s="42" t="inlineStr">
+      <c r="F24" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G23" s="42" t="inlineStr">
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H23" s="42" t="inlineStr">
+      <c r="H24" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="72" t="n">
+      <c r="I24" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J23" s="72" t="n">
+      <c r="J24" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K23" s="72" t="n">
+      <c r="K24" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L23" s="72" t="n">
+      <c r="L24" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M23" s="72" t="n"/>
-      <c r="N23" s="42" t="n">
+      <c r="M24" s="72" t="n"/>
+      <c r="N24" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O23" s="42" t="n">
+      <c r="O24" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CR23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS23" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="61" t="inlineStr">
+      <c r="CS24" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="B25" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="61" t="inlineStr">
+      <c r="C25" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D24" s="61" t="inlineStr">
+      <c r="D25" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E24" s="64" t="n">
+      <c r="E25" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F24" s="64" t="inlineStr">
+      <c r="F25" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G24" s="73" t="n">
+      <c r="G25" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H24" s="65" t="inlineStr">
+      <c r="H25" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="66" t="n">
+      <c r="I25" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J24" s="66" t="n">
+      <c r="J25" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K24" s="67" t="n">
+      <c r="K25" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L24" s="68" t="n">
+      <c r="L25" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="69" t="n">
+      <c r="M25" s="68" t="n"/>
+      <c r="N25" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O24" s="69" t="n"/>
-      <c r="CR24" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS24" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="75" t="inlineStr">
+      <c r="O25" s="69" t="n"/>
+      <c r="CS25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT25" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B25" s="76" t="inlineStr">
+      <c r="B26" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="75" t="inlineStr">
+      <c r="C26" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D25" s="75" t="inlineStr">
+      <c r="D26" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E25" s="77" t="n">
+      <c r="E26" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F25" s="78" t="inlineStr">
+      <c r="F26" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G25" s="79" t="n">
+      <c r="G26" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H25" s="80" t="inlineStr">
+      <c r="H26" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I25" s="81" t="n">
+      <c r="I26" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J25" s="81" t="n">
+      <c r="J26" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K25" s="82" t="inlineStr">
+      <c r="K26" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L25" s="83" t="inlineStr">
+      <c r="L26" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M25" s="83" t="n"/>
-      <c r="N25" s="84" t="n"/>
-      <c r="O25" s="69" t="n"/>
-      <c r="CR25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS25" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43">
-      <c r="A26" s="42" t="inlineStr">
+      <c r="M26" s="83" t="n"/>
+      <c r="N26" s="84" t="n"/>
+      <c r="O26" s="69" t="n"/>
+      <c r="CS26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT26" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="43">
+      <c r="A27" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C27" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D26" s="42" t="inlineStr">
+      <c r="D27" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E26" s="42" t="n">
+      <c r="E27" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F26" s="42" t="inlineStr">
+      <c r="F27" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G26" s="47" t="n">
+      <c r="G27" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H26" s="42" t="inlineStr">
+      <c r="H27" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I26" s="72" t="n">
+      <c r="I27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J26" s="72" t="n">
+      <c r="J27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K26" s="72" t="n">
+      <c r="K27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L26" s="72" t="n">
+      <c r="L27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CR26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CS26" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="43"/>
+      <c r="CS27" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CT27" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="28" ht="15.75" customHeight="1" s="43"/>
     <row r="29"/>
     <row r="30"/>
@@ -2573,29 +2619,30 @@
     <row r="32"/>
     <row r="33"/>
     <row r="34" ht="15.75" customHeight="1" s="43"/>
-    <row r="35" ht="15.75" customHeight="1" s="43">
-      <c r="A35" s="42" t="n"/>
-    </row>
-    <row r="36" ht="15.75" customHeight="1" s="43"/>
+    <row r="35" ht="15.75" customHeight="1" s="43"/>
+    <row r="36" ht="15.75" customHeight="1" s="43">
+      <c r="A36" s="42" t="n"/>
+    </row>
     <row r="37"/>
-    <row r="38" ht="15.75" customHeight="1" s="43">
-      <c r="A38" s="42" t="n"/>
-    </row>
+    <row r="38" ht="15.75" customHeight="1" s="43"/>
     <row r="39" ht="15.75" customHeight="1" s="43">
       <c r="A39" s="42" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="43">
       <c r="A40" s="42" t="n"/>
     </row>
-    <row r="41"/>
-    <row r="42">
-      <c r="A42" s="42" t="n"/>
-    </row>
+    <row r="41">
+      <c r="A41" s="42" t="n"/>
+    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="42" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="42" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-21
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CT45"/>
+  <dimension ref="A1:CU45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1017,14 +1017,17 @@
         <v>46281.73324260417</v>
       </c>
       <c r="CR1" s="56" t="n">
-        <v>46285.69801302979</v>
-      </c>
-      <c r="CS1" s="44" t="inlineStr">
+        <v>46285.69801303241</v>
+      </c>
+      <c r="CS1" s="56" t="n">
+        <v>46286.77502968439</v>
+      </c>
+      <c r="CT1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CT1" s="44" t="inlineStr">
+      <c r="CU1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1078,12 +1081,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CS2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT2" s="58" t="inlineStr">
+      <c r="CT2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1137,12 +1140,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CS3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT3" s="58" t="inlineStr">
+      <c r="CT3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1197,12 +1200,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CS4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1285,15 +1288,15 @@
       <c r="CQ5" s="42" t="n">
         <v>2334.35</v>
       </c>
-      <c r="CR5" t="n">
+      <c r="CR5" s="42" t="n">
         <v>2239.35</v>
       </c>
-      <c r="CS5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1353,12 +1356,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CS6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1413,12 +1416,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CS7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1499,12 +1502,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CS8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1552,12 +1555,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CS9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1605,12 +1608,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CS10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1662,12 +1665,12 @@
       <c r="CQ11" s="42" t="n">
         <v>2581.35</v>
       </c>
-      <c r="CS11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1699,6 +1702,11 @@
           <t>Sep 14</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="BK12" s="42" t="n">
         <v>2064.06</v>
       </c>
@@ -1714,7 +1722,7 @@
       <c r="CQ12" s="42" t="n">
         <v>1985.35</v>
       </c>
-      <c r="CR12" t="n">
+      <c r="CR12" s="42" t="n">
         <v>1986.35</v>
       </c>
     </row>
@@ -1809,7 +1817,7 @@
       <c r="CQ14" s="42" t="n">
         <v>3584.35</v>
       </c>
-      <c r="CR14" t="n">
+      <c r="CR14" s="42" t="n">
         <v>3519.35</v>
       </c>
     </row>
@@ -1857,37 +1865,37 @@
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="43">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>#8-460C</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>1 bath</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>732</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="42" t="inlineStr">
         <is>
           <t>S11</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="42" t="inlineStr">
         <is>
           <t>Oct 13</t>
         </is>
       </c>
-      <c r="CR16" t="n">
+      <c r="CR16" s="42" t="n">
         <v>2158.35</v>
       </c>
     </row>
@@ -1908,8 +1916,8 @@
       <c r="AJ17" s="42" t="n"/>
       <c r="AN17" s="42" t="n"/>
       <c r="AP17" s="42" t="n"/>
-      <c r="CS17" s="42" t="n"/>
       <c r="CT17" s="42" t="n"/>
+      <c r="CU17" s="42" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -1965,12 +1973,12 @@
       <c r="AJ18" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CS18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT18" s="58" t="inlineStr">
+      <c r="CT18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2024,12 +2032,12 @@
       <c r="AI19" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CS19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CT19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU19" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2116,12 +2124,12 @@
       <c r="AC20" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CS20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT20" s="58" t="inlineStr">
+      <c r="CT20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2200,12 +2208,12 @@
       <c r="W21" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CS21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT21" s="58" t="inlineStr">
+      <c r="CT21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2268,12 +2276,12 @@
       <c r="W22" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CS22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT22" s="58" t="inlineStr">
+      <c r="CT22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2340,12 +2348,12 @@
       <c r="Q23" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CS23" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT23" s="71" t="inlineStr">
+      <c r="CT23" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2409,12 +2417,12 @@
       <c r="O24" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CS24" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT24" s="58" t="inlineStr">
+      <c r="CT24" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2474,12 +2482,12 @@
         <v>1964.85</v>
       </c>
       <c r="O25" s="69" t="n"/>
-      <c r="CS25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT25" s="71" t="inlineStr">
+      <c r="CT25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2541,12 +2549,12 @@
       <c r="M26" s="83" t="n"/>
       <c r="N26" s="84" t="n"/>
       <c r="O26" s="69" t="n"/>
-      <c r="CS26" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT26" s="71" t="inlineStr">
+      <c r="CT26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU26" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2601,12 +2609,12 @@
       <c r="L27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CS27" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CT27" s="58" t="inlineStr">
+      <c r="CT27" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CU27" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-22
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CU45"/>
+  <dimension ref="A1:CV45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1020,14 +1020,17 @@
         <v>46285.69801303241</v>
       </c>
       <c r="CS1" s="56" t="n">
-        <v>46286.77502968439</v>
-      </c>
-      <c r="CT1" s="44" t="inlineStr">
+        <v>46286.7750296875</v>
+      </c>
+      <c r="CT1" s="56" t="n">
+        <v>46287.73372728883</v>
+      </c>
+      <c r="CU1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CU1" s="44" t="inlineStr">
+      <c r="CV1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1081,12 +1084,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CT2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU2" s="58" t="inlineStr">
+      <c r="CU2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1140,12 +1143,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CT3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU3" s="58" t="inlineStr">
+      <c r="CU3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1200,12 +1203,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CT4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1291,12 +1294,15 @@
       <c r="CR5" s="42" t="n">
         <v>2239.35</v>
       </c>
-      <c r="CT5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CT5" t="n">
+        <v>2221.35</v>
       </c>
       <c r="CU5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1356,12 +1362,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CT6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1416,12 +1422,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CT7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1502,12 +1508,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CT8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1555,12 +1561,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CT9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1608,12 +1614,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CT10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1665,12 +1671,15 @@
       <c r="CQ11" s="42" t="n">
         <v>2581.35</v>
       </c>
-      <c r="CT11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CT11" t="n">
+        <v>2558.35</v>
       </c>
       <c r="CU11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1702,7 +1711,7 @@
           <t>Sep 14</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1820,6 +1829,9 @@
       <c r="CR14" s="42" t="n">
         <v>3519.35</v>
       </c>
+      <c r="CT14" t="n">
+        <v>3487.35</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
@@ -1897,6 +1909,9 @@
       </c>
       <c r="CR16" s="42" t="n">
         <v>2158.35</v>
+      </c>
+      <c r="CT16" t="n">
+        <v>2139.35</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
@@ -1916,8 +1931,8 @@
       <c r="AJ17" s="42" t="n"/>
       <c r="AN17" s="42" t="n"/>
       <c r="AP17" s="42" t="n"/>
-      <c r="CT17" s="42" t="n"/>
       <c r="CU17" s="42" t="n"/>
+      <c r="CV17" s="42" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -1973,12 +1988,12 @@
       <c r="AJ18" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CT18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU18" s="58" t="inlineStr">
+      <c r="CU18" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV18" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2032,12 +2047,12 @@
       <c r="AI19" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CT19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CU19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV19" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2124,12 +2139,12 @@
       <c r="AC20" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CT20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU20" s="58" t="inlineStr">
+      <c r="CU20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2208,12 +2223,12 @@
       <c r="W21" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CT21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU21" s="58" t="inlineStr">
+      <c r="CU21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2276,12 +2291,12 @@
       <c r="W22" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CT22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU22" s="58" t="inlineStr">
+      <c r="CU22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2348,12 +2363,12 @@
       <c r="Q23" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CT23" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU23" s="71" t="inlineStr">
+      <c r="CU23" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV23" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2417,12 +2432,12 @@
       <c r="O24" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CT24" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU24" s="58" t="inlineStr">
+      <c r="CU24" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2482,12 +2497,12 @@
         <v>1964.85</v>
       </c>
       <c r="O25" s="69" t="n"/>
-      <c r="CT25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU25" s="71" t="inlineStr">
+      <c r="CU25" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2549,12 +2564,12 @@
       <c r="M26" s="83" t="n"/>
       <c r="N26" s="84" t="n"/>
       <c r="O26" s="69" t="n"/>
-      <c r="CT26" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU26" s="71" t="inlineStr">
+      <c r="CU26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV26" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2609,12 +2624,12 @@
       <c r="L27" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CT27" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CU27" s="58" t="inlineStr">
+      <c r="CU27" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CV27" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-23
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CV45"/>
+  <dimension ref="A1:CW46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1023,14 +1023,17 @@
         <v>46286.7750296875</v>
       </c>
       <c r="CT1" s="56" t="n">
-        <v>46287.73372728883</v>
-      </c>
-      <c r="CU1" s="44" t="inlineStr">
+        <v>46287.73372729167</v>
+      </c>
+      <c r="CU1" s="56" t="n">
+        <v>46288.74192784238</v>
+      </c>
+      <c r="CV1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CV1" s="44" t="inlineStr">
+      <c r="CW1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1084,12 +1087,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CU2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV2" s="58" t="inlineStr">
+      <c r="CV2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1143,12 +1146,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CU3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV3" s="58" t="inlineStr">
+      <c r="CV3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1203,12 +1206,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CU4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1294,15 +1297,15 @@
       <c r="CR5" s="42" t="n">
         <v>2239.35</v>
       </c>
-      <c r="CT5" t="n">
+      <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CU5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1362,12 +1365,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CU6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1422,12 +1425,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CU7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1508,12 +1511,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CU8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1561,12 +1564,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CU9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1614,12 +1617,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CU10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1671,15 +1674,15 @@
       <c r="CQ11" s="42" t="n">
         <v>2581.35</v>
       </c>
-      <c r="CT11" t="n">
+      <c r="CT11" s="42" t="n">
         <v>2558.35</v>
       </c>
-      <c r="CU11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CV11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1829,8 +1832,11 @@
       <c r="CR14" s="42" t="n">
         <v>3519.35</v>
       </c>
-      <c r="CT14" t="n">
+      <c r="CT14" s="42" t="n">
         <v>3487.35</v>
+      </c>
+      <c r="CU14" t="n">
+        <v>3564.35</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
@@ -1910,99 +1916,69 @@
       <c r="CR16" s="42" t="n">
         <v>2158.35</v>
       </c>
-      <c r="CT16" t="n">
+      <c r="CT16" s="42" t="n">
         <v>2139.35</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n"/>
-      <c r="C17" s="42" t="n"/>
-      <c r="D17" s="42" t="n"/>
-      <c r="E17" s="42" t="n"/>
-      <c r="F17" s="42" t="n"/>
-      <c r="G17" s="42" t="n"/>
-      <c r="H17" s="42" t="n"/>
-      <c r="AH17" s="42" t="n"/>
-      <c r="AJ17" s="42" t="n"/>
-      <c r="AN17" s="42" t="n"/>
-      <c r="AP17" s="42" t="n"/>
-      <c r="CU17" s="42" t="n"/>
-      <c r="CV17" s="42" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>#4-461</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1 bath</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Sep 24</t>
+        </is>
+      </c>
+      <c r="CU17" t="n">
+        <v>1967.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B18" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C18" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E18" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F18" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G18" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H18" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z18" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB18" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE18" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG18" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ18" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CU18" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV18" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n"/>
+      <c r="C18" s="42" t="n"/>
+      <c r="D18" s="42" t="n"/>
+      <c r="E18" s="42" t="n"/>
+      <c r="F18" s="42" t="n"/>
+      <c r="G18" s="42" t="n"/>
+      <c r="H18" s="42" t="n"/>
+      <c r="AH18" s="42" t="n"/>
+      <c r="AJ18" s="42" t="n"/>
+      <c r="AN18" s="42" t="n"/>
+      <c r="AP18" s="42" t="n"/>
+      <c r="CV18" s="42" t="n"/>
+      <c r="CW18" s="42" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B19" s="42" t="inlineStr">
@@ -2012,25 +1988,25 @@
       </c>
       <c r="C19" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E19" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F19" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G19" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H19" s="42" t="inlineStr">
@@ -2038,21 +2014,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF19" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z19" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB19" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE19" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG19" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI19" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CU19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ19" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CV19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2061,581 +2043,639 @@
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F20" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H20" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF20" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG20" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI20" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CV20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="43">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D20" s="42" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E21" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F20" s="42" t="inlineStr">
+      <c r="F21" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G20" s="42" t="inlineStr">
+      <c r="G21" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H20" s="42" t="inlineStr">
+      <c r="H21" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I20" s="42" t="n">
+      <c r="I21" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J20" s="42" t="n">
+      <c r="J21" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K20" s="42" t="n">
+      <c r="K21" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L20" s="42" t="n">
+      <c r="L21" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N20" s="42" t="n">
+      <c r="N21" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O20" s="42" t="n">
+      <c r="O21" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q20" s="42" t="n">
+      <c r="Q21" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T20" s="42" t="n">
+      <c r="T21" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U20" s="42" t="n">
+      <c r="U21" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V20" s="42" t="n">
+      <c r="V21" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W20" s="42" t="n">
+      <c r="W21" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA20" s="42" t="n">
+      <c r="AA21" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB20" s="42" t="n">
+      <c r="AB21" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC20" s="42" t="n">
+      <c r="AC21" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CU20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV20" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="43">
-      <c r="A21" s="61" t="inlineStr">
+      <c r="CV21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW21" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="B22" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="61" t="inlineStr">
+      <c r="C22" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D21" s="61" t="inlineStr">
+      <c r="D22" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E21" s="63" t="n">
+      <c r="E22" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F21" s="64" t="inlineStr">
+      <c r="F22" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G21" s="64" t="inlineStr">
+      <c r="G22" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H21" s="65" t="inlineStr">
+      <c r="H22" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="66" t="n">
+      <c r="I22" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J21" s="67" t="n">
+      <c r="J22" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K21" s="66" t="n">
+      <c r="K22" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L21" s="68" t="n">
+      <c r="L22" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M21" s="68" t="n"/>
-      <c r="N21" s="69" t="n">
+      <c r="M22" s="68" t="n"/>
+      <c r="N22" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O21" s="69" t="n">
+      <c r="O22" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q21" s="42" t="n">
+      <c r="Q22" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T21" s="42" t="n">
+      <c r="T22" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U21" s="42" t="n">
+      <c r="U22" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V21" s="42" t="n">
+      <c r="V22" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W21" s="42" t="n">
+      <c r="W22" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CU21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV21" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="42" t="inlineStr">
+      <c r="CV22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW22" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E23" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F22" s="42" t="inlineStr">
+      <c r="F23" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G22" s="42" t="inlineStr">
+      <c r="G23" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H22" s="42" t="inlineStr">
+      <c r="H23" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="42" t="n">
+      <c r="I23" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M22" s="42" t="n">
+      <c r="M23" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N22" s="42" t="n">
+      <c r="N23" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q22" s="42" t="n">
+      <c r="Q23" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V22" s="42" t="n">
+      <c r="V23" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W22" s="42" t="n">
+      <c r="W23" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CU22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV22" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="CV23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B24" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="61" t="inlineStr">
+      <c r="C24" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D23" s="61" t="inlineStr">
+      <c r="D24" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E23" s="63" t="n">
+      <c r="E24" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F23" s="64" t="inlineStr">
+      <c r="F24" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G23" s="64" t="inlineStr">
+      <c r="G24" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H23" s="65" t="inlineStr">
+      <c r="H24" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="66" t="n">
+      <c r="I24" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J23" s="67" t="n">
+      <c r="J24" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K23" s="66" t="n">
+      <c r="K24" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L23" s="68" t="n">
+      <c r="L24" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M23" s="68" t="n"/>
-      <c r="N23" s="69" t="n">
+      <c r="M24" s="68" t="n"/>
+      <c r="N24" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O23" s="69" t="n">
+      <c r="O24" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q23" s="42" t="n">
+      <c r="Q24" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CU23" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV23" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="CV24" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW24" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B25" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="42" t="inlineStr">
+      <c r="C25" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D24" s="42" t="inlineStr">
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E25" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F24" s="42" t="inlineStr">
+      <c r="F25" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G24" s="42" t="inlineStr">
+      <c r="G25" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H24" s="42" t="inlineStr">
+      <c r="H25" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="72" t="n">
+      <c r="I25" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J24" s="72" t="n">
+      <c r="J25" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K24" s="72" t="n">
+      <c r="K25" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L24" s="72" t="n">
+      <c r="L25" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M24" s="72" t="n"/>
-      <c r="N24" s="42" t="n">
+      <c r="M25" s="72" t="n"/>
+      <c r="N25" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O24" s="42" t="n">
+      <c r="O25" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CU24" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV24" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="61" t="inlineStr">
+      <c r="CV25" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW25" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="B26" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="61" t="inlineStr">
+      <c r="C26" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D25" s="61" t="inlineStr">
+      <c r="D26" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E25" s="64" t="n">
+      <c r="E26" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F25" s="64" t="inlineStr">
+      <c r="F26" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G25" s="73" t="n">
+      <c r="G26" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H25" s="65" t="inlineStr">
+      <c r="H26" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I25" s="66" t="n">
+      <c r="I26" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J25" s="66" t="n">
+      <c r="J26" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K25" s="67" t="n">
+      <c r="K26" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L25" s="68" t="n">
+      <c r="L26" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M25" s="68" t="n"/>
-      <c r="N25" s="69" t="n">
+      <c r="M26" s="68" t="n"/>
+      <c r="N26" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O25" s="69" t="n"/>
-      <c r="CU25" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV25" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43">
-      <c r="A26" s="75" t="inlineStr">
+      <c r="O26" s="69" t="n"/>
+      <c r="CV26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW26" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="43">
+      <c r="A27" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B26" s="76" t="inlineStr">
+      <c r="B27" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C26" s="75" t="inlineStr">
+      <c r="C27" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D26" s="75" t="inlineStr">
+      <c r="D27" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E26" s="77" t="n">
+      <c r="E27" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F26" s="78" t="inlineStr">
+      <c r="F27" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G26" s="79" t="n">
+      <c r="G27" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H26" s="80" t="inlineStr">
+      <c r="H27" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I26" s="81" t="n">
+      <c r="I27" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J26" s="81" t="n">
+      <c r="J27" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K26" s="82" t="inlineStr">
+      <c r="K27" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L26" s="83" t="inlineStr">
+      <c r="L27" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M26" s="83" t="n"/>
-      <c r="N26" s="84" t="n"/>
-      <c r="O26" s="69" t="n"/>
-      <c r="CU26" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV26" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="43">
-      <c r="A27" s="42" t="inlineStr">
+      <c r="M27" s="83" t="n"/>
+      <c r="N27" s="84" t="n"/>
+      <c r="O27" s="69" t="n"/>
+      <c r="CV27" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW27" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="43">
+      <c r="A28" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B28" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D27" s="42" t="inlineStr">
+      <c r="D28" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E27" s="42" t="n">
+      <c r="E28" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F27" s="42" t="inlineStr">
+      <c r="F28" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G27" s="47" t="n">
+      <c r="G28" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H27" s="42" t="inlineStr">
+      <c r="H28" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I27" s="72" t="n">
+      <c r="I28" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J27" s="72" t="n">
+      <c r="J28" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K27" s="72" t="n">
+      <c r="K28" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L27" s="72" t="n">
+      <c r="L28" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CU27" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CV27" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="43"/>
+      <c r="CV28" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CW28" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="29"/>
     <row r="30"/>
     <row r="31" ht="15.75" customHeight="1" s="43"/>
@@ -2643,29 +2683,30 @@
     <row r="33"/>
     <row r="34" ht="15.75" customHeight="1" s="43"/>
     <row r="35" ht="15.75" customHeight="1" s="43"/>
-    <row r="36" ht="15.75" customHeight="1" s="43">
-      <c r="A36" s="42" t="n"/>
-    </row>
-    <row r="37"/>
+    <row r="36" ht="15.75" customHeight="1" s="43"/>
+    <row r="37">
+      <c r="A37" s="42" t="n"/>
+    </row>
     <row r="38" ht="15.75" customHeight="1" s="43"/>
-    <row r="39" ht="15.75" customHeight="1" s="43">
-      <c r="A39" s="42" t="n"/>
-    </row>
+    <row r="39" ht="15.75" customHeight="1" s="43"/>
     <row r="40" ht="15.75" customHeight="1" s="43">
       <c r="A40" s="42" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="42" t="n"/>
     </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="42" t="n"/>
-    </row>
+    <row r="42">
+      <c r="A42" s="42" t="n"/>
+    </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="42" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="42" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-24
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CW46"/>
+  <dimension ref="A1:CX46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1026,14 +1026,17 @@
         <v>46287.73372729167</v>
       </c>
       <c r="CU1" s="56" t="n">
-        <v>46288.74192784238</v>
-      </c>
-      <c r="CV1" s="44" t="inlineStr">
+        <v>46288.74192784722</v>
+      </c>
+      <c r="CV1" s="56" t="n">
+        <v>46289.74303366279</v>
+      </c>
+      <c r="CW1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CW1" s="44" t="inlineStr">
+      <c r="CX1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1087,12 +1090,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CV2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW2" s="58" t="inlineStr">
+      <c r="CW2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1146,12 +1149,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CV3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW3" s="58" t="inlineStr">
+      <c r="CW3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1206,12 +1209,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CV4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1300,12 +1303,12 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CV5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1365,12 +1368,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CV6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1425,12 +1428,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CV7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1511,12 +1514,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CV8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1564,12 +1567,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CV9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1617,12 +1620,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CV10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1677,12 +1680,12 @@
       <c r="CT11" s="42" t="n">
         <v>2558.35</v>
       </c>
-      <c r="CV11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1835,7 +1838,7 @@
       <c r="CT14" s="42" t="n">
         <v>3487.35</v>
       </c>
-      <c r="CU14" t="n">
+      <c r="CU14" s="42" t="n">
         <v>3564.35</v>
       </c>
     </row>
@@ -1921,37 +1924,42 @@
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>#4-461</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>1 bath</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="42" t="inlineStr">
         <is>
           <t>605</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="42" t="inlineStr">
         <is>
           <t>Sep 24</t>
         </is>
       </c>
-      <c r="CU17" t="n">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="CU17" s="42" t="n">
         <v>1967.35</v>
       </c>
     </row>
@@ -1972,8 +1980,8 @@
       <c r="AJ18" s="42" t="n"/>
       <c r="AN18" s="42" t="n"/>
       <c r="AP18" s="42" t="n"/>
-      <c r="CV18" s="42" t="n"/>
       <c r="CW18" s="42" t="n"/>
+      <c r="CX18" s="42" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
@@ -2029,12 +2037,12 @@
       <c r="AJ19" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CV19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW19" s="58" t="inlineStr">
+      <c r="CW19" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX19" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2088,12 +2096,12 @@
       <c r="AI20" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CV20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CW20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX20" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2180,12 +2188,12 @@
       <c r="AC21" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CV21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW21" s="58" t="inlineStr">
+      <c r="CW21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2264,12 +2272,12 @@
       <c r="W22" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CV22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW22" s="58" t="inlineStr">
+      <c r="CW22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2332,12 +2340,12 @@
       <c r="W23" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CV23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW23" s="58" t="inlineStr">
+      <c r="CW23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2404,12 +2412,12 @@
       <c r="Q24" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CV24" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW24" s="71" t="inlineStr">
+      <c r="CW24" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX24" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2473,12 +2481,12 @@
       <c r="O25" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CV25" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW25" s="58" t="inlineStr">
+      <c r="CW25" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2538,12 +2546,12 @@
         <v>1964.85</v>
       </c>
       <c r="O26" s="69" t="n"/>
-      <c r="CV26" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW26" s="71" t="inlineStr">
+      <c r="CW26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX26" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2605,12 +2613,12 @@
       <c r="M27" s="83" t="n"/>
       <c r="N27" s="84" t="n"/>
       <c r="O27" s="69" t="n"/>
-      <c r="CV27" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW27" s="71" t="inlineStr">
+      <c r="CW27" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2665,12 +2673,12 @@
       <c r="L28" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CV28" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CW28" s="58" t="inlineStr">
+      <c r="CW28" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CX28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-25
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CX46"/>
+  <dimension ref="A1:CY47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1029,14 +1029,17 @@
         <v>46288.74192784722</v>
       </c>
       <c r="CV1" s="56" t="n">
-        <v>46289.74303366279</v>
-      </c>
-      <c r="CW1" s="44" t="inlineStr">
+        <v>46289.74303365741</v>
+      </c>
+      <c r="CW1" s="56" t="n">
+        <v>46290.74600479449</v>
+      </c>
+      <c r="CX1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CX1" s="44" t="inlineStr">
+      <c r="CY1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1090,12 +1093,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CW2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX2" s="58" t="inlineStr">
+      <c r="CX2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1149,12 +1152,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CW3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX3" s="58" t="inlineStr">
+      <c r="CX3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1209,12 +1212,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CW4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1303,12 +1306,12 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CW5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1368,12 +1371,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CW6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1428,12 +1431,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CW7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1514,12 +1517,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CW8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1567,12 +1570,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CW9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1620,12 +1623,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CW10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CX10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1680,12 +1683,15 @@
       <c r="CT11" s="42" t="n">
         <v>2558.35</v>
       </c>
-      <c r="CW11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CW11" t="n">
+        <v>2535.35</v>
       </c>
       <c r="CX11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1841,6 +1847,9 @@
       <c r="CU14" s="42" t="n">
         <v>3564.35</v>
       </c>
+      <c r="CW14" t="n">
+        <v>3532.35</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="43">
       <c r="A15" s="42" t="inlineStr">
@@ -1954,7 +1963,7 @@
           <t>Sep 24</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1964,94 +1973,64 @@
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
-      <c r="A18" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B18" s="42" t="n"/>
-      <c r="C18" s="42" t="n"/>
-      <c r="D18" s="42" t="n"/>
-      <c r="E18" s="42" t="n"/>
-      <c r="F18" s="42" t="n"/>
-      <c r="G18" s="42" t="n"/>
-      <c r="H18" s="42" t="n"/>
-      <c r="AH18" s="42" t="n"/>
-      <c r="AJ18" s="42" t="n"/>
-      <c r="AN18" s="42" t="n"/>
-      <c r="AP18" s="42" t="n"/>
-      <c r="CW18" s="42" t="n"/>
-      <c r="CX18" s="42" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>#9-478C</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>955</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Nov 21</t>
+        </is>
+      </c>
+      <c r="CW18" t="n">
+        <v>3205.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C19" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E19" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F19" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G19" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H19" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z19" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB19" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE19" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG19" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ19" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CW19" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX19" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="n"/>
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="42" t="n"/>
+      <c r="E19" s="42" t="n"/>
+      <c r="F19" s="42" t="n"/>
+      <c r="G19" s="42" t="n"/>
+      <c r="H19" s="42" t="n"/>
+      <c r="AH19" s="42" t="n"/>
+      <c r="AJ19" s="42" t="n"/>
+      <c r="AN19" s="42" t="n"/>
+      <c r="AP19" s="42" t="n"/>
+      <c r="CX19" s="42" t="n"/>
+      <c r="CY19" s="42" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B20" s="42" t="inlineStr">
@@ -2061,25 +2040,25 @@
       </c>
       <c r="C20" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D20" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E20" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F20" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G20" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H20" s="42" t="inlineStr">
@@ -2087,21 +2066,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF20" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z20" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB20" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE20" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG20" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI20" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CW20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ20" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CX20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2110,581 +2095,639 @@
     <row r="21" ht="15.75" customHeight="1" s="43">
       <c r="A21" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E21" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F21" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H21" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF21" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG21" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI21" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CX21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="43">
+      <c r="A22" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E21" s="42" t="n">
+      <c r="E22" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F21" s="42" t="inlineStr">
+      <c r="F22" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="G22" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H21" s="42" t="inlineStr">
+      <c r="H22" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I21" s="42" t="n">
+      <c r="I22" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J21" s="42" t="n">
+      <c r="J22" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K21" s="42" t="n">
+      <c r="K22" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L21" s="42" t="n">
+      <c r="L22" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N21" s="42" t="n">
+      <c r="N22" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O21" s="42" t="n">
+      <c r="O22" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q21" s="42" t="n">
+      <c r="Q22" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T21" s="42" t="n">
+      <c r="T22" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U21" s="42" t="n">
+      <c r="U22" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V21" s="42" t="n">
+      <c r="V22" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W21" s="42" t="n">
+      <c r="W22" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA21" s="42" t="n">
+      <c r="AA22" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB21" s="42" t="n">
+      <c r="AB22" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC21" s="42" t="n">
+      <c r="AC22" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CW21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX21" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="43">
-      <c r="A22" s="61" t="inlineStr">
+      <c r="CX22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY22" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B22" s="62" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="61" t="inlineStr">
+      <c r="C23" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D22" s="61" t="inlineStr">
+      <c r="D23" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="63" t="n">
+      <c r="E23" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F22" s="64" t="inlineStr">
+      <c r="F23" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G22" s="64" t="inlineStr">
+      <c r="G23" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H22" s="65" t="inlineStr">
+      <c r="H23" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="66" t="n">
+      <c r="I23" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J22" s="67" t="n">
+      <c r="J23" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K22" s="66" t="n">
+      <c r="K23" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L22" s="68" t="n">
+      <c r="L23" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M22" s="68" t="n"/>
-      <c r="N22" s="69" t="n">
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O22" s="69" t="n">
+      <c r="O23" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q22" s="42" t="n">
+      <c r="Q23" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T22" s="42" t="n">
+      <c r="T23" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U22" s="42" t="n">
+      <c r="U23" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V22" s="42" t="n">
+      <c r="V23" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W22" s="42" t="n">
+      <c r="W23" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CW22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX22" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="42" t="inlineStr">
+      <c r="CX23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B24" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E24" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F23" s="42" t="inlineStr">
+      <c r="F24" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G23" s="42" t="inlineStr">
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H23" s="42" t="inlineStr">
+      <c r="H24" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="42" t="n">
+      <c r="I24" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M23" s="42" t="n">
+      <c r="M24" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N23" s="42" t="n">
+      <c r="N24" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q23" s="42" t="n">
+      <c r="Q24" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V23" s="42" t="n">
+      <c r="V24" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W23" s="42" t="n">
+      <c r="W24" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CW23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX23" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="61" t="inlineStr">
+      <c r="CX24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="B25" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="61" t="inlineStr">
+      <c r="C25" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D24" s="61" t="inlineStr">
+      <c r="D25" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E24" s="63" t="n">
+      <c r="E25" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F24" s="64" t="inlineStr">
+      <c r="F25" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G24" s="64" t="inlineStr">
+      <c r="G25" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H24" s="65" t="inlineStr">
+      <c r="H25" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="66" t="n">
+      <c r="I25" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J24" s="67" t="n">
+      <c r="J25" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K24" s="66" t="n">
+      <c r="K25" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L24" s="68" t="n">
+      <c r="L25" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="69" t="n">
+      <c r="M25" s="68" t="n"/>
+      <c r="N25" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O24" s="69" t="n">
+      <c r="O25" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q24" s="42" t="n">
+      <c r="Q25" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CW24" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX24" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="42" t="inlineStr">
+      <c r="CX25" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY25" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C26" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D25" s="42" t="inlineStr">
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E25" s="42" t="n">
+      <c r="E26" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F25" s="42" t="inlineStr">
+      <c r="F26" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G25" s="42" t="inlineStr">
+      <c r="G26" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H25" s="42" t="inlineStr">
+      <c r="H26" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I25" s="72" t="n">
+      <c r="I26" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J25" s="72" t="n">
+      <c r="J26" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K25" s="72" t="n">
+      <c r="K26" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L25" s="72" t="n">
+      <c r="L26" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M25" s="72" t="n"/>
-      <c r="N25" s="42" t="n">
+      <c r="M26" s="72" t="n"/>
+      <c r="N26" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O25" s="42" t="n">
+      <c r="O26" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CW25" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX25" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43">
-      <c r="A26" s="61" t="inlineStr">
+      <c r="CX26" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY26" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="43">
+      <c r="A27" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B26" s="62" t="inlineStr">
+      <c r="B27" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C26" s="61" t="inlineStr">
+      <c r="C27" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D26" s="61" t="inlineStr">
+      <c r="D27" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E26" s="64" t="n">
+      <c r="E27" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F26" s="64" t="inlineStr">
+      <c r="F27" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G26" s="73" t="n">
+      <c r="G27" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H26" s="65" t="inlineStr">
+      <c r="H27" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I26" s="66" t="n">
+      <c r="I27" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J26" s="66" t="n">
+      <c r="J27" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K26" s="67" t="n">
+      <c r="K27" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L26" s="68" t="n">
+      <c r="L27" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M26" s="68" t="n"/>
-      <c r="N26" s="69" t="n">
+      <c r="M27" s="68" t="n"/>
+      <c r="N27" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O26" s="69" t="n"/>
-      <c r="CW26" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX26" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="43">
-      <c r="A27" s="75" t="inlineStr">
+      <c r="O27" s="69" t="n"/>
+      <c r="CX27" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY27" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="43">
+      <c r="A28" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B27" s="76" t="inlineStr">
+      <c r="B28" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C27" s="75" t="inlineStr">
+      <c r="C28" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D27" s="75" t="inlineStr">
+      <c r="D28" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E27" s="77" t="n">
+      <c r="E28" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F27" s="78" t="inlineStr">
+      <c r="F28" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G27" s="79" t="n">
+      <c r="G28" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H27" s="80" t="inlineStr">
+      <c r="H28" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I27" s="81" t="n">
+      <c r="I28" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J27" s="81" t="n">
+      <c r="J28" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K27" s="82" t="inlineStr">
+      <c r="K28" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L27" s="83" t="inlineStr">
+      <c r="L28" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M27" s="83" t="n"/>
-      <c r="N27" s="84" t="n"/>
-      <c r="O27" s="69" t="n"/>
-      <c r="CW27" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX27" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="43">
-      <c r="A28" s="42" t="inlineStr">
+      <c r="M28" s="83" t="n"/>
+      <c r="N28" s="84" t="n"/>
+      <c r="O28" s="69" t="n"/>
+      <c r="CX28" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY28" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B29" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C29" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D28" s="42" t="inlineStr">
+      <c r="D29" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E28" s="42" t="n">
+      <c r="E29" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F28" s="42" t="inlineStr">
+      <c r="F29" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G28" s="47" t="n">
+      <c r="G29" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H28" s="42" t="inlineStr">
+      <c r="H29" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I28" s="72" t="n">
+      <c r="I29" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J28" s="72" t="n">
+      <c r="J29" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K28" s="72" t="n">
+      <c r="K29" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L28" s="72" t="n">
+      <c r="L29" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CW28" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CX28" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
+      <c r="CX29" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CY29" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="30"/>
     <row r="31" ht="15.75" customHeight="1" s="43"/>
     <row r="32"/>
@@ -2692,29 +2735,30 @@
     <row r="34" ht="15.75" customHeight="1" s="43"/>
     <row r="35" ht="15.75" customHeight="1" s="43"/>
     <row r="36" ht="15.75" customHeight="1" s="43"/>
-    <row r="37">
-      <c r="A37" s="42" t="n"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" s="43"/>
+    <row r="37"/>
+    <row r="38" ht="15.75" customHeight="1" s="43">
+      <c r="A38" s="42" t="n"/>
+    </row>
     <row r="39" ht="15.75" customHeight="1" s="43"/>
-    <row r="40" ht="15.75" customHeight="1" s="43">
-      <c r="A40" s="42" t="n"/>
-    </row>
+    <row r="40" ht="15.75" customHeight="1" s="43"/>
     <row r="41">
       <c r="A41" s="42" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="42" t="n"/>
     </row>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" s="42" t="n"/>
-    </row>
+    <row r="43">
+      <c r="A43" s="42" t="n"/>
+    </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="42" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="42" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-26
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CY47"/>
+  <dimension ref="A1:CZ47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1032,14 +1032,17 @@
         <v>46289.74303365741</v>
       </c>
       <c r="CW1" s="56" t="n">
-        <v>46290.74600479449</v>
-      </c>
-      <c r="CX1" s="44" t="inlineStr">
+        <v>46290.74600479167</v>
+      </c>
+      <c r="CX1" s="56" t="n">
+        <v>46291.70971938389</v>
+      </c>
+      <c r="CY1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CY1" s="44" t="inlineStr">
+      <c r="CZ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1093,12 +1096,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CX2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY2" s="58" t="inlineStr">
+      <c r="CY2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1152,12 +1155,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CX3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY3" s="58" t="inlineStr">
+      <c r="CY3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1212,12 +1215,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CX4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1306,12 +1309,12 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CX5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1371,12 +1374,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CX6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1431,12 +1434,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CX7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1517,12 +1520,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CX8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1570,12 +1573,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CX9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1623,12 +1626,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CX10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1683,15 +1686,15 @@
       <c r="CT11" s="42" t="n">
         <v>2558.35</v>
       </c>
-      <c r="CW11" t="n">
+      <c r="CW11" s="42" t="n">
         <v>2535.35</v>
       </c>
-      <c r="CX11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1847,7 +1850,7 @@
       <c r="CU14" s="42" t="n">
         <v>3564.35</v>
       </c>
-      <c r="CW14" t="n">
+      <c r="CW14" s="42" t="n">
         <v>3532.35</v>
       </c>
     </row>
@@ -1973,37 +1976,37 @@
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>#9-478C</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>955</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="42" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="42" t="inlineStr">
         <is>
           <t>Nov 21</t>
         </is>
       </c>
-      <c r="CW18" t="n">
+      <c r="CW18" s="42" t="n">
         <v>3205.35</v>
       </c>
     </row>
@@ -2024,8 +2027,8 @@
       <c r="AJ19" s="42" t="n"/>
       <c r="AN19" s="42" t="n"/>
       <c r="AP19" s="42" t="n"/>
-      <c r="CX19" s="42" t="n"/>
       <c r="CY19" s="42" t="n"/>
+      <c r="CZ19" s="42" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
@@ -2081,12 +2084,12 @@
       <c r="AJ20" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="CX20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY20" s="58" t="inlineStr">
+      <c r="CY20" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ20" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2140,12 +2143,12 @@
       <c r="AI21" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="CX21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CY21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ21" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2232,12 +2235,12 @@
       <c r="AC22" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CX22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY22" s="58" t="inlineStr">
+      <c r="CY22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2316,12 +2319,12 @@
       <c r="W23" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CX23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY23" s="58" t="inlineStr">
+      <c r="CY23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ23" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2384,12 +2387,12 @@
       <c r="W24" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CX24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY24" s="58" t="inlineStr">
+      <c r="CY24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2456,12 +2459,12 @@
       <c r="Q25" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CX25" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY25" s="71" t="inlineStr">
+      <c r="CY25" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ25" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2525,12 +2528,12 @@
       <c r="O26" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CX26" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY26" s="58" t="inlineStr">
+      <c r="CY26" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2590,12 +2593,12 @@
         <v>1964.85</v>
       </c>
       <c r="O27" s="69" t="n"/>
-      <c r="CX27" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY27" s="71" t="inlineStr">
+      <c r="CY27" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2657,12 +2660,12 @@
       <c r="M28" s="83" t="n"/>
       <c r="N28" s="84" t="n"/>
       <c r="O28" s="69" t="n"/>
-      <c r="CX28" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY28" s="71" t="inlineStr">
+      <c r="CY28" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ28" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2717,12 +2720,12 @@
       <c r="L29" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CX29" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CY29" s="58" t="inlineStr">
+      <c r="CY29" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CZ29" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-28
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CZ47"/>
+  <dimension ref="A1:DA48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1035,14 +1035,17 @@
         <v>46290.74600479167</v>
       </c>
       <c r="CX1" s="56" t="n">
-        <v>46291.70971938389</v>
-      </c>
-      <c r="CY1" s="44" t="inlineStr">
+        <v>46291.70971938658</v>
+      </c>
+      <c r="CY1" s="56" t="n">
+        <v>46293.83729743735</v>
+      </c>
+      <c r="CZ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="CZ1" s="44" t="inlineStr">
+      <c r="DA1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1096,12 +1099,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CY2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ2" s="58" t="inlineStr">
+      <c r="CZ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1155,12 +1158,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CY3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ3" s="58" t="inlineStr">
+      <c r="CZ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1215,12 +1218,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CY4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1309,12 +1312,12 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CY5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1374,12 +1377,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CY6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1434,12 +1437,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CY7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1520,12 +1523,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CY8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1573,12 +1576,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CY9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1626,12 +1629,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CY10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1689,12 +1692,12 @@
       <c r="CW11" s="42" t="n">
         <v>2535.35</v>
       </c>
-      <c r="CY11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="CZ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2011,94 +2014,64 @@
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="n"/>
-      <c r="C19" s="42" t="n"/>
-      <c r="D19" s="42" t="n"/>
-      <c r="E19" s="42" t="n"/>
-      <c r="F19" s="42" t="n"/>
-      <c r="G19" s="42" t="n"/>
-      <c r="H19" s="42" t="n"/>
-      <c r="AH19" s="42" t="n"/>
-      <c r="AJ19" s="42" t="n"/>
-      <c r="AN19" s="42" t="n"/>
-      <c r="AP19" s="42" t="n"/>
-      <c r="CY19" s="42" t="n"/>
-      <c r="CZ19" s="42" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>#8-452B</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>874</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Oct 02</t>
+        </is>
+      </c>
+      <c r="CY19" t="n">
+        <v>2631.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B20" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C20" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D20" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E20" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F20" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G20" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H20" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z20" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB20" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE20" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG20" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ20" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CY20" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ20" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="42" t="n"/>
+      <c r="E20" s="42" t="n"/>
+      <c r="F20" s="42" t="n"/>
+      <c r="G20" s="42" t="n"/>
+      <c r="H20" s="42" t="n"/>
+      <c r="AH20" s="42" t="n"/>
+      <c r="AJ20" s="42" t="n"/>
+      <c r="AN20" s="42" t="n"/>
+      <c r="AP20" s="42" t="n"/>
+      <c r="CZ20" s="42" t="n"/>
+      <c r="DA20" s="42" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B21" s="42" t="inlineStr">
@@ -2108,25 +2081,25 @@
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E21" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F21" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G21" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H21" s="42" t="inlineStr">
@@ -2134,21 +2107,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF21" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z21" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB21" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE21" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG21" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI21" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CY21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ21" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="CZ21" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA21" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2157,581 +2136,639 @@
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C22" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D22" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E22" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F22" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G22" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H22" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF22" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG22" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI22" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="CZ22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="43">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E23" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F22" s="42" t="inlineStr">
+      <c r="F23" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G22" s="42" t="inlineStr">
+      <c r="G23" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H22" s="42" t="inlineStr">
+      <c r="H23" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I22" s="42" t="n">
+      <c r="I23" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J22" s="42" t="n">
+      <c r="J23" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K22" s="42" t="n">
+      <c r="K23" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L22" s="42" t="n">
+      <c r="L23" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N22" s="42" t="n">
+      <c r="N23" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O22" s="42" t="n">
+      <c r="O23" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q22" s="42" t="n">
+      <c r="Q23" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T22" s="42" t="n">
+      <c r="T23" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U22" s="42" t="n">
+      <c r="U23" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V22" s="42" t="n">
+      <c r="V23" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W22" s="42" t="n">
+      <c r="W23" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA22" s="42" t="n">
+      <c r="AA23" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB22" s="42" t="n">
+      <c r="AB23" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC22" s="42" t="n">
+      <c r="AC23" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CY22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ22" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="43">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="CZ23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B24" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="61" t="inlineStr">
+      <c r="C24" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D23" s="61" t="inlineStr">
+      <c r="D24" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="63" t="n">
+      <c r="E24" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F23" s="64" t="inlineStr">
+      <c r="F24" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G23" s="64" t="inlineStr">
+      <c r="G24" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H23" s="65" t="inlineStr">
+      <c r="H24" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="66" t="n">
+      <c r="I24" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J23" s="67" t="n">
+      <c r="J24" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K23" s="66" t="n">
+      <c r="K24" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L23" s="68" t="n">
+      <c r="L24" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M23" s="68" t="n"/>
-      <c r="N23" s="69" t="n">
+      <c r="M24" s="68" t="n"/>
+      <c r="N24" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O23" s="69" t="n">
+      <c r="O24" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q23" s="42" t="n">
+      <c r="Q24" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T23" s="42" t="n">
+      <c r="T24" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U23" s="42" t="n">
+      <c r="U24" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V23" s="42" t="n">
+      <c r="V24" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W23" s="42" t="n">
+      <c r="W24" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CY23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ23" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="CZ24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B25" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="42" t="inlineStr">
+      <c r="C25" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D24" s="42" t="inlineStr">
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E25" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F24" s="42" t="inlineStr">
+      <c r="F25" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G24" s="42" t="inlineStr">
+      <c r="G25" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H24" s="42" t="inlineStr">
+      <c r="H25" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="42" t="n">
+      <c r="I25" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M24" s="42" t="n">
+      <c r="M25" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N24" s="42" t="n">
+      <c r="N25" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q24" s="42" t="n">
+      <c r="Q25" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V24" s="42" t="n">
+      <c r="V25" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W24" s="42" t="n">
+      <c r="W25" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CY24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ24" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="61" t="inlineStr">
+      <c r="CZ25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA25" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="B26" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="61" t="inlineStr">
+      <c r="C26" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D25" s="61" t="inlineStr">
+      <c r="D26" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E25" s="63" t="n">
+      <c r="E26" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F25" s="64" t="inlineStr">
+      <c r="F26" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G25" s="64" t="inlineStr">
+      <c r="G26" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H25" s="65" t="inlineStr">
+      <c r="H26" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I25" s="66" t="n">
+      <c r="I26" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J25" s="67" t="n">
+      <c r="J26" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K25" s="66" t="n">
+      <c r="K26" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L25" s="68" t="n">
+      <c r="L26" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M25" s="68" t="n"/>
-      <c r="N25" s="69" t="n">
+      <c r="M26" s="68" t="n"/>
+      <c r="N26" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O25" s="69" t="n">
+      <c r="O26" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q25" s="42" t="n">
+      <c r="Q26" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CY25" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ25" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43">
-      <c r="A26" s="42" t="inlineStr">
+      <c r="CZ26" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA26" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="43">
+      <c r="A27" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C27" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D26" s="42" t="inlineStr">
+      <c r="D27" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E26" s="42" t="n">
+      <c r="E27" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F26" s="42" t="inlineStr">
+      <c r="F27" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G26" s="42" t="inlineStr">
+      <c r="G27" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H26" s="42" t="inlineStr">
+      <c r="H27" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I26" s="72" t="n">
+      <c r="I27" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J26" s="72" t="n">
+      <c r="J27" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K26" s="72" t="n">
+      <c r="K27" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L26" s="72" t="n">
+      <c r="L27" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M26" s="72" t="n"/>
-      <c r="N26" s="42" t="n">
+      <c r="M27" s="72" t="n"/>
+      <c r="N27" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O26" s="42" t="n">
+      <c r="O27" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CY26" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ26" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="43">
-      <c r="A27" s="61" t="inlineStr">
+      <c r="CZ27" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA27" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="43">
+      <c r="A28" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B27" s="62" t="inlineStr">
+      <c r="B28" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C27" s="61" t="inlineStr">
+      <c r="C28" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D27" s="61" t="inlineStr">
+      <c r="D28" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E27" s="64" t="n">
+      <c r="E28" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F27" s="64" t="inlineStr">
+      <c r="F28" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G27" s="73" t="n">
+      <c r="G28" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H27" s="65" t="inlineStr">
+      <c r="H28" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I27" s="66" t="n">
+      <c r="I28" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J27" s="66" t="n">
+      <c r="J28" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K27" s="67" t="n">
+      <c r="K28" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L27" s="68" t="n">
+      <c r="L28" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M27" s="68" t="n"/>
-      <c r="N27" s="69" t="n">
+      <c r="M28" s="68" t="n"/>
+      <c r="N28" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O27" s="69" t="n"/>
-      <c r="CY27" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ27" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="43">
-      <c r="A28" s="75" t="inlineStr">
+      <c r="O28" s="69" t="n"/>
+      <c r="CZ28" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA28" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B28" s="76" t="inlineStr">
+      <c r="B29" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C28" s="75" t="inlineStr">
+      <c r="C29" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D28" s="75" t="inlineStr">
+      <c r="D29" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E28" s="77" t="n">
+      <c r="E29" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F28" s="78" t="inlineStr">
+      <c r="F29" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G28" s="79" t="n">
+      <c r="G29" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H28" s="80" t="inlineStr">
+      <c r="H29" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I28" s="81" t="n">
+      <c r="I29" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J28" s="81" t="n">
+      <c r="J29" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K28" s="82" t="inlineStr">
+      <c r="K29" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L28" s="83" t="inlineStr">
+      <c r="L29" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M28" s="83" t="n"/>
-      <c r="N28" s="84" t="n"/>
-      <c r="O28" s="69" t="n"/>
-      <c r="CY28" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ28" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="42" t="inlineStr">
+      <c r="M29" s="83" t="n"/>
+      <c r="N29" s="84" t="n"/>
+      <c r="O29" s="69" t="n"/>
+      <c r="CZ29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA29" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B30" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C30" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D29" s="42" t="inlineStr">
+      <c r="D30" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E29" s="42" t="n">
+      <c r="E30" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F29" s="42" t="inlineStr">
+      <c r="F30" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G29" s="47" t="n">
+      <c r="G30" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H29" s="42" t="inlineStr">
+      <c r="H30" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I29" s="72" t="n">
+      <c r="I30" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J29" s="72" t="n">
+      <c r="J30" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K29" s="72" t="n">
+      <c r="K30" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L29" s="72" t="n">
+      <c r="L30" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CY29" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="CZ29" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
+      <c r="CZ30" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DA30" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="31" ht="15.75" customHeight="1" s="43"/>
     <row r="32"/>
     <row r="33"/>
@@ -2739,29 +2776,30 @@
     <row r="35" ht="15.75" customHeight="1" s="43"/>
     <row r="36" ht="15.75" customHeight="1" s="43"/>
     <row r="37"/>
-    <row r="38" ht="15.75" customHeight="1" s="43">
-      <c r="A38" s="42" t="n"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1" s="43"/>
+    <row r="38" ht="15.75" customHeight="1" s="43"/>
+    <row r="39" ht="15.75" customHeight="1" s="43">
+      <c r="A39" s="42" t="n"/>
+    </row>
     <row r="40" ht="15.75" customHeight="1" s="43"/>
-    <row r="41">
-      <c r="A41" s="42" t="n"/>
-    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="42" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="42" t="n"/>
     </row>
-    <row r="44"/>
-    <row r="45">
-      <c r="A45" s="42" t="n"/>
-    </row>
+    <row r="44">
+      <c r="A44" s="42" t="n"/>
+    </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="42" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="42" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-09-30
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DA48"/>
+  <dimension ref="A1:DB49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1038,14 +1038,17 @@
         <v>46291.70971938658</v>
       </c>
       <c r="CY1" s="56" t="n">
-        <v>46293.83729743735</v>
-      </c>
-      <c r="CZ1" s="44" t="inlineStr">
+        <v>46293.83729744213</v>
+      </c>
+      <c r="CZ1" s="56" t="n">
+        <v>46295.7652899918</v>
+      </c>
+      <c r="DA1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DA1" s="44" t="inlineStr">
+      <c r="DB1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1099,12 +1102,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CZ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA2" s="58" t="inlineStr">
+      <c r="DA2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1158,12 +1161,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="CZ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA3" s="58" t="inlineStr">
+      <c r="DA3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1218,12 +1221,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="CZ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1312,12 +1315,15 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CZ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CZ5" t="n">
+        <v>2203.35</v>
       </c>
       <c r="DA5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1377,12 +1383,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CZ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1437,12 +1443,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="CZ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1523,12 +1529,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="CZ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1576,12 +1582,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="CZ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1629,12 +1635,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="CZ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DA10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1692,12 +1698,15 @@
       <c r="CW11" s="42" t="n">
         <v>2535.35</v>
       </c>
-      <c r="CZ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="CZ11" t="n">
+        <v>2513.35</v>
       </c>
       <c r="DA11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1937,6 +1946,9 @@
       <c r="CT16" s="42" t="n">
         <v>2139.35</v>
       </c>
+      <c r="CZ16" t="n">
+        <v>2120.35</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -1977,6 +1989,9 @@
       <c r="CU17" s="42" t="n">
         <v>1967.35</v>
       </c>
+      <c r="CZ17" t="n">
+        <v>1948.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -2012,131 +2027,107 @@
       <c r="CW18" s="42" t="n">
         <v>3205.35</v>
       </c>
+      <c r="CZ18" t="n">
+        <v>3236.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>#8-452B</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="42" t="inlineStr">
         <is>
           <t>874</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="42" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="42" t="inlineStr">
         <is>
           <t>Oct 02</t>
         </is>
       </c>
-      <c r="CY19" t="n">
+      <c r="CY19" s="42" t="n">
         <v>2631.35</v>
       </c>
+      <c r="CZ19" t="n">
+        <v>2609.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" s="42" t="inlineStr">
-        <is>
-          <t>— Off Market —</t>
-        </is>
-      </c>
-      <c r="B20" s="42" t="n"/>
-      <c r="C20" s="42" t="n"/>
-      <c r="D20" s="42" t="n"/>
-      <c r="E20" s="42" t="n"/>
-      <c r="F20" s="42" t="n"/>
-      <c r="G20" s="42" t="n"/>
-      <c r="H20" s="42" t="n"/>
-      <c r="AH20" s="42" t="n"/>
-      <c r="AJ20" s="42" t="n"/>
-      <c r="AN20" s="42" t="n"/>
-      <c r="AP20" s="42" t="n"/>
-      <c r="CZ20" s="42" t="n"/>
-      <c r="DA20" s="42" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>#9-492A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>874</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Oct 22</t>
+        </is>
+      </c>
+      <c r="CZ20" t="n">
+        <v>2644.35</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>5-418</t>
-        </is>
-      </c>
-      <c r="B21" s="42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C21" s="42" t="inlineStr">
-        <is>
-          <t>Building 5, Floor 4</t>
-        </is>
-      </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>2 bed, 1.5 bath</t>
-        </is>
-      </c>
-      <c r="E21" s="42" t="n">
-        <v>1157</v>
-      </c>
-      <c r="F21" s="42" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="G21" s="42" t="inlineStr">
-        <is>
-          <t>Jun 12</t>
-        </is>
-      </c>
-      <c r="H21" s="42" t="inlineStr">
-        <is>
-          <t>Off Market</t>
-        </is>
-      </c>
-      <c r="Z21" s="57" t="n">
-        <v>3379.06</v>
-      </c>
-      <c r="AB21" s="42" t="n">
-        <v>3534.06</v>
-      </c>
-      <c r="AE21" s="42" t="n">
-        <v>3696.06</v>
-      </c>
-      <c r="AG21" s="42" t="n">
-        <v>3663.06</v>
-      </c>
-      <c r="AJ21" s="42" t="n">
-        <v>3610.06</v>
-      </c>
-      <c r="CZ21" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA21" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>— Off Market —</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="42" t="n"/>
+      <c r="D21" s="42" t="n"/>
+      <c r="E21" s="42" t="n"/>
+      <c r="F21" s="42" t="n"/>
+      <c r="G21" s="42" t="n"/>
+      <c r="H21" s="42" t="n"/>
+      <c r="AH21" s="42" t="n"/>
+      <c r="AJ21" s="42" t="n"/>
+      <c r="AN21" s="42" t="n"/>
+      <c r="AP21" s="42" t="n"/>
+      <c r="DA21" s="42" t="n"/>
+      <c r="DB21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>9-486A</t>
+          <t>5-418</t>
         </is>
       </c>
       <c r="B22" s="42" t="inlineStr">
@@ -2146,25 +2137,25 @@
       </c>
       <c r="C22" s="42" t="inlineStr">
         <is>
-          <t>Building 9, Floor 3</t>
+          <t>Building 5, Floor 4</t>
         </is>
       </c>
       <c r="D22" s="42" t="inlineStr">
         <is>
-          <t>1 bed, 1 bath</t>
+          <t>2 bed, 1.5 bath</t>
         </is>
       </c>
       <c r="E22" s="42" t="n">
-        <v>638</v>
+        <v>1157</v>
       </c>
       <c r="F22" s="42" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>B22</t>
         </is>
       </c>
       <c r="G22" s="42" t="inlineStr">
         <is>
-          <t>Available Now</t>
+          <t>Jun 12</t>
         </is>
       </c>
       <c r="H22" s="42" t="inlineStr">
@@ -2172,21 +2163,27 @@
           <t>Off Market</t>
         </is>
       </c>
-      <c r="AF22" s="42" t="n">
-        <v>2357.06</v>
+      <c r="Z22" s="57" t="n">
+        <v>3379.06</v>
+      </c>
+      <c r="AB22" s="42" t="n">
+        <v>3534.06</v>
+      </c>
+      <c r="AE22" s="42" t="n">
+        <v>3696.06</v>
       </c>
       <c r="AG22" s="42" t="n">
-        <v>2316.06</v>
-      </c>
-      <c r="AI22" s="42" t="n">
-        <v>2430.06</v>
-      </c>
-      <c r="CZ22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3663.06</v>
+      </c>
+      <c r="AJ22" s="42" t="n">
+        <v>3610.06</v>
       </c>
       <c r="DA22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2195,581 +2192,639 @@
     <row r="23" ht="15.75" customHeight="1" s="43">
       <c r="A23" s="42" t="inlineStr">
         <is>
+          <t>9-486A</t>
+        </is>
+      </c>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>Building 9, Floor 3</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>1 bed, 1 bath</t>
+        </is>
+      </c>
+      <c r="E23" s="42" t="n">
+        <v>638</v>
+      </c>
+      <c r="F23" s="42" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="G23" s="42" t="inlineStr">
+        <is>
+          <t>Available Now</t>
+        </is>
+      </c>
+      <c r="H23" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
+      <c r="AF23" s="42" t="n">
+        <v>2357.06</v>
+      </c>
+      <c r="AG23" s="42" t="n">
+        <v>2316.06</v>
+      </c>
+      <c r="AI23" s="42" t="n">
+        <v>2430.06</v>
+      </c>
+      <c r="DA23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="43">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
           <t>9-490A</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B24" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E24" s="42" t="n">
         <v>1044</v>
       </c>
-      <c r="F23" s="42" t="inlineStr">
+      <c r="F24" s="42" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G23" s="42" t="inlineStr">
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H23" s="42" t="inlineStr">
+      <c r="H24" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I23" s="42" t="n">
+      <c r="I24" s="42" t="n">
         <v>3414.5</v>
       </c>
-      <c r="J23" s="42" t="n">
+      <c r="J24" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="K23" s="42" t="n">
+      <c r="K24" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="L23" s="42" t="n">
+      <c r="L24" s="42" t="n">
         <v>3353.85</v>
       </c>
-      <c r="N23" s="42" t="n">
+      <c r="N24" s="42" t="n">
         <v>3392.85</v>
       </c>
-      <c r="O23" s="42" t="n">
+      <c r="O24" s="42" t="n">
         <v>3334.85</v>
       </c>
-      <c r="Q23" s="42" t="n">
+      <c r="Q24" s="42" t="n">
         <v>3275.85</v>
       </c>
-      <c r="T23" s="42" t="n">
+      <c r="T24" s="42" t="n">
         <v>3423.85</v>
       </c>
-      <c r="U23" s="42" t="n">
+      <c r="U24" s="42" t="n">
         <v>3500.85</v>
       </c>
-      <c r="V23" s="42" t="n">
+      <c r="V24" s="42" t="n">
         <v>3569.06</v>
       </c>
-      <c r="W23" s="42" t="n">
+      <c r="W24" s="42" t="n">
         <v>3239.06</v>
       </c>
-      <c r="AA23" s="42" t="n">
+      <c r="AA24" s="42" t="n">
         <v>3248.06</v>
       </c>
-      <c r="AB23" s="42" t="n">
+      <c r="AB24" s="42" t="n">
         <v>3403.06</v>
       </c>
-      <c r="AC23" s="42" t="n">
+      <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="CZ23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA23" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="43">
-      <c r="A24" s="61" t="inlineStr">
+      <c r="DA24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="43">
+      <c r="A25" s="61" t="inlineStr">
         <is>
           <t>8-470A</t>
         </is>
       </c>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="B25" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C24" s="61" t="inlineStr">
+      <c r="C25" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D24" s="61" t="inlineStr">
+      <c r="D25" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E24" s="63" t="n">
+      <c r="E25" s="63" t="n">
         <v>1044</v>
       </c>
-      <c r="F24" s="64" t="inlineStr">
+      <c r="F25" s="64" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="G24" s="64" t="inlineStr">
+      <c r="G25" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H24" s="65" t="inlineStr">
+      <c r="H25" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I24" s="66" t="n">
+      <c r="I25" s="66" t="n">
         <v>3429.5</v>
       </c>
-      <c r="J24" s="67" t="n">
+      <c r="J25" s="67" t="n">
         <v>3368.85</v>
       </c>
-      <c r="K24" s="66" t="n">
+      <c r="K25" s="66" t="n">
         <v>3368.85</v>
       </c>
-      <c r="L24" s="68" t="n">
+      <c r="L25" s="68" t="n">
         <v>3368.85</v>
       </c>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="69" t="n">
+      <c r="M25" s="68" t="n"/>
+      <c r="N25" s="69" t="n">
         <v>3407.85</v>
       </c>
-      <c r="O24" s="69" t="n">
+      <c r="O25" s="69" t="n">
         <v>3349.85</v>
       </c>
-      <c r="Q24" s="42" t="n">
+      <c r="Q25" s="42" t="n">
         <v>3290.85</v>
       </c>
-      <c r="T24" s="42" t="n">
+      <c r="T25" s="42" t="n">
         <v>3438.85</v>
       </c>
-      <c r="U24" s="42" t="n">
+      <c r="U25" s="42" t="n">
         <v>3515.85</v>
       </c>
-      <c r="V24" s="42" t="n">
+      <c r="V25" s="42" t="n">
         <v>3584.06</v>
       </c>
-      <c r="W24" s="42" t="n">
+      <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="CZ24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA24" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="43">
-      <c r="A25" s="42" t="inlineStr">
+      <c r="DA25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB25" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="43">
+      <c r="A26" s="42" t="inlineStr">
         <is>
           <t>9-486B</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C26" s="42" t="inlineStr">
         <is>
           <t>Building 9, Floor 4</t>
         </is>
       </c>
-      <c r="D25" s="42" t="inlineStr">
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E25" s="42" t="n">
+      <c r="E26" s="42" t="n">
         <v>639</v>
       </c>
-      <c r="F25" s="42" t="inlineStr">
+      <c r="F26" s="42" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="G25" s="42" t="inlineStr">
+      <c r="G26" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H25" s="42" t="inlineStr">
+      <c r="H26" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I25" s="42" t="n">
+      <c r="I26" s="42" t="n">
         <v>2325.5</v>
       </c>
-      <c r="M25" s="42" t="n">
+      <c r="M26" s="42" t="n">
         <v>2296.85</v>
       </c>
-      <c r="N25" s="42" t="n">
+      <c r="N26" s="42" t="n">
         <v>2311.85</v>
       </c>
-      <c r="Q25" s="42" t="n">
+      <c r="Q26" s="42" t="n">
         <v>2392.85</v>
       </c>
-      <c r="V25" s="42" t="n">
+      <c r="V26" s="42" t="n">
         <v>2429.06</v>
       </c>
-      <c r="W25" s="42" t="n">
+      <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="CZ25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA25" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="43">
-      <c r="A26" s="61" t="inlineStr">
+      <c r="DA26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB26" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="43">
+      <c r="A27" s="61" t="inlineStr">
         <is>
           <t>8-464A</t>
         </is>
       </c>
-      <c r="B26" s="62" t="inlineStr">
+      <c r="B27" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C26" s="61" t="inlineStr">
+      <c r="C27" s="61" t="inlineStr">
         <is>
           <t>Building 8, Floor 3</t>
         </is>
       </c>
-      <c r="D26" s="61" t="inlineStr">
+      <c r="D27" s="61" t="inlineStr">
         <is>
           <t>2 bed, 1.5 bath</t>
         </is>
       </c>
-      <c r="E26" s="63" t="n">
+      <c r="E27" s="63" t="n">
         <v>1016</v>
       </c>
-      <c r="F26" s="64" t="inlineStr">
+      <c r="F27" s="64" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="G26" s="64" t="inlineStr">
+      <c r="G27" s="64" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H26" s="65" t="inlineStr">
+      <c r="H27" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I26" s="66" t="n">
+      <c r="I27" s="66" t="n">
         <v>3219.5</v>
       </c>
-      <c r="J26" s="67" t="n">
+      <c r="J27" s="67" t="n">
         <v>3158.85</v>
       </c>
-      <c r="K26" s="66" t="n">
+      <c r="K27" s="66" t="n">
         <v>3158.85</v>
       </c>
-      <c r="L26" s="68" t="n">
+      <c r="L27" s="68" t="n">
         <v>3158.85</v>
       </c>
-      <c r="M26" s="68" t="n"/>
-      <c r="N26" s="69" t="n">
+      <c r="M27" s="68" t="n"/>
+      <c r="N27" s="69" t="n">
         <v>3197.85</v>
       </c>
-      <c r="O26" s="69" t="n">
+      <c r="O27" s="69" t="n">
         <v>3139.85</v>
       </c>
-      <c r="Q26" s="42" t="n">
+      <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="CZ26" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA26" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="43">
-      <c r="A27" s="42" t="inlineStr">
+      <c r="DA27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB27" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="43">
+      <c r="A28" s="42" t="inlineStr">
         <is>
           <t>8-464C</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B28" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>Building 8, Floor 1</t>
         </is>
       </c>
-      <c r="D27" s="42" t="inlineStr">
+      <c r="D28" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E27" s="42" t="n">
+      <c r="E28" s="42" t="n">
         <v>970</v>
       </c>
-      <c r="F27" s="42" t="inlineStr">
+      <c r="F28" s="42" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="G27" s="42" t="inlineStr">
+      <c r="G28" s="42" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="H27" s="42" t="inlineStr">
+      <c r="H28" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I27" s="72" t="n">
+      <c r="I28" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="J27" s="72" t="n">
+      <c r="J28" s="72" t="n">
         <v>3044.85</v>
       </c>
-      <c r="K27" s="72" t="n">
+      <c r="K28" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="L27" s="72" t="n">
+      <c r="L28" s="72" t="n">
         <v>2983.85</v>
       </c>
-      <c r="M27" s="72" t="n"/>
-      <c r="N27" s="42" t="n">
+      <c r="M28" s="72" t="n"/>
+      <c r="N28" s="42" t="n">
         <v>3022.85</v>
       </c>
-      <c r="O27" s="42" t="n">
+      <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="CZ27" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA27" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="43">
-      <c r="A28" s="61" t="inlineStr">
+      <c r="DA28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB28" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="61" t="inlineStr">
         <is>
           <t>6-475</t>
         </is>
       </c>
-      <c r="B28" s="62" t="inlineStr">
+      <c r="B29" s="62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C28" s="61" t="inlineStr">
+      <c r="C29" s="61" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D28" s="61" t="inlineStr">
+      <c r="D29" s="61" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E28" s="64" t="n">
+      <c r="E29" s="64" t="n">
         <v>651</v>
       </c>
-      <c r="F28" s="64" t="inlineStr">
+      <c r="F29" s="64" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="G28" s="73" t="n">
+      <c r="G29" s="73" t="n">
         <v>46109</v>
       </c>
-      <c r="H28" s="65" t="inlineStr">
+      <c r="H29" s="65" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I28" s="66" t="n">
+      <c r="I29" s="66" t="n">
         <v>2155.5</v>
       </c>
-      <c r="J28" s="66" t="n">
+      <c r="J29" s="66" t="n">
         <v>1969.85</v>
       </c>
-      <c r="K28" s="67" t="n">
+      <c r="K29" s="67" t="n">
         <v>1969.85</v>
       </c>
-      <c r="L28" s="68" t="n">
+      <c r="L29" s="68" t="n">
         <v>1969.85</v>
       </c>
-      <c r="M28" s="68" t="n"/>
-      <c r="N28" s="69" t="n">
+      <c r="M29" s="68" t="n"/>
+      <c r="N29" s="69" t="n">
         <v>1964.85</v>
       </c>
-      <c r="O28" s="69" t="n"/>
-      <c r="CZ28" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA28" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="75" t="inlineStr">
+      <c r="O29" s="69" t="n"/>
+      <c r="DA29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB29" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="75" t="inlineStr">
         <is>
           <t>6-436</t>
         </is>
       </c>
-      <c r="B29" s="76" t="inlineStr">
+      <c r="B30" s="76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C29" s="75" t="inlineStr">
+      <c r="C30" s="75" t="inlineStr">
         <is>
           <t>Building 6, Floor 2</t>
         </is>
       </c>
-      <c r="D29" s="75" t="inlineStr">
+      <c r="D30" s="75" t="inlineStr">
         <is>
           <t>2 bed, 2.5 bath</t>
         </is>
       </c>
-      <c r="E29" s="77" t="n">
+      <c r="E30" s="77" t="n">
         <v>1227</v>
       </c>
-      <c r="F29" s="78" t="inlineStr">
+      <c r="F30" s="78" t="inlineStr">
         <is>
           <t>B27</t>
         </is>
       </c>
-      <c r="G29" s="79" t="n">
+      <c r="G30" s="79" t="n">
         <v>46077</v>
       </c>
-      <c r="H29" s="80" t="inlineStr">
+      <c r="H30" s="80" t="inlineStr">
         <is>
           <t>⚠ "Contact Us" — may be leased; Off Market</t>
         </is>
       </c>
-      <c r="I29" s="81" t="n">
+      <c r="I30" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="J29" s="81" t="n">
+      <c r="J30" s="81" t="n">
         <v>3376.5</v>
       </c>
-      <c r="K29" s="82" t="inlineStr">
+      <c r="K30" s="82" t="inlineStr">
         <is>
           <t>⚠ Contact Us</t>
         </is>
       </c>
-      <c r="L29" s="83" t="inlineStr">
+      <c r="L30" s="83" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="M29" s="83" t="n"/>
-      <c r="N29" s="84" t="n"/>
-      <c r="O29" s="69" t="n"/>
-      <c r="CZ29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA29" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="42" t="inlineStr">
+      <c r="M30" s="83" t="n"/>
+      <c r="N30" s="84" t="n"/>
+      <c r="O30" s="69" t="n"/>
+      <c r="DA30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB30" s="71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="43">
+      <c r="A31" s="42" t="inlineStr">
         <is>
           <t>6-481</t>
         </is>
       </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B31" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C30" s="42" t="inlineStr">
+      <c r="C31" s="42" t="inlineStr">
         <is>
           <t>Building 6, Floor 1</t>
         </is>
       </c>
-      <c r="D30" s="42" t="inlineStr">
+      <c r="D31" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E30" s="42" t="n">
+      <c r="E31" s="42" t="n">
         <v>605</v>
       </c>
-      <c r="F30" s="42" t="inlineStr">
+      <c r="F31" s="42" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="G30" s="47" t="n">
+      <c r="G31" s="47" t="n">
         <v>46118</v>
       </c>
-      <c r="H30" s="42" t="inlineStr">
+      <c r="H31" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
       </c>
-      <c r="I30" s="72" t="n">
+      <c r="I31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="J30" s="72" t="n">
+      <c r="J31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="K30" s="72" t="n">
+      <c r="K31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="L30" s="72" t="n">
+      <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="CZ30" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DA30" s="58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" s="43"/>
+      <c r="DA31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DB31" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="32"/>
     <row r="33"/>
     <row r="34" ht="15.75" customHeight="1" s="43"/>
@@ -2777,29 +2832,30 @@
     <row r="36" ht="15.75" customHeight="1" s="43"/>
     <row r="37"/>
     <row r="38" ht="15.75" customHeight="1" s="43"/>
-    <row r="39" ht="15.75" customHeight="1" s="43">
-      <c r="A39" s="42" t="n"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" s="43"/>
+    <row r="39" ht="15.75" customHeight="1" s="43"/>
+    <row r="40" ht="15.75" customHeight="1" s="43">
+      <c r="A40" s="42" t="n"/>
+    </row>
     <row r="41"/>
-    <row r="42">
-      <c r="A42" s="42" t="n"/>
-    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="42" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="42" t="n"/>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="42" t="n"/>
-    </row>
+    <row r="45">
+      <c r="A45" s="42" t="n"/>
+    </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="42" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="42" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-01
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DB49"/>
+  <dimension ref="A1:DC49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1041,14 +1041,17 @@
         <v>46293.83729744213</v>
       </c>
       <c r="CZ1" s="56" t="n">
-        <v>46295.7652899918</v>
-      </c>
-      <c r="DA1" s="44" t="inlineStr">
+        <v>46295.76528998843</v>
+      </c>
+      <c r="DA1" s="56" t="n">
+        <v>46296.78383817949</v>
+      </c>
+      <c r="DB1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DB1" s="44" t="inlineStr">
+      <c r="DC1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1102,12 +1105,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DA2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB2" s="58" t="inlineStr">
+      <c r="DB2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1161,12 +1164,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DA3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB3" s="58" t="inlineStr">
+      <c r="DB3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1221,12 +1224,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DA4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1315,15 +1318,18 @@
       <c r="CT5" s="42" t="n">
         <v>2221.35</v>
       </c>
-      <c r="CZ5" t="n">
+      <c r="CZ5" s="42" t="n">
         <v>2203.35</v>
       </c>
-      <c r="DA5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DA5" t="n">
+        <v>2184.35</v>
       </c>
       <c r="DB5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1383,12 +1389,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DA6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1443,12 +1449,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DA7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1529,12 +1535,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DA8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1582,12 +1588,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DA9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1635,12 +1641,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DA10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1698,15 +1704,18 @@
       <c r="CW11" s="42" t="n">
         <v>2535.35</v>
       </c>
-      <c r="CZ11" t="n">
+      <c r="CZ11" s="42" t="n">
         <v>2513.35</v>
       </c>
-      <c r="DA11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DA11" t="n">
+        <v>2491.35</v>
       </c>
       <c r="DB11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1946,8 +1955,11 @@
       <c r="CT16" s="42" t="n">
         <v>2139.35</v>
       </c>
-      <c r="CZ16" t="n">
+      <c r="CZ16" s="42" t="n">
         <v>2120.35</v>
+      </c>
+      <c r="DA16" t="n">
+        <v>2101.35</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
@@ -1989,8 +2001,11 @@
       <c r="CU17" s="42" t="n">
         <v>1967.35</v>
       </c>
-      <c r="CZ17" t="n">
+      <c r="CZ17" s="42" t="n">
         <v>1948.35</v>
+      </c>
+      <c r="DA17" t="n">
+        <v>1929.35</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
@@ -2027,7 +2042,7 @@
       <c r="CW18" s="42" t="n">
         <v>3205.35</v>
       </c>
-      <c r="CZ18" t="n">
+      <c r="CZ18" s="42" t="n">
         <v>3236.35</v>
       </c>
     </row>
@@ -2065,43 +2080,49 @@
       <c r="CY19" s="42" t="n">
         <v>2631.35</v>
       </c>
-      <c r="CZ19" t="n">
+      <c r="CZ19" s="42" t="n">
         <v>2609.35</v>
       </c>
+      <c r="DA19" t="n">
+        <v>2587.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>#9-492A</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>1 bed, 1 bath</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="42" t="inlineStr">
         <is>
           <t>874</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="42" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="42" t="inlineStr">
         <is>
           <t>Oct 22</t>
         </is>
       </c>
-      <c r="CZ20" t="n">
+      <c r="CZ20" s="42" t="n">
         <v>2644.35</v>
+      </c>
+      <c r="DA20" t="n">
+        <v>2621.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2121,8 +2142,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DA21" s="42" t="n"/>
       <c r="DB21" s="42" t="n"/>
+      <c r="DC21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2178,12 +2199,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DA22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB22" s="58" t="inlineStr">
+      <c r="DB22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2237,12 +2258,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DA23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DB23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2329,12 +2350,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DA24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB24" s="58" t="inlineStr">
+      <c r="DB24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2413,12 +2434,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DA25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB25" s="58" t="inlineStr">
+      <c r="DB25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2481,12 +2502,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DA26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB26" s="58" t="inlineStr">
+      <c r="DB26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2553,12 +2574,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DA27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB27" s="71" t="inlineStr">
+      <c r="DB27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2622,12 +2643,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DA28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB28" s="58" t="inlineStr">
+      <c r="DB28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2687,12 +2708,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DA29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB29" s="71" t="inlineStr">
+      <c r="DB29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2754,12 +2775,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DA30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB30" s="71" t="inlineStr">
+      <c r="DB30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2814,12 +2835,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DA31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DB31" s="58" t="inlineStr">
+      <c r="DB31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DC31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-02
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DC49"/>
+  <dimension ref="A1:DD49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1044,14 +1044,17 @@
         <v>46295.76528998843</v>
       </c>
       <c r="DA1" s="56" t="n">
-        <v>46296.78383817949</v>
-      </c>
-      <c r="DB1" s="44" t="inlineStr">
+        <v>46296.78383818287</v>
+      </c>
+      <c r="DB1" s="56" t="n">
+        <v>46297.76379051826</v>
+      </c>
+      <c r="DC1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DC1" s="44" t="inlineStr">
+      <c r="DD1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1105,12 +1108,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DB2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC2" s="58" t="inlineStr">
+      <c r="DC2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1164,12 +1167,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DB3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC3" s="58" t="inlineStr">
+      <c r="DC3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1224,12 +1227,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DB4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1321,15 +1324,18 @@
       <c r="CZ5" s="42" t="n">
         <v>2203.35</v>
       </c>
-      <c r="DA5" t="n">
+      <c r="DA5" s="42" t="n">
         <v>2184.35</v>
       </c>
-      <c r="DB5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DB5" t="n">
+        <v>2222.35</v>
       </c>
       <c r="DC5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1389,12 +1395,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DB6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1449,12 +1455,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DB7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1535,12 +1541,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DB8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1588,12 +1594,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DB9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1641,12 +1647,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DB10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1707,15 +1713,15 @@
       <c r="CZ11" s="42" t="n">
         <v>2513.35</v>
       </c>
-      <c r="DA11" t="n">
+      <c r="DA11" s="42" t="n">
         <v>2491.35</v>
       </c>
-      <c r="DB11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1770,6 +1776,9 @@
       <c r="CR12" s="42" t="n">
         <v>1986.35</v>
       </c>
+      <c r="DB12" t="n">
+        <v>1961.35</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -1958,7 +1967,7 @@
       <c r="CZ16" s="42" t="n">
         <v>2120.35</v>
       </c>
-      <c r="DA16" t="n">
+      <c r="DA16" s="42" t="n">
         <v>2101.35</v>
       </c>
     </row>
@@ -2004,7 +2013,7 @@
       <c r="CZ17" s="42" t="n">
         <v>1948.35</v>
       </c>
-      <c r="DA17" t="n">
+      <c r="DA17" s="42" t="n">
         <v>1929.35</v>
       </c>
     </row>
@@ -2083,7 +2092,7 @@
       <c r="CZ19" s="42" t="n">
         <v>2609.35</v>
       </c>
-      <c r="DA19" t="n">
+      <c r="DA19" s="42" t="n">
         <v>2587.35</v>
       </c>
     </row>
@@ -2121,7 +2130,7 @@
       <c r="CZ20" s="42" t="n">
         <v>2644.35</v>
       </c>
-      <c r="DA20" t="n">
+      <c r="DA20" s="42" t="n">
         <v>2621.35</v>
       </c>
     </row>
@@ -2142,8 +2151,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DB21" s="42" t="n"/>
       <c r="DC21" s="42" t="n"/>
+      <c r="DD21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2199,12 +2208,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DB22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC22" s="58" t="inlineStr">
+      <c r="DC22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2258,12 +2267,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DB23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DC23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2350,12 +2359,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DB24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC24" s="58" t="inlineStr">
+      <c r="DC24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2434,12 +2443,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DB25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC25" s="58" t="inlineStr">
+      <c r="DC25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2502,12 +2511,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DB26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC26" s="58" t="inlineStr">
+      <c r="DC26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2574,12 +2583,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DB27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC27" s="71" t="inlineStr">
+      <c r="DC27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2643,12 +2652,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DB28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC28" s="58" t="inlineStr">
+      <c r="DC28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2708,12 +2717,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DB29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC29" s="71" t="inlineStr">
+      <c r="DC29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2775,12 +2784,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DB30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC30" s="71" t="inlineStr">
+      <c r="DC30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2835,12 +2844,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DB31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DC31" s="58" t="inlineStr">
+      <c r="DC31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DD31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-04
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DD49"/>
+  <dimension ref="A1:DE49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1047,14 +1047,17 @@
         <v>46296.78383818287</v>
       </c>
       <c r="DB1" s="56" t="n">
-        <v>46297.76379051826</v>
-      </c>
-      <c r="DC1" s="44" t="inlineStr">
+        <v>46297.76379052083</v>
+      </c>
+      <c r="DC1" s="56" t="n">
+        <v>46299.72608766154</v>
+      </c>
+      <c r="DD1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DD1" s="44" t="inlineStr">
+      <c r="DE1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1108,12 +1111,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DC2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD2" s="58" t="inlineStr">
+      <c r="DD2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1167,12 +1170,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DC3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD3" s="58" t="inlineStr">
+      <c r="DD3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1227,12 +1230,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DC4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1327,15 +1330,18 @@
       <c r="DA5" s="42" t="n">
         <v>2184.35</v>
       </c>
-      <c r="DB5" t="n">
+      <c r="DB5" s="42" t="n">
         <v>2222.35</v>
       </c>
-      <c r="DC5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DC5" t="n">
+        <v>2204.35</v>
       </c>
       <c r="DD5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1395,12 +1401,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DC6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1455,12 +1461,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DC7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1541,12 +1547,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DC8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1594,12 +1600,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DC9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1647,12 +1653,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DC10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1716,12 +1722,15 @@
       <c r="DA11" s="42" t="n">
         <v>2491.35</v>
       </c>
-      <c r="DC11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DC11" t="n">
+        <v>2469.35</v>
       </c>
       <c r="DD11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1776,8 +1785,11 @@
       <c r="CR12" s="42" t="n">
         <v>1986.35</v>
       </c>
-      <c r="DB12" t="n">
+      <c r="DB12" s="42" t="n">
         <v>1961.35</v>
+      </c>
+      <c r="DC12" t="n">
+        <v>1942.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1970,6 +1982,9 @@
       <c r="DA16" s="42" t="n">
         <v>2101.35</v>
       </c>
+      <c r="DC16" t="n">
+        <v>2081.35</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
       <c r="A17" s="42" t="inlineStr">
@@ -2016,6 +2031,9 @@
       <c r="DA17" s="42" t="n">
         <v>1929.35</v>
       </c>
+      <c r="DC17" t="n">
+        <v>1910.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -2095,6 +2113,9 @@
       <c r="DA19" s="42" t="n">
         <v>2587.35</v>
       </c>
+      <c r="DC19" t="n">
+        <v>2565.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
@@ -2132,6 +2153,9 @@
       </c>
       <c r="DA20" s="42" t="n">
         <v>2621.35</v>
+      </c>
+      <c r="DC20" t="n">
+        <v>2599.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2151,8 +2175,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DC21" s="42" t="n"/>
       <c r="DD21" s="42" t="n"/>
+      <c r="DE21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2208,12 +2232,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DC22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD22" s="58" t="inlineStr">
+      <c r="DD22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2267,12 +2291,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DC23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DD23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2359,12 +2383,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DC24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD24" s="58" t="inlineStr">
+      <c r="DD24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2443,12 +2467,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DC25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD25" s="58" t="inlineStr">
+      <c r="DD25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2511,12 +2535,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DC26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD26" s="58" t="inlineStr">
+      <c r="DD26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2583,12 +2607,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DC27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD27" s="71" t="inlineStr">
+      <c r="DD27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2652,12 +2676,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DC28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD28" s="58" t="inlineStr">
+      <c r="DD28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2717,12 +2741,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DC29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD29" s="71" t="inlineStr">
+      <c r="DD29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2784,12 +2808,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DC30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD30" s="71" t="inlineStr">
+      <c r="DD30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2844,12 +2868,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DC31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DD31" s="58" t="inlineStr">
+      <c r="DD31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DE31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-06
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DE49"/>
+  <dimension ref="A1:DF49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1050,14 +1050,17 @@
         <v>46297.76379052083</v>
       </c>
       <c r="DC1" s="56" t="n">
-        <v>46299.72608766154</v>
-      </c>
-      <c r="DD1" s="44" t="inlineStr">
+        <v>46299.72608766203</v>
+      </c>
+      <c r="DD1" s="56" t="n">
+        <v>46301.57840095825</v>
+      </c>
+      <c r="DE1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DE1" s="44" t="inlineStr">
+      <c r="DF1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1111,12 +1114,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DD2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE2" s="58" t="inlineStr">
+      <c r="DE2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1170,12 +1173,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DD3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE3" s="58" t="inlineStr">
+      <c r="DE3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1230,12 +1233,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DD4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1333,15 +1336,15 @@
       <c r="DB5" s="42" t="n">
         <v>2222.35</v>
       </c>
-      <c r="DC5" t="n">
+      <c r="DC5" s="42" t="n">
         <v>2204.35</v>
       </c>
-      <c r="DD5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1401,12 +1404,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DD6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1461,12 +1464,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DD7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1547,12 +1550,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DD8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1600,12 +1603,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DD9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1653,12 +1656,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DD10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1722,15 +1725,15 @@
       <c r="DA11" s="42" t="n">
         <v>2491.35</v>
       </c>
-      <c r="DC11" t="n">
+      <c r="DC11" s="42" t="n">
         <v>2469.35</v>
       </c>
-      <c r="DD11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1788,8 +1791,11 @@
       <c r="DB12" s="42" t="n">
         <v>1961.35</v>
       </c>
-      <c r="DC12" t="n">
+      <c r="DC12" s="42" t="n">
         <v>1942.35</v>
+      </c>
+      <c r="DD12" t="n">
+        <v>1931.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1982,7 +1988,7 @@
       <c r="DA16" s="42" t="n">
         <v>2101.35</v>
       </c>
-      <c r="DC16" t="n">
+      <c r="DC16" s="42" t="n">
         <v>2081.35</v>
       </c>
     </row>
@@ -2031,7 +2037,7 @@
       <c r="DA17" s="42" t="n">
         <v>1929.35</v>
       </c>
-      <c r="DC17" t="n">
+      <c r="DC17" s="42" t="n">
         <v>1910.35</v>
       </c>
     </row>
@@ -2113,7 +2119,7 @@
       <c r="DA19" s="42" t="n">
         <v>2587.35</v>
       </c>
-      <c r="DC19" t="n">
+      <c r="DC19" s="42" t="n">
         <v>2565.35</v>
       </c>
     </row>
@@ -2154,7 +2160,7 @@
       <c r="DA20" s="42" t="n">
         <v>2621.35</v>
       </c>
-      <c r="DC20" t="n">
+      <c r="DC20" s="42" t="n">
         <v>2599.35</v>
       </c>
     </row>
@@ -2175,8 +2181,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DD21" s="42" t="n"/>
       <c r="DE21" s="42" t="n"/>
+      <c r="DF21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2232,12 +2238,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DD22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE22" s="58" t="inlineStr">
+      <c r="DE22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2291,12 +2297,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DD23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DE23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2383,12 +2389,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DD24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE24" s="58" t="inlineStr">
+      <c r="DE24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2467,12 +2473,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DD25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE25" s="58" t="inlineStr">
+      <c r="DE25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2535,12 +2541,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DD26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE26" s="58" t="inlineStr">
+      <c r="DE26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2607,12 +2613,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DD27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE27" s="71" t="inlineStr">
+      <c r="DE27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2676,12 +2682,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DD28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE28" s="58" t="inlineStr">
+      <c r="DE28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2741,12 +2747,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DD29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE29" s="71" t="inlineStr">
+      <c r="DE29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2808,12 +2814,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DD30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE30" s="71" t="inlineStr">
+      <c r="DE30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2868,12 +2874,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DD31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DE31" s="58" t="inlineStr">
+      <c r="DE31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DF31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-08
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DG49"/>
+  <dimension ref="A1:DH49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1056,14 +1056,17 @@
         <v>46301.57840096065</v>
       </c>
       <c r="DE1" s="56" t="n">
-        <v>46301.78665378426</v>
-      </c>
-      <c r="DF1" s="44" t="inlineStr">
+        <v>46301.78665378472</v>
+      </c>
+      <c r="DF1" s="56" t="n">
+        <v>46303.8016057431</v>
+      </c>
+      <c r="DG1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DG1" s="44" t="inlineStr">
+      <c r="DH1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1117,12 +1120,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DF2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG2" s="58" t="inlineStr">
+      <c r="DG2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1176,12 +1179,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DF3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG3" s="58" t="inlineStr">
+      <c r="DG3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1236,12 +1239,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DF4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1342,15 +1345,15 @@
       <c r="DC5" s="42" t="n">
         <v>2204.35</v>
       </c>
-      <c r="DE5" t="n">
+      <c r="DE5" s="42" t="n">
         <v>2149.35</v>
       </c>
-      <c r="DF5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1410,12 +1413,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DF6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1470,12 +1473,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DF7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1556,12 +1559,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DF8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1609,12 +1612,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DF9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1662,12 +1665,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DF10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1734,15 +1737,18 @@
       <c r="DC11" s="42" t="n">
         <v>2469.35</v>
       </c>
-      <c r="DE11" t="n">
+      <c r="DE11" s="42" t="n">
         <v>2446.35</v>
       </c>
-      <c r="DF11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DF11" t="n">
+        <v>2453.35</v>
       </c>
       <c r="DG11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1806,8 +1812,11 @@
       <c r="DD12" s="42" t="n">
         <v>1931.35</v>
       </c>
-      <c r="DE12" t="n">
+      <c r="DE12" s="42" t="n">
         <v>1876.35</v>
+      </c>
+      <c r="DF12" t="n">
+        <v>1866.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1855,6 +1864,9 @@
       <c r="CM13" s="42" t="n">
         <v>2459.06</v>
       </c>
+      <c r="DF13" t="n">
+        <v>2348.35</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -2003,8 +2015,11 @@
       <c r="DC16" s="42" t="n">
         <v>2081.35</v>
       </c>
-      <c r="DE16" t="n">
+      <c r="DE16" s="42" t="n">
         <v>2063.35</v>
+      </c>
+      <c r="DF16" t="n">
+        <v>2069.35</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="43">
@@ -2055,7 +2070,7 @@
       <c r="DC17" s="42" t="n">
         <v>1910.35</v>
       </c>
-      <c r="DE17" t="n">
+      <c r="DE17" s="42" t="n">
         <v>1892.35</v>
       </c>
     </row>
@@ -2128,6 +2143,11 @@
           <t>Oct 02</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="CY19" s="42" t="n">
         <v>2631.35</v>
       </c>
@@ -2140,7 +2160,7 @@
       <c r="DC19" s="42" t="n">
         <v>2565.35</v>
       </c>
-      <c r="DE19" t="n">
+      <c r="DE19" s="42" t="n">
         <v>2543.35</v>
       </c>
     </row>
@@ -2184,7 +2204,7 @@
       <c r="DC20" s="42" t="n">
         <v>2599.35</v>
       </c>
-      <c r="DE20" t="n">
+      <c r="DE20" s="42" t="n">
         <v>2577.35</v>
       </c>
     </row>
@@ -2205,8 +2225,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DF21" s="42" t="n"/>
       <c r="DG21" s="42" t="n"/>
+      <c r="DH21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2262,12 +2282,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DF22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG22" s="58" t="inlineStr">
+      <c r="DG22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2321,12 +2341,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DF23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DG23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2413,12 +2433,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DF24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG24" s="58" t="inlineStr">
+      <c r="DG24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2497,12 +2517,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DF25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG25" s="58" t="inlineStr">
+      <c r="DG25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2565,12 +2585,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DF26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG26" s="58" t="inlineStr">
+      <c r="DG26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2637,12 +2657,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DF27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG27" s="71" t="inlineStr">
+      <c r="DG27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2706,12 +2726,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DF28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG28" s="58" t="inlineStr">
+      <c r="DG28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2771,12 +2791,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DF29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG29" s="71" t="inlineStr">
+      <c r="DG29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2838,12 +2858,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DF30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG30" s="71" t="inlineStr">
+      <c r="DG30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2898,12 +2918,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DF31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DG31" s="58" t="inlineStr">
+      <c r="DG31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DH31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-09
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DH49"/>
+  <dimension ref="A1:DI49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1059,14 +1059,17 @@
         <v>46301.78665378472</v>
       </c>
       <c r="DF1" s="56" t="n">
-        <v>46303.8016057431</v>
-      </c>
-      <c r="DG1" s="44" t="inlineStr">
+        <v>46303.80160574074</v>
+      </c>
+      <c r="DG1" s="56" t="n">
+        <v>46304.78105941539</v>
+      </c>
+      <c r="DH1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DH1" s="44" t="inlineStr">
+      <c r="DI1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1120,12 +1123,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DG2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH2" s="58" t="inlineStr">
+      <c r="DH2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1179,12 +1182,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DG3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH3" s="58" t="inlineStr">
+      <c r="DH3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1239,12 +1242,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DG4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1348,12 +1351,12 @@
       <c r="DE5" s="42" t="n">
         <v>2149.35</v>
       </c>
-      <c r="DG5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1413,12 +1416,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DG6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1473,12 +1476,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DG7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1559,12 +1562,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DG8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1612,12 +1615,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DG9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1665,12 +1668,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DG10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1740,15 +1743,15 @@
       <c r="DE11" s="42" t="n">
         <v>2446.35</v>
       </c>
-      <c r="DF11" t="n">
+      <c r="DF11" s="42" t="n">
         <v>2453.35</v>
       </c>
-      <c r="DG11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1815,8 +1818,11 @@
       <c r="DE12" s="42" t="n">
         <v>1876.35</v>
       </c>
-      <c r="DF12" t="n">
+      <c r="DF12" s="42" t="n">
         <v>1866.35</v>
+      </c>
+      <c r="DG12" t="n">
+        <v>1861.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1864,7 +1870,7 @@
       <c r="CM13" s="42" t="n">
         <v>2459.06</v>
       </c>
-      <c r="DF13" t="n">
+      <c r="DF13" s="42" t="n">
         <v>2348.35</v>
       </c>
     </row>
@@ -2018,7 +2024,7 @@
       <c r="DE16" s="42" t="n">
         <v>2063.35</v>
       </c>
-      <c r="DF16" t="n">
+      <c r="DF16" s="42" t="n">
         <v>2069.35</v>
       </c>
     </row>
@@ -2143,7 +2149,7 @@
           <t>Oct 02</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -2225,8 +2231,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DG21" s="42" t="n"/>
       <c r="DH21" s="42" t="n"/>
+      <c r="DI21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2282,12 +2288,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DG22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH22" s="58" t="inlineStr">
+      <c r="DH22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2341,12 +2347,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DG23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DH23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2433,12 +2439,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DG24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH24" s="58" t="inlineStr">
+      <c r="DH24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2517,12 +2523,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DG25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH25" s="58" t="inlineStr">
+      <c r="DH25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2585,12 +2591,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DG26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH26" s="58" t="inlineStr">
+      <c r="DH26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2657,12 +2663,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DG27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH27" s="71" t="inlineStr">
+      <c r="DH27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2726,12 +2732,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DG28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH28" s="58" t="inlineStr">
+      <c r="DH28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2791,12 +2797,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DG29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH29" s="71" t="inlineStr">
+      <c r="DH29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2858,12 +2864,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DG30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH30" s="71" t="inlineStr">
+      <c r="DH30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2918,12 +2924,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DG31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DH31" s="58" t="inlineStr">
+      <c r="DH31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DI31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-10
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DI49"/>
+  <dimension ref="A1:DJ49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1062,14 +1062,17 @@
         <v>46303.80160574074</v>
       </c>
       <c r="DG1" s="56" t="n">
-        <v>46304.78105941539</v>
-      </c>
-      <c r="DH1" s="44" t="inlineStr">
+        <v>46304.78105940972</v>
+      </c>
+      <c r="DH1" s="56" t="n">
+        <v>46305.73969836593</v>
+      </c>
+      <c r="DI1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DI1" s="44" t="inlineStr">
+      <c r="DJ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1123,12 +1126,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DH2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI2" s="58" t="inlineStr">
+      <c r="DI2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1182,12 +1185,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DH3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI3" s="58" t="inlineStr">
+      <c r="DI3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1242,12 +1245,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DH4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1351,12 +1354,15 @@
       <c r="DE5" s="42" t="n">
         <v>2149.35</v>
       </c>
-      <c r="DH5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DH5" t="n">
+        <v>2132.35</v>
       </c>
       <c r="DI5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1416,12 +1422,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DH6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1476,12 +1482,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DH7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1562,12 +1568,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DH8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1615,12 +1621,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DH9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1668,12 +1674,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DH10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1746,12 +1752,15 @@
       <c r="DF11" s="42" t="n">
         <v>2453.35</v>
       </c>
-      <c r="DH11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DH11" t="n">
+        <v>2432.35</v>
       </c>
       <c r="DI11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1821,8 +1830,11 @@
       <c r="DF12" s="42" t="n">
         <v>1866.35</v>
       </c>
-      <c r="DG12" t="n">
+      <c r="DG12" s="42" t="n">
         <v>1861.35</v>
+      </c>
+      <c r="DH12" t="n">
+        <v>1856.35</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
@@ -1873,6 +1885,9 @@
       <c r="DF13" s="42" t="n">
         <v>2348.35</v>
       </c>
+      <c r="DH13" t="n">
+        <v>2327.35</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -2006,6 +2021,11 @@
           <t>Oct 13</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="CR16" s="42" t="n">
         <v>2158.35</v>
       </c>
@@ -2079,6 +2099,9 @@
       <c r="DE17" s="42" t="n">
         <v>1892.35</v>
       </c>
+      <c r="DH17" t="n">
+        <v>1874.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -2117,6 +2140,9 @@
       <c r="CZ18" s="42" t="n">
         <v>3236.35</v>
       </c>
+      <c r="DH18" t="n">
+        <v>3204.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
@@ -2212,6 +2238,9 @@
       </c>
       <c r="DE20" s="42" t="n">
         <v>2577.35</v>
+      </c>
+      <c r="DH20" t="n">
+        <v>2556.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2231,8 +2260,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DH21" s="42" t="n"/>
       <c r="DI21" s="42" t="n"/>
+      <c r="DJ21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2288,12 +2317,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DH22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI22" s="58" t="inlineStr">
+      <c r="DI22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2347,12 +2376,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DH23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DI23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2439,12 +2468,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DH24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI24" s="58" t="inlineStr">
+      <c r="DI24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2523,12 +2552,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DH25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI25" s="58" t="inlineStr">
+      <c r="DI25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2591,12 +2620,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DH26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI26" s="58" t="inlineStr">
+      <c r="DI26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2663,12 +2692,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DH27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI27" s="71" t="inlineStr">
+      <c r="DI27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2732,12 +2761,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DH28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI28" s="58" t="inlineStr">
+      <c r="DI28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2797,12 +2826,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DH29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI29" s="71" t="inlineStr">
+      <c r="DI29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2864,12 +2893,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DH30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI30" s="71" t="inlineStr">
+      <c r="DI30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2924,12 +2953,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DH31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DI31" s="58" t="inlineStr">
+      <c r="DI31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DJ31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-11
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DJ49"/>
+  <dimension ref="A1:DK49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1065,14 +1065,17 @@
         <v>46304.78105940972</v>
       </c>
       <c r="DH1" s="56" t="n">
-        <v>46305.73969836593</v>
-      </c>
-      <c r="DI1" s="44" t="inlineStr">
+        <v>46305.73969836806</v>
+      </c>
+      <c r="DI1" s="56" t="n">
+        <v>46306.7495936861</v>
+      </c>
+      <c r="DJ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DJ1" s="44" t="inlineStr">
+      <c r="DK1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1126,12 +1129,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DI2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ2" s="58" t="inlineStr">
+      <c r="DJ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1185,12 +1188,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DI3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ3" s="58" t="inlineStr">
+      <c r="DJ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1245,12 +1248,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DI4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1354,15 +1357,15 @@
       <c r="DE5" s="42" t="n">
         <v>2149.35</v>
       </c>
-      <c r="DH5" t="n">
+      <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DI5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1422,12 +1425,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DI6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1482,12 +1485,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DI7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1568,12 +1571,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DI8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1621,12 +1624,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DI9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1674,12 +1677,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DI10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1752,15 +1755,18 @@
       <c r="DF11" s="42" t="n">
         <v>2453.35</v>
       </c>
-      <c r="DH11" t="n">
+      <c r="DH11" s="42" t="n">
         <v>2432.35</v>
       </c>
-      <c r="DI11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DI11" t="n">
+        <v>2425.35</v>
       </c>
       <c r="DJ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1833,7 +1839,7 @@
       <c r="DG12" s="42" t="n">
         <v>1861.35</v>
       </c>
-      <c r="DH12" t="n">
+      <c r="DH12" s="42" t="n">
         <v>1856.35</v>
       </c>
     </row>
@@ -1885,7 +1891,7 @@
       <c r="DF13" s="42" t="n">
         <v>2348.35</v>
       </c>
-      <c r="DH13" t="n">
+      <c r="DH13" s="42" t="n">
         <v>2327.35</v>
       </c>
     </row>
@@ -2021,7 +2027,7 @@
           <t>Oct 13</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -2099,7 +2105,7 @@
       <c r="DE17" s="42" t="n">
         <v>1892.35</v>
       </c>
-      <c r="DH17" t="n">
+      <c r="DH17" s="42" t="n">
         <v>1874.35</v>
       </c>
     </row>
@@ -2140,7 +2146,7 @@
       <c r="CZ18" s="42" t="n">
         <v>3236.35</v>
       </c>
-      <c r="DH18" t="n">
+      <c r="DH18" s="42" t="n">
         <v>3204.35</v>
       </c>
     </row>
@@ -2239,7 +2245,7 @@
       <c r="DE20" s="42" t="n">
         <v>2577.35</v>
       </c>
-      <c r="DH20" t="n">
+      <c r="DH20" s="42" t="n">
         <v>2556.35</v>
       </c>
     </row>
@@ -2260,8 +2266,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DI21" s="42" t="n"/>
       <c r="DJ21" s="42" t="n"/>
+      <c r="DK21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2317,12 +2323,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DI22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ22" s="58" t="inlineStr">
+      <c r="DJ22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2376,12 +2382,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DI23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DJ23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2468,12 +2474,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DI24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ24" s="58" t="inlineStr">
+      <c r="DJ24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2552,12 +2558,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DI25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ25" s="58" t="inlineStr">
+      <c r="DJ25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2620,12 +2626,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DI26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ26" s="58" t="inlineStr">
+      <c r="DJ26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2692,12 +2698,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DI27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ27" s="71" t="inlineStr">
+      <c r="DJ27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2761,12 +2767,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DI28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ28" s="58" t="inlineStr">
+      <c r="DJ28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2826,12 +2832,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DI29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ29" s="71" t="inlineStr">
+      <c r="DJ29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2893,12 +2899,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DI30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ30" s="71" t="inlineStr">
+      <c r="DJ30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2953,12 +2959,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DI31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DJ31" s="58" t="inlineStr">
+      <c r="DJ31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DK31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-13
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DK49"/>
+  <dimension ref="A1:DL49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1068,14 +1068,17 @@
         <v>46305.73969836806</v>
       </c>
       <c r="DI1" s="56" t="n">
-        <v>46306.7495936861</v>
-      </c>
-      <c r="DJ1" s="44" t="inlineStr">
+        <v>46306.74959368056</v>
+      </c>
+      <c r="DJ1" s="56" t="n">
+        <v>46308.82637601649</v>
+      </c>
+      <c r="DK1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DK1" s="44" t="inlineStr">
+      <c r="DL1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1129,12 +1132,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DJ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK2" s="58" t="inlineStr">
+      <c r="DK2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1188,12 +1191,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DJ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK3" s="58" t="inlineStr">
+      <c r="DK3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1248,12 +1251,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DJ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1360,12 +1363,12 @@
       <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DJ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1425,12 +1428,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DJ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1485,12 +1488,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DJ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1571,12 +1574,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DJ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1624,12 +1627,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DJ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1677,12 +1680,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DJ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1722,6 +1725,11 @@
           <t>Oct 12</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="BI11" s="42" t="n">
         <v>2603.06</v>
       </c>
@@ -1758,15 +1766,15 @@
       <c r="DH11" s="42" t="n">
         <v>2432.35</v>
       </c>
-      <c r="DI11" t="n">
+      <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DJ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2148,6 +2156,9 @@
       </c>
       <c r="DH18" s="42" t="n">
         <v>3204.35</v>
+      </c>
+      <c r="DJ18" t="n">
+        <v>3110.35</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
@@ -2266,8 +2277,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DJ21" s="42" t="n"/>
       <c r="DK21" s="42" t="n"/>
+      <c r="DL21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2323,12 +2334,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DJ22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK22" s="58" t="inlineStr">
+      <c r="DK22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2382,12 +2393,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DJ23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DK23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2474,12 +2485,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DJ24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK24" s="58" t="inlineStr">
+      <c r="DK24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2558,12 +2569,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DJ25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK25" s="58" t="inlineStr">
+      <c r="DK25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2626,12 +2637,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DJ26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK26" s="58" t="inlineStr">
+      <c r="DK26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2698,12 +2709,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DJ27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK27" s="71" t="inlineStr">
+      <c r="DK27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2767,12 +2778,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DJ28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK28" s="58" t="inlineStr">
+      <c r="DK28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2832,12 +2843,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DJ29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK29" s="71" t="inlineStr">
+      <c r="DK29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2899,12 +2910,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DJ30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK30" s="71" t="inlineStr">
+      <c r="DK30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2959,12 +2970,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DJ31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DK31" s="58" t="inlineStr">
+      <c r="DK31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DL31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-14
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DL49"/>
+  <dimension ref="A1:DM49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1071,14 +1071,17 @@
         <v>46306.74959368056</v>
       </c>
       <c r="DJ1" s="56" t="n">
-        <v>46308.82637601649</v>
-      </c>
-      <c r="DK1" s="44" t="inlineStr">
+        <v>46308.82637601852</v>
+      </c>
+      <c r="DK1" s="56" t="n">
+        <v>46309.74708657582</v>
+      </c>
+      <c r="DL1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DL1" s="44" t="inlineStr">
+      <c r="DM1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1132,12 +1135,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DK2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL2" s="58" t="inlineStr">
+      <c r="DL2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1191,12 +1194,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DK3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL3" s="58" t="inlineStr">
+      <c r="DL3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1251,12 +1254,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DK4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1363,12 +1366,12 @@
       <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DK5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1428,12 +1431,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DK6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1488,12 +1491,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DK7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1574,12 +1577,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DK8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1627,12 +1630,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DK9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1680,12 +1683,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DK10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1725,7 +1728,7 @@
           <t>Oct 12</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -1769,12 +1772,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DK11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1902,6 +1905,9 @@
       <c r="DH13" s="42" t="n">
         <v>2327.35</v>
       </c>
+      <c r="DK13" t="n">
+        <v>2288.35</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -2116,6 +2122,9 @@
       <c r="DH17" s="42" t="n">
         <v>1874.35</v>
       </c>
+      <c r="DK17" t="n">
+        <v>1869.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -2157,7 +2166,7 @@
       <c r="DH18" s="42" t="n">
         <v>3204.35</v>
       </c>
-      <c r="DJ18" t="n">
+      <c r="DJ18" s="42" t="n">
         <v>3110.35</v>
       </c>
     </row>
@@ -2258,6 +2267,9 @@
       </c>
       <c r="DH20" s="42" t="n">
         <v>2556.35</v>
+      </c>
+      <c r="DK20" t="n">
+        <v>2517.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2277,8 +2289,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DK21" s="42" t="n"/>
       <c r="DL21" s="42" t="n"/>
+      <c r="DM21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2334,12 +2346,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DK22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL22" s="58" t="inlineStr">
+      <c r="DL22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2393,12 +2405,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DK23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DL23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2485,12 +2497,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DK24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL24" s="58" t="inlineStr">
+      <c r="DL24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2569,12 +2581,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DK25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL25" s="58" t="inlineStr">
+      <c r="DL25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2637,12 +2649,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DK26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL26" s="58" t="inlineStr">
+      <c r="DL26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2709,12 +2721,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DK27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL27" s="71" t="inlineStr">
+      <c r="DL27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2778,12 +2790,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DK28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL28" s="58" t="inlineStr">
+      <c r="DL28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2843,12 +2855,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DK29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL29" s="71" t="inlineStr">
+      <c r="DL29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2910,12 +2922,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DK30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL30" s="71" t="inlineStr">
+      <c r="DL30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2970,12 +2982,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DK31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DL31" s="58" t="inlineStr">
+      <c r="DL31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DM31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-16
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DM49"/>
+  <dimension ref="A1:DN49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1074,14 +1074,17 @@
         <v>46308.82637601852</v>
       </c>
       <c r="DK1" s="56" t="n">
-        <v>46309.74708657582</v>
-      </c>
-      <c r="DL1" s="44" t="inlineStr">
+        <v>46309.74708657408</v>
+      </c>
+      <c r="DL1" s="56" t="n">
+        <v>46311.72108512666</v>
+      </c>
+      <c r="DM1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DM1" s="44" t="inlineStr">
+      <c r="DN1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1135,12 +1138,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DL2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM2" s="58" t="inlineStr">
+      <c r="DM2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1194,12 +1197,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DL3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM3" s="58" t="inlineStr">
+      <c r="DM3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1254,12 +1257,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DL4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1366,12 +1369,12 @@
       <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DL5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1431,12 +1434,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DL6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1491,12 +1494,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DL7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1577,12 +1580,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DL8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1630,12 +1633,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DL9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1683,12 +1686,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DL10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1772,12 +1775,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DL11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1905,7 +1908,7 @@
       <c r="DH13" s="42" t="n">
         <v>2327.35</v>
       </c>
-      <c r="DK13" t="n">
+      <c r="DK13" s="42" t="n">
         <v>2288.35</v>
       </c>
     </row>
@@ -2122,8 +2125,11 @@
       <c r="DH17" s="42" t="n">
         <v>1874.35</v>
       </c>
-      <c r="DK17" t="n">
+      <c r="DK17" s="42" t="n">
         <v>1869.35</v>
+      </c>
+      <c r="DL17" t="n">
+        <v>1864.35</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
@@ -2221,6 +2227,9 @@
       <c r="DE19" s="42" t="n">
         <v>2543.35</v>
       </c>
+      <c r="DL19" t="n">
+        <v>2483.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
@@ -2268,7 +2277,7 @@
       <c r="DH20" s="42" t="n">
         <v>2556.35</v>
       </c>
-      <c r="DK20" t="n">
+      <c r="DK20" s="42" t="n">
         <v>2517.35</v>
       </c>
     </row>
@@ -2289,8 +2298,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DL21" s="42" t="n"/>
       <c r="DM21" s="42" t="n"/>
+      <c r="DN21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2346,12 +2355,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DL22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM22" s="58" t="inlineStr">
+      <c r="DM22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2405,12 +2414,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DL23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DM23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2497,12 +2506,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DL24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM24" s="58" t="inlineStr">
+      <c r="DM24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2581,12 +2590,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DL25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM25" s="58" t="inlineStr">
+      <c r="DM25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2649,12 +2658,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DL26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM26" s="58" t="inlineStr">
+      <c r="DM26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2721,12 +2730,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DL27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM27" s="71" t="inlineStr">
+      <c r="DM27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2790,12 +2799,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DL28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM28" s="58" t="inlineStr">
+      <c r="DM28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2855,12 +2864,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DL29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM29" s="71" t="inlineStr">
+      <c r="DM29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2922,12 +2931,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DL30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM30" s="71" t="inlineStr">
+      <c r="DM30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2982,12 +2991,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DL31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DM31" s="58" t="inlineStr">
+      <c r="DM31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DN31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-17
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DN49"/>
+  <dimension ref="A1:DO49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1077,14 +1077,17 @@
         <v>46309.74708657408</v>
       </c>
       <c r="DL1" s="56" t="n">
-        <v>46311.72108512666</v>
-      </c>
-      <c r="DM1" s="44" t="inlineStr">
+        <v>46311.72108512731</v>
+      </c>
+      <c r="DM1" s="56" t="n">
+        <v>46312.67900343905</v>
+      </c>
+      <c r="DN1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DN1" s="44" t="inlineStr">
+      <c r="DO1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1138,12 +1141,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DM2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN2" s="58" t="inlineStr">
+      <c r="DN2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1197,12 +1200,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DM3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN3" s="58" t="inlineStr">
+      <c r="DN3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1257,12 +1260,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DM4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1369,12 +1372,15 @@
       <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DM5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DM5" t="n">
+        <v>2108.35</v>
       </c>
       <c r="DN5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1434,12 +1440,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DM6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1494,12 +1500,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DM7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1580,12 +1586,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DM8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1633,12 +1639,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DM9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1686,12 +1692,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DM10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1775,12 +1781,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DM11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1911,6 +1917,9 @@
       <c r="DK13" s="42" t="n">
         <v>2288.35</v>
       </c>
+      <c r="DM13" t="n">
+        <v>2258.35</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="43">
       <c r="A14" s="42" t="inlineStr">
@@ -2128,8 +2137,11 @@
       <c r="DK17" s="42" t="n">
         <v>1869.35</v>
       </c>
-      <c r="DL17" t="n">
+      <c r="DL17" s="42" t="n">
         <v>1864.35</v>
+      </c>
+      <c r="DM17" t="n">
+        <v>1856.35</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
@@ -2175,6 +2187,9 @@
       <c r="DJ18" s="42" t="n">
         <v>3110.35</v>
       </c>
+      <c r="DM18" t="n">
+        <v>3058.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
@@ -2227,8 +2242,11 @@
       <c r="DE19" s="42" t="n">
         <v>2543.35</v>
       </c>
-      <c r="DL19" t="n">
+      <c r="DL19" s="42" t="n">
         <v>2483.35</v>
+      </c>
+      <c r="DM19" t="n">
+        <v>2453.35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
@@ -2279,6 +2297,9 @@
       </c>
       <c r="DK20" s="42" t="n">
         <v>2517.35</v>
+      </c>
+      <c r="DM20" t="n">
+        <v>2487.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2298,8 +2319,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DM21" s="42" t="n"/>
       <c r="DN21" s="42" t="n"/>
+      <c r="DO21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2355,12 +2376,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DM22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN22" s="58" t="inlineStr">
+      <c r="DN22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2414,12 +2435,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DM23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DN23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2506,12 +2527,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DM24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN24" s="58" t="inlineStr">
+      <c r="DN24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2590,12 +2611,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DM25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN25" s="58" t="inlineStr">
+      <c r="DN25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2658,12 +2679,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DM26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN26" s="58" t="inlineStr">
+      <c r="DN26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2730,12 +2751,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DM27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN27" s="71" t="inlineStr">
+      <c r="DN27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2799,12 +2820,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DM28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN28" s="58" t="inlineStr">
+      <c r="DN28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2864,12 +2885,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DM29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN29" s="71" t="inlineStr">
+      <c r="DN29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2931,12 +2952,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DM30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN30" s="71" t="inlineStr">
+      <c r="DN30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2991,12 +3012,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DM31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DN31" s="58" t="inlineStr">
+      <c r="DN31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DO31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-18
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DO49"/>
+  <dimension ref="A1:DP49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1080,14 +1080,17 @@
         <v>46311.72108512731</v>
       </c>
       <c r="DM1" s="56" t="n">
-        <v>46312.67900343905</v>
-      </c>
-      <c r="DN1" s="44" t="inlineStr">
+        <v>46312.6790034375</v>
+      </c>
+      <c r="DN1" s="56" t="n">
+        <v>46313.68536211279</v>
+      </c>
+      <c r="DO1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DO1" s="44" t="inlineStr">
+      <c r="DP1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1141,12 +1144,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DN2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO2" s="58" t="inlineStr">
+      <c r="DO2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1200,12 +1203,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DN3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO3" s="58" t="inlineStr">
+      <c r="DO3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1260,12 +1263,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DN4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1372,15 +1375,15 @@
       <c r="DH5" s="42" t="n">
         <v>2132.35</v>
       </c>
-      <c r="DM5" t="n">
+      <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DN5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1440,12 +1443,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DN6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1500,12 +1503,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DN7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1586,12 +1589,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DN8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1639,12 +1642,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DN9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1692,12 +1695,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DN10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1781,12 +1784,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DN11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1917,7 +1920,7 @@
       <c r="DK13" s="42" t="n">
         <v>2288.35</v>
       </c>
-      <c r="DM13" t="n">
+      <c r="DM13" s="42" t="n">
         <v>2258.35</v>
       </c>
     </row>
@@ -2140,7 +2143,7 @@
       <c r="DL17" s="42" t="n">
         <v>1864.35</v>
       </c>
-      <c r="DM17" t="n">
+      <c r="DM17" s="42" t="n">
         <v>1856.35</v>
       </c>
     </row>
@@ -2187,7 +2190,7 @@
       <c r="DJ18" s="42" t="n">
         <v>3110.35</v>
       </c>
-      <c r="DM18" t="n">
+      <c r="DM18" s="42" t="n">
         <v>3058.35</v>
       </c>
     </row>
@@ -2245,7 +2248,7 @@
       <c r="DL19" s="42" t="n">
         <v>2483.35</v>
       </c>
-      <c r="DM19" t="n">
+      <c r="DM19" s="42" t="n">
         <v>2453.35</v>
       </c>
     </row>
@@ -2298,8 +2301,11 @@
       <c r="DK20" s="42" t="n">
         <v>2517.35</v>
       </c>
-      <c r="DM20" t="n">
+      <c r="DM20" s="42" t="n">
         <v>2487.35</v>
+      </c>
+      <c r="DN20" t="n">
+        <v>2494.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2319,8 +2325,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DN21" s="42" t="n"/>
       <c r="DO21" s="42" t="n"/>
+      <c r="DP21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2376,12 +2382,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DN22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO22" s="58" t="inlineStr">
+      <c r="DO22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2435,12 +2441,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DN23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DO23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2527,12 +2533,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DN24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO24" s="58" t="inlineStr">
+      <c r="DO24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2611,12 +2617,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DN25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO25" s="58" t="inlineStr">
+      <c r="DO25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2679,12 +2685,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DN26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO26" s="58" t="inlineStr">
+      <c r="DO26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2751,12 +2757,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DN27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO27" s="71" t="inlineStr">
+      <c r="DO27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2820,12 +2826,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DN28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO28" s="58" t="inlineStr">
+      <c r="DO28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2885,12 +2891,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DN29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO29" s="71" t="inlineStr">
+      <c r="DO29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2952,12 +2958,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DN30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO30" s="71" t="inlineStr">
+      <c r="DO30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3012,12 +3018,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DN31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DO31" s="58" t="inlineStr">
+      <c r="DO31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DP31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-19
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DP49"/>
+  <dimension ref="A1:DQ49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1083,14 +1083,17 @@
         <v>46312.6790034375</v>
       </c>
       <c r="DN1" s="56" t="n">
-        <v>46313.68536211279</v>
-      </c>
-      <c r="DO1" s="44" t="inlineStr">
+        <v>46313.68536211806</v>
+      </c>
+      <c r="DO1" s="56" t="n">
+        <v>46314.80054927085</v>
+      </c>
+      <c r="DP1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DP1" s="44" t="inlineStr">
+      <c r="DQ1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1144,12 +1147,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DO2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP2" s="58" t="inlineStr">
+      <c r="DP2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1203,12 +1206,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DO3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP3" s="58" t="inlineStr">
+      <c r="DP3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1263,12 +1266,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DO4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1308,7 +1311,11 @@
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="H5" s="42" t="n"/>
+      <c r="H5" s="42" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="AH5" s="42" t="n">
         <v>2648.06</v>
       </c>
@@ -1378,12 +1385,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DO5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1443,12 +1450,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DO6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1503,12 +1510,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DO7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1589,12 +1596,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DO8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1642,12 +1649,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DO9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1695,12 +1702,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DO10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1784,12 +1791,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DO11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2304,8 +2311,11 @@
       <c r="DM20" s="42" t="n">
         <v>2487.35</v>
       </c>
-      <c r="DN20" t="n">
+      <c r="DN20" s="42" t="n">
         <v>2494.35</v>
+      </c>
+      <c r="DO20" t="n">
+        <v>2487.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2325,8 +2335,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DO21" s="42" t="n"/>
       <c r="DP21" s="42" t="n"/>
+      <c r="DQ21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2382,12 +2392,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DO22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP22" s="58" t="inlineStr">
+      <c r="DP22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2441,12 +2451,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DO23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DP23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2533,12 +2543,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DO24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP24" s="58" t="inlineStr">
+      <c r="DP24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2617,12 +2627,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DO25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP25" s="58" t="inlineStr">
+      <c r="DP25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2685,12 +2695,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DO26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP26" s="58" t="inlineStr">
+      <c r="DP26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2757,12 +2767,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DO27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP27" s="71" t="inlineStr">
+      <c r="DP27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2826,12 +2836,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DO28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP28" s="58" t="inlineStr">
+      <c r="DP28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2891,12 +2901,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DO29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP29" s="71" t="inlineStr">
+      <c r="DP29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2958,12 +2968,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DO30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP30" s="71" t="inlineStr">
+      <c r="DP30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3018,12 +3028,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DO31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DP31" s="58" t="inlineStr">
+      <c r="DP31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DQ31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-20
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DQ49"/>
+  <dimension ref="A1:DR49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1086,14 +1086,17 @@
         <v>46313.68536211806</v>
       </c>
       <c r="DO1" s="56" t="n">
-        <v>46314.80054927085</v>
-      </c>
-      <c r="DP1" s="44" t="inlineStr">
+        <v>46314.80054927083</v>
+      </c>
+      <c r="DP1" s="56" t="n">
+        <v>46315.74546484306</v>
+      </c>
+      <c r="DQ1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DQ1" s="44" t="inlineStr">
+      <c r="DR1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1147,12 +1150,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DP2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ2" s="58" t="inlineStr">
+      <c r="DQ2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1206,12 +1209,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DP3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ3" s="58" t="inlineStr">
+      <c r="DQ3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1266,12 +1269,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DP4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1385,12 +1388,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DP5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1450,12 +1453,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DP6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1510,12 +1513,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DP7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1596,12 +1599,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DP8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1649,12 +1652,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DP9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1702,12 +1705,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DP10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1791,12 +1794,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DP11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2290,6 +2293,11 @@
           <t>Oct 22</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Off Market</t>
+        </is>
+      </c>
       <c r="CZ20" s="42" t="n">
         <v>2644.35</v>
       </c>
@@ -2314,7 +2322,7 @@
       <c r="DN20" s="42" t="n">
         <v>2494.35</v>
       </c>
-      <c r="DO20" t="n">
+      <c r="DO20" s="42" t="n">
         <v>2487.35</v>
       </c>
     </row>
@@ -2335,8 +2343,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DP21" s="42" t="n"/>
       <c r="DQ21" s="42" t="n"/>
+      <c r="DR21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2392,12 +2400,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DP22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ22" s="58" t="inlineStr">
+      <c r="DQ22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2451,12 +2459,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DP23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DQ23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2543,12 +2551,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DP24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ24" s="58" t="inlineStr">
+      <c r="DQ24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2627,12 +2635,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DP25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ25" s="58" t="inlineStr">
+      <c r="DQ25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2695,12 +2703,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DP26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ26" s="58" t="inlineStr">
+      <c r="DQ26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2767,12 +2775,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DP27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ27" s="71" t="inlineStr">
+      <c r="DQ27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2836,12 +2844,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DP28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ28" s="58" t="inlineStr">
+      <c r="DQ28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2901,12 +2909,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DP29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ29" s="71" t="inlineStr">
+      <c r="DQ29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2968,12 +2976,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DP30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ30" s="71" t="inlineStr">
+      <c r="DQ30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3028,12 +3036,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DP31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DQ31" s="58" t="inlineStr">
+      <c r="DQ31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DR31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-21
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DR49"/>
+  <dimension ref="A1:DS49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1089,14 +1089,17 @@
         <v>46314.80054927083</v>
       </c>
       <c r="DP1" s="56" t="n">
-        <v>46315.74546484306</v>
-      </c>
-      <c r="DQ1" s="44" t="inlineStr">
+        <v>46315.74546483796</v>
+      </c>
+      <c r="DQ1" s="56" t="n">
+        <v>46316.74907998247</v>
+      </c>
+      <c r="DR1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DR1" s="44" t="inlineStr">
+      <c r="DS1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1150,12 +1153,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DQ2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR2" s="58" t="inlineStr">
+      <c r="DR2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1209,12 +1212,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DQ3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR3" s="58" t="inlineStr">
+      <c r="DR3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1269,12 +1272,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DQ4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1388,12 +1391,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DQ5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1453,12 +1456,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DQ6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1513,12 +1516,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DQ7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1599,12 +1602,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DQ8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1652,12 +1655,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DQ9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1705,12 +1708,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DQ10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1794,12 +1797,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DQ11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2293,7 +2296,7 @@
           <t>Oct 22</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>Off Market</t>
         </is>
@@ -2343,8 +2346,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DQ21" s="42" t="n"/>
       <c r="DR21" s="42" t="n"/>
+      <c r="DS21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2400,12 +2403,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DQ22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR22" s="58" t="inlineStr">
+      <c r="DR22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2459,12 +2462,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DQ23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DR23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2551,12 +2554,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DQ24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR24" s="58" t="inlineStr">
+      <c r="DR24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2635,12 +2638,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DQ25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR25" s="58" t="inlineStr">
+      <c r="DR25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2703,12 +2706,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DQ26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR26" s="58" t="inlineStr">
+      <c r="DR26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2775,12 +2778,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DQ27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR27" s="71" t="inlineStr">
+      <c r="DR27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2844,12 +2847,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DQ28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR28" s="58" t="inlineStr">
+      <c r="DR28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2909,12 +2912,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DQ29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR29" s="71" t="inlineStr">
+      <c r="DR29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2976,12 +2979,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DQ30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR30" s="71" t="inlineStr">
+      <c r="DR30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3036,12 +3039,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DQ31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DR31" s="58" t="inlineStr">
+      <c r="DR31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DS31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-22
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DS49"/>
+  <dimension ref="A1:DT49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1092,14 +1092,17 @@
         <v>46315.74546483796</v>
       </c>
       <c r="DQ1" s="56" t="n">
-        <v>46316.74907998247</v>
-      </c>
-      <c r="DR1" s="44" t="inlineStr">
+        <v>46316.74907997685</v>
+      </c>
+      <c r="DR1" s="56" t="n">
+        <v>46317.75544007214</v>
+      </c>
+      <c r="DS1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DS1" s="44" t="inlineStr">
+      <c r="DT1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1153,12 +1156,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DR2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS2" s="58" t="inlineStr">
+      <c r="DS2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1212,12 +1215,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DR3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS3" s="58" t="inlineStr">
+      <c r="DS3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1272,12 +1275,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DR4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1391,12 +1394,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DR5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1456,12 +1459,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DR6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1516,12 +1519,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DR7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1602,12 +1605,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DR8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1655,12 +1658,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DR9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1708,12 +1711,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DR10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1797,12 +1800,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DR11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2206,6 +2209,9 @@
       <c r="DM18" s="42" t="n">
         <v>3058.35</v>
       </c>
+      <c r="DR18" t="n">
+        <v>2968.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
@@ -2264,6 +2270,9 @@
       <c r="DM19" s="42" t="n">
         <v>2453.35</v>
       </c>
+      <c r="DR19" t="n">
+        <v>2384.35</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
       <c r="A20" s="42" t="inlineStr">
@@ -2327,6 +2336,9 @@
       </c>
       <c r="DO20" s="42" t="n">
         <v>2487.35</v>
+      </c>
+      <c r="DR20" t="n">
+        <v>2424.35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="43">
@@ -2346,8 +2358,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DR21" s="42" t="n"/>
       <c r="DS21" s="42" t="n"/>
+      <c r="DT21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2403,12 +2415,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DR22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS22" s="58" t="inlineStr">
+      <c r="DS22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2462,12 +2474,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DR23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DS23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2554,12 +2566,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DR24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS24" s="58" t="inlineStr">
+      <c r="DS24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2638,12 +2650,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DR25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS25" s="58" t="inlineStr">
+      <c r="DS25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2706,12 +2718,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DR26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS26" s="58" t="inlineStr">
+      <c r="DS26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2778,12 +2790,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DR27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS27" s="71" t="inlineStr">
+      <c r="DS27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2847,12 +2859,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DR28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS28" s="58" t="inlineStr">
+      <c r="DS28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2912,12 +2924,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DR29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS29" s="71" t="inlineStr">
+      <c r="DS29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2979,12 +2991,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DR30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS30" s="71" t="inlineStr">
+      <c r="DS30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3039,12 +3051,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DR31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DS31" s="58" t="inlineStr">
+      <c r="DS31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DT31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-23
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DT49"/>
+  <dimension ref="A1:DU49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1095,14 +1095,17 @@
         <v>46316.74907997685</v>
       </c>
       <c r="DR1" s="56" t="n">
-        <v>46317.75544007214</v>
-      </c>
-      <c r="DS1" s="44" t="inlineStr">
+        <v>46317.75544006944</v>
+      </c>
+      <c r="DS1" s="56" t="n">
+        <v>46318.74313290935</v>
+      </c>
+      <c r="DT1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DT1" s="44" t="inlineStr">
+      <c r="DU1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1156,12 +1159,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DS2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT2" s="58" t="inlineStr">
+      <c r="DT2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1215,12 +1218,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DS3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT3" s="58" t="inlineStr">
+      <c r="DT3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1275,12 +1278,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DS4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1394,12 +1397,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DS5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1459,12 +1462,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DS6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1519,12 +1522,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DS7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1605,12 +1608,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DS8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1658,12 +1661,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DS9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1711,12 +1714,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DS10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1800,12 +1803,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DS11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2209,7 +2212,7 @@
       <c r="DM18" s="42" t="n">
         <v>3058.35</v>
       </c>
-      <c r="DR18" t="n">
+      <c r="DR18" s="42" t="n">
         <v>2968.35</v>
       </c>
     </row>
@@ -2270,7 +2273,7 @@
       <c r="DM19" s="42" t="n">
         <v>2453.35</v>
       </c>
-      <c r="DR19" t="n">
+      <c r="DR19" s="42" t="n">
         <v>2384.35</v>
       </c>
     </row>
@@ -2337,7 +2340,7 @@
       <c r="DO20" s="42" t="n">
         <v>2487.35</v>
       </c>
-      <c r="DR20" t="n">
+      <c r="DR20" s="42" t="n">
         <v>2424.35</v>
       </c>
     </row>
@@ -2358,8 +2361,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DS21" s="42" t="n"/>
       <c r="DT21" s="42" t="n"/>
+      <c r="DU21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2415,12 +2418,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DS22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT22" s="58" t="inlineStr">
+      <c r="DT22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2474,12 +2477,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DS23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DT23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2566,12 +2569,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DS24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT24" s="58" t="inlineStr">
+      <c r="DT24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2650,12 +2653,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DS25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT25" s="58" t="inlineStr">
+      <c r="DT25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2718,12 +2721,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DS26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT26" s="58" t="inlineStr">
+      <c r="DT26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2790,12 +2793,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DS27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT27" s="71" t="inlineStr">
+      <c r="DT27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2859,12 +2862,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DS28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT28" s="58" t="inlineStr">
+      <c r="DT28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2924,12 +2927,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DS29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT29" s="71" t="inlineStr">
+      <c r="DT29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2991,12 +2994,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DS30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT30" s="71" t="inlineStr">
+      <c r="DT30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3051,12 +3054,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DS31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DT31" s="58" t="inlineStr">
+      <c r="DT31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DU31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-24
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DU49"/>
+  <dimension ref="A1:DV49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1098,14 +1098,17 @@
         <v>46317.75544006944</v>
       </c>
       <c r="DS1" s="56" t="n">
-        <v>46318.74313290935</v>
-      </c>
-      <c r="DT1" s="44" t="inlineStr">
+        <v>46318.7431329051</v>
+      </c>
+      <c r="DT1" s="56" t="n">
+        <v>46319.68865832777</v>
+      </c>
+      <c r="DU1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DU1" s="44" t="inlineStr">
+      <c r="DV1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1159,12 +1162,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DT2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU2" s="58" t="inlineStr">
+      <c r="DU2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1218,12 +1221,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DT3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU3" s="58" t="inlineStr">
+      <c r="DU3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1278,12 +1281,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DT4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1397,12 +1400,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DT5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1462,12 +1465,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DT6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1522,12 +1525,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DT7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1608,12 +1611,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DT8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1661,12 +1664,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DT9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1714,12 +1717,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DT10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1803,12 +1806,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DT11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2275,6 +2278,9 @@
       </c>
       <c r="DR19" s="42" t="n">
         <v>2384.35</v>
+      </c>
+      <c r="DT19" t="n">
+        <v>2318.35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
@@ -2361,8 +2367,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DT21" s="42" t="n"/>
       <c r="DU21" s="42" t="n"/>
+      <c r="DV21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2418,12 +2424,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DT22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU22" s="58" t="inlineStr">
+      <c r="DU22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2477,12 +2483,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DT23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DU23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2569,12 +2575,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DT24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU24" s="58" t="inlineStr">
+      <c r="DU24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2653,12 +2659,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DT25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU25" s="58" t="inlineStr">
+      <c r="DU25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2721,12 +2727,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DT26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU26" s="58" t="inlineStr">
+      <c r="DU26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2793,12 +2799,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DT27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU27" s="71" t="inlineStr">
+      <c r="DU27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2862,12 +2868,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DT28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU28" s="58" t="inlineStr">
+      <c r="DU28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2927,12 +2933,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DT29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU29" s="71" t="inlineStr">
+      <c r="DU29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2994,12 +3000,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DT30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU30" s="71" t="inlineStr">
+      <c r="DU30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3054,12 +3060,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DT31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DU31" s="58" t="inlineStr">
+      <c r="DU31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DV31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-25
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DV49"/>
+  <dimension ref="A1:DW49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1101,14 +1101,17 @@
         <v>46318.7431329051</v>
       </c>
       <c r="DT1" s="56" t="n">
-        <v>46319.68865832777</v>
-      </c>
-      <c r="DU1" s="44" t="inlineStr">
+        <v>46319.68865833333</v>
+      </c>
+      <c r="DU1" s="56" t="n">
+        <v>46320.70944459354</v>
+      </c>
+      <c r="DV1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DV1" s="44" t="inlineStr">
+      <c r="DW1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1162,12 +1165,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DU2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV2" s="58" t="inlineStr">
+      <c r="DV2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1221,12 +1224,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DU3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV3" s="58" t="inlineStr">
+      <c r="DV3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1281,12 +1284,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DU4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1400,12 +1403,12 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DU5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1465,12 +1468,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DU6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1525,12 +1528,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DU7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1611,12 +1614,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DU8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1664,12 +1667,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DU9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1717,12 +1720,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DU10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1806,12 +1809,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DU11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2279,8 +2282,11 @@
       <c r="DR19" s="42" t="n">
         <v>2384.35</v>
       </c>
-      <c r="DT19" t="n">
+      <c r="DT19" s="42" t="n">
         <v>2318.35</v>
+      </c>
+      <c r="DU19" t="n">
+        <v>2312.35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
@@ -2367,8 +2373,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DU21" s="42" t="n"/>
       <c r="DV21" s="42" t="n"/>
+      <c r="DW21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2424,12 +2430,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DU22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV22" s="58" t="inlineStr">
+      <c r="DV22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2483,12 +2489,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DU23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DV23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2575,12 +2581,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DU24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV24" s="58" t="inlineStr">
+      <c r="DV24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2659,12 +2665,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DU25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV25" s="58" t="inlineStr">
+      <c r="DV25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2727,12 +2733,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DU26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV26" s="58" t="inlineStr">
+      <c r="DV26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2799,12 +2805,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DU27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV27" s="71" t="inlineStr">
+      <c r="DV27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2868,12 +2874,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DU28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV28" s="58" t="inlineStr">
+      <c r="DV28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2933,12 +2939,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DU29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV29" s="71" t="inlineStr">
+      <c r="DV29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3000,12 +3006,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DU30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV30" s="71" t="inlineStr">
+      <c r="DV30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3060,12 +3066,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DU31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DV31" s="58" t="inlineStr">
+      <c r="DV31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DW31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-29
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DW49"/>
+  <dimension ref="A1:DX49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1104,14 +1104,17 @@
         <v>46319.68865833333</v>
       </c>
       <c r="DU1" s="56" t="n">
-        <v>46320.70944459354</v>
-      </c>
-      <c r="DV1" s="44" t="inlineStr">
+        <v>46320.7094445949</v>
+      </c>
+      <c r="DV1" s="56" t="n">
+        <v>46324.78878304464</v>
+      </c>
+      <c r="DW1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DW1" s="44" t="inlineStr">
+      <c r="DX1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1165,12 +1168,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DV2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW2" s="58" t="inlineStr">
+      <c r="DW2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1224,12 +1227,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DV3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW3" s="58" t="inlineStr">
+      <c r="DW3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1284,12 +1287,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DV4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1403,12 +1406,15 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DV5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="DV5" t="n">
+        <v>2056.35</v>
       </c>
       <c r="DW5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1468,12 +1474,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DV6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1528,12 +1534,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DV7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1614,12 +1620,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DV8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1667,12 +1673,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DV9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1720,12 +1726,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DV10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1809,12 +1815,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DV11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1890,6 +1896,9 @@
       <c r="DH12" s="42" t="n">
         <v>1856.35</v>
       </c>
+      <c r="DV12" t="n">
+        <v>1806.35</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="43">
       <c r="A13" s="42" t="inlineStr">
@@ -2171,6 +2180,9 @@
       <c r="DM17" s="42" t="n">
         <v>1856.35</v>
       </c>
+      <c r="DV17" t="n">
+        <v>1806.35</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="43">
       <c r="A18" s="42" t="inlineStr">
@@ -2285,8 +2297,11 @@
       <c r="DT19" s="42" t="n">
         <v>2318.35</v>
       </c>
-      <c r="DU19" t="n">
+      <c r="DU19" s="42" t="n">
         <v>2312.35</v>
+      </c>
+      <c r="DV19" t="n">
+        <v>2395.35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
@@ -2373,8 +2388,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DV21" s="42" t="n"/>
       <c r="DW21" s="42" t="n"/>
+      <c r="DX21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2430,12 +2445,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DV22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW22" s="58" t="inlineStr">
+      <c r="DW22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2489,12 +2504,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DV23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DW23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2581,12 +2596,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DV24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW24" s="58" t="inlineStr">
+      <c r="DW24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2665,12 +2680,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DV25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW25" s="58" t="inlineStr">
+      <c r="DW25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2733,12 +2748,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DV26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW26" s="58" t="inlineStr">
+      <c r="DW26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2805,12 +2820,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DV27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW27" s="71" t="inlineStr">
+      <c r="DW27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2874,12 +2889,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DV28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW28" s="58" t="inlineStr">
+      <c r="DW28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2939,12 +2954,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DV29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW29" s="71" t="inlineStr">
+      <c r="DW29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3006,12 +3021,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DV30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW30" s="71" t="inlineStr">
+      <c r="DW30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3066,12 +3081,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DV31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DW31" s="58" t="inlineStr">
+      <c r="DW31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DX31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Daily Thornton Place tracker update - 2026-10-30
</commit_message>
<xml_diff>
--- a/data/Thornton_Tracker.xlsx
+++ b/data/Thornton_Tracker.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:DX49"/>
+  <dimension ref="A1:DY49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="42" min="18" max="19"/>
@@ -1107,14 +1107,17 @@
         <v>46320.7094445949</v>
       </c>
       <c r="DV1" s="56" t="n">
-        <v>46324.78878304464</v>
-      </c>
-      <c r="DW1" s="44" t="inlineStr">
+        <v>46324.78878304398</v>
+      </c>
+      <c r="DW1" s="56" t="n">
+        <v>46325.77215515017</v>
+      </c>
+      <c r="DX1" s="44" t="inlineStr">
         <is>
           <t>$ Change</t>
         </is>
       </c>
-      <c r="DX1" s="44" t="inlineStr">
+      <c r="DY1" s="44" t="inlineStr">
         <is>
           <t>% Change</t>
         </is>
@@ -1168,12 +1171,12 @@
       <c r="AP2" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DW2" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX2" s="58" t="inlineStr">
+      <c r="DX2" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY2" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1227,12 +1230,12 @@
         <v>2224.06</v>
       </c>
       <c r="AQ3" s="42" t="n"/>
-      <c r="DW3" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX3" s="58" t="inlineStr">
+      <c r="DX3" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY3" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1287,12 +1290,12 @@
       <c r="AW4" s="57" t="n">
         <v>2117.06</v>
       </c>
-      <c r="DW4" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX4" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY4" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1406,15 +1409,15 @@
       <c r="DM5" s="42" t="n">
         <v>2108.35</v>
       </c>
-      <c r="DV5" t="n">
+      <c r="DV5" s="42" t="n">
         <v>2056.35</v>
       </c>
-      <c r="DW5" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX5" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY5" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1474,12 +1477,12 @@
       <c r="AX6" s="57" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DW6" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX6" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY6" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1534,12 +1537,12 @@
       <c r="BJ7" s="59" t="n">
         <v>3236.06</v>
       </c>
-      <c r="DW7" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX7" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY7" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1620,12 +1623,12 @@
       <c r="BJ8" s="59" t="n">
         <v>3522.06</v>
       </c>
-      <c r="DW8" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX8" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY8" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1673,12 +1676,12 @@
       <c r="BF9" s="42" t="n">
         <v>2064.06</v>
       </c>
-      <c r="DW9" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX9" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY9" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1726,12 +1729,12 @@
       <c r="BH10" s="42" t="n">
         <v>3628.06</v>
       </c>
-      <c r="DW10" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX10" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY10" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1815,12 +1818,12 @@
       <c r="DI11" s="42" t="n">
         <v>2425.35</v>
       </c>
-      <c r="DW11" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX11" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY11" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1896,7 +1899,7 @@
       <c r="DH12" s="42" t="n">
         <v>1856.35</v>
       </c>
-      <c r="DV12" t="n">
+      <c r="DV12" s="42" t="n">
         <v>1806.35</v>
       </c>
     </row>
@@ -2180,7 +2183,7 @@
       <c r="DM17" s="42" t="n">
         <v>1856.35</v>
       </c>
-      <c r="DV17" t="n">
+      <c r="DV17" s="42" t="n">
         <v>1806.35</v>
       </c>
     </row>
@@ -2233,6 +2236,9 @@
       <c r="DR18" s="42" t="n">
         <v>2968.35</v>
       </c>
+      <c r="DW18" t="n">
+        <v>2881.35</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="43">
       <c r="A19" s="42" t="inlineStr">
@@ -2300,8 +2306,11 @@
       <c r="DU19" s="42" t="n">
         <v>2312.35</v>
       </c>
-      <c r="DV19" t="n">
+      <c r="DV19" s="42" t="n">
         <v>2395.35</v>
+      </c>
+      <c r="DW19" t="n">
+        <v>2388.35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="43">
@@ -2388,8 +2397,8 @@
       <c r="AJ21" s="42" t="n"/>
       <c r="AN21" s="42" t="n"/>
       <c r="AP21" s="42" t="n"/>
-      <c r="DW21" s="42" t="n"/>
       <c r="DX21" s="42" t="n"/>
+      <c r="DY21" s="42" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="43">
       <c r="A22" s="42" t="inlineStr">
@@ -2445,12 +2454,12 @@
       <c r="AJ22" s="42" t="n">
         <v>3610.06</v>
       </c>
-      <c r="DW22" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX22" s="58" t="inlineStr">
+      <c r="DX22" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2504,12 +2513,12 @@
       <c r="AI23" s="42" t="n">
         <v>2430.06</v>
       </c>
-      <c r="DW23" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="DX23" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY23" s="42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2596,12 +2605,12 @@
       <c r="AC24" s="42" t="n">
         <v>3394.06</v>
       </c>
-      <c r="DW24" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX24" s="58" t="inlineStr">
+      <c r="DX24" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY24" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2680,12 +2689,12 @@
       <c r="W25" s="42" t="n">
         <v>3254.06</v>
       </c>
-      <c r="DW25" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX25" s="58" t="inlineStr">
+      <c r="DX25" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2748,12 +2757,12 @@
       <c r="W26" s="42" t="n">
         <v>2304.06</v>
       </c>
-      <c r="DW26" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX26" s="58" t="inlineStr">
+      <c r="DX26" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY26" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2820,12 +2829,12 @@
       <c r="Q27" s="42" t="n">
         <v>3080.85</v>
       </c>
-      <c r="DW27" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX27" s="71" t="inlineStr">
+      <c r="DX27" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY27" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2889,12 +2898,12 @@
       <c r="O28" s="42" t="n">
         <v>2964.85</v>
       </c>
-      <c r="DW28" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX28" s="58" t="inlineStr">
+      <c r="DX28" s="72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY28" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2954,12 +2963,12 @@
         <v>1964.85</v>
       </c>
       <c r="O29" s="69" t="n"/>
-      <c r="DW29" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX29" s="71" t="inlineStr">
+      <c r="DX29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY29" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3021,12 +3030,12 @@
       <c r="M30" s="83" t="n"/>
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="69" t="n"/>
-      <c r="DW30" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX30" s="71" t="inlineStr">
+      <c r="DX30" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY30" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3081,12 +3090,12 @@
       <c r="L31" s="72" t="n">
         <v>1855.85</v>
       </c>
-      <c r="DW31" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="DX31" s="58" t="inlineStr">
+      <c r="DX31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="DY31" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>